<commit_message>
Day 13: Plan A/B weather decision made explicit · sunny=Achensee (boat or free promenade walk) · rain=Swarovski Crystal Worlds · key decisions updated · Excel regenerated
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -5173,7 +5173,7 @@
     <row r="236" ht="22" customHeight="1">
       <c r="A236" s="5" t="inlineStr">
         <is>
-          <t>Key: ✅ Arrive dam by 8:45am — reach Kebema bridge 10:30am · beats 45min photo queue by midday  |  ️ Swarovski: go if raining · skip if clear · 5min off A12 at Wattens · no booking needed  |   Achensee: if kids tired → skip boat · park Pertisau + Gaisalm promenade walk (free, same views)</t>
+          <t>Key: ✅ Arrive dam by 8:45am — reach Kebema bridge 10:30am · beats 45min photo queue by midday  |  ☀️ Plan A (sunny): Achensee — steamboat ~€22/adult OR free Gaisalm promenade walk if kids tired  |  ️ Plan B (rain/cloudy): Swarovski Crystal Worlds — 5min off A12 · ~€22/adult · no booking needed</t>
         </is>
       </c>
     </row>
@@ -5321,51 +5321,51 @@
         </is>
       </c>
     </row>
-    <row r="243" ht="30" customHeight="1">
-      <c r="A243" s="16" t="inlineStr"/>
-      <c r="B243" s="17" t="inlineStr">
+    <row r="243" ht="50" customHeight="1">
+      <c r="A243" s="6" t="inlineStr"/>
+      <c r="B243" s="7" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C243" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D243" s="17" t="inlineStr"/>
-      <c r="E243" s="18" t="inlineStr">
-        <is>
-          <t>⭐ Swarovski Crystal Worlds (Wattens) — ️ Weather-dependent: — ~€22/adult · allow 1.5–2hrs</t>
-        </is>
-      </c>
-      <c r="F243" s="19" t="inlineStr">
-        <is>
-          <t>€22 / 2hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="244" ht="30" customHeight="1">
-      <c r="A244" s="6" t="inlineStr"/>
-      <c r="B244" s="7" t="inlineStr">
+      <c r="C243" s="8" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="D243" s="7" t="inlineStr"/>
+      <c r="E243" s="9" t="inlineStr">
+        <is>
+          <t>☀️ Plan A — Sunny: Achensee — 50 min drive north from Schlegeis · park at Pertisau · Option 1: Achensee steamboat ~€22/adult · allow 1.5hrs · Option 2 (kids tired): Gaisalm promenade walk — free · same fjord-like views ·</t>
+        </is>
+      </c>
+      <c r="F243" s="10" t="inlineStr">
+        <is>
+          <t>50 min / €22 / 5hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="50" customHeight="1">
+      <c r="A244" s="20" t="inlineStr"/>
+      <c r="B244" s="21" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C244" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D244" s="7" t="inlineStr"/>
-      <c r="E244" s="9" t="inlineStr">
-        <is>
-          <t>➕ Optional: Achensee steamboat (Pertisau) — 50 min drive north from Schlegeis · ~€22/adult</t>
-        </is>
-      </c>
-      <c r="F244" s="10" t="inlineStr">
-        <is>
-          <t>50 min / €22</t>
+      <c r="C244" s="22" t="inlineStr">
+        <is>
+          <t>Hike</t>
+        </is>
+      </c>
+      <c r="D244" s="21" t="inlineStr"/>
+      <c r="E244" s="23" t="inlineStr">
+        <is>
+          <t>️ Plan B — Rain/Cloudy: Swarovski Crystal Worlds — 5 min off A12 at Wattens · ~€22/adult · allow 1.5–2hrs · indoor immersive art installation · perfect rainy-day refuge after cold wet Olpererhütte hike · no booking neede</t>
+        </is>
+      </c>
+      <c r="F244" s="24" t="inlineStr">
+        <is>
+          <t>5 min / €22 / 2hr</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day 14: fix timing · 7:45am departure · first cable car 8am · arrive Seebensee 9:45am (beats 10:30am winds) · accurate 5.6km/1.5hr distance · Drachensee 10:15am · Coburger Hutte 11am · back 3pm · e-bikes optional noted
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -970,7 +970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F311"/>
+  <dimension ref="A1:F312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5514,18 +5514,18 @@
     <row r="254" ht="15" customHeight="1">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>Timeline: Tonight: ATM Ehrwald €60–80 cash ▸ 8:30am Bichlbach ▸ 8:45am Ehrwalder Almbahn €26 ▸ Zugspitze platform ▸ 9:15am Seebensee mirror (before 10:30am) ▸ 10:15am Drachensee climb ▸ 11:30am Coburger Hütte Kaiserschmarrn ▸ 1pm descent ▸ 2:30pm Bichlbach + pack ▸ 7:30pm Heiterwanger See sunset</t>
+          <t>Timeline: Tonight: ATM Ehrwald €60–80 ▸ 7:45am Bichlbach ▸ 8:00am Ehrwalder Almbahn (first car) ▸ 8:10am hike ▸ 9:45am Seebensee mirror ▸ 10:15am Drachensee climb ▸ 11:00am Coburger Hütte Kaiserschmarrn ▸ 12:45pm descent ▸ 2:45pm back at car ▸ 3pm Bichlbach ▸ 7:30pm Heiterwanger See sunset</t>
         </is>
       </c>
     </row>
     <row r="255" ht="22" customHeight="1">
       <c r="A255" s="5" t="inlineStr">
         <is>
-          <t>Key: ✅ ATM in Ehrwald tonight — €60–80 cash · Coburger Hütte cash only · no card reader  |   Seebensee mirror reflection before 10:30am — winds create ripples by midday · early start essential  |  ⚠️ Drachensee path slippery if rained Jul 2 — best-grip boots · 260m steep climb</t>
-        </is>
-      </c>
-    </row>
-    <row r="256" ht="40" customHeight="1">
+          <t>Key: ✅ ATM in Ehrwald tonight — €60–80 cash · Coburger Hütte cash only · no card reader  |  ✅ 7:45am departure — first cable car 8:00am · arrive Seebensee 9:45am · beats 10:30am winds  |  ⚠️ Seebensee mirror reflection before 10:30am — winds create ripples by midday · 9:45am arrival ✅  |  ⚠️ Drachensee path slippery if rained Jul 2 — best-grip boots · 217m steep climb · 30–45 min  |  ➕ E-bikes optional at valley station — cuts Seebensee hike from 1.5hrs to 25 min · saves legs for Drachensee</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="50" customHeight="1">
       <c r="A256" s="16" t="inlineStr"/>
       <c r="B256" s="17" t="inlineStr">
         <is>
@@ -5540,12 +5540,12 @@
       <c r="D256" s="17" t="inlineStr"/>
       <c r="E256" s="18" t="inlineStr">
         <is>
-          <t>Tonight (Jul 2 evening): ATM in Ehrwald — withdraw €60–80 cash for the family · Coburger Hütte is cash only — no card reader on the mountain</t>
+          <t>Tonight (Jul 2 evening): ATM in Ehrwald — withdraw €60–80 cash for the family · Coburger Hütte is cash only — no card reader on the mountain · budget: Kaiserschmarrn ~€12 · Tiroler Gröstl ~€14 · drinks ~€4–6 each</t>
         </is>
       </c>
       <c r="F256" s="19" t="inlineStr">
         <is>
-          <t>€60</t>
+          <t>€60 / €12 / €14</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5564,7 @@
       <c r="D257" s="7" t="inlineStr"/>
       <c r="E257" s="9" t="inlineStr">
         <is>
-          <t>⏰ 8:30am — Depart Bichlbach — 5 min drive to the Ehrwalder Almbahn valley station · free parking for cable car guests · arrive ~8:35am</t>
+          <t>7:45am — Depart Bichlbach — 5 min drive to Ehrwalder Almbahn valley station · free parking for cable car guests · arrive ~7:55am</t>
         </is>
       </c>
       <c r="F257" s="10" t="inlineStr">
@@ -5573,7 +5573,7 @@
         </is>
       </c>
     </row>
-    <row r="258" ht="32" customHeight="1">
+    <row r="258" ht="44" customHeight="1">
       <c r="A258" s="16" t="inlineStr"/>
       <c r="B258" s="17" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
       <c r="D258" s="17" t="inlineStr"/>
       <c r="E258" s="18" t="inlineStr">
         <is>
-          <t>⭐ 8:45am — Ehrwalder Almbahn — ~€26/adult · free parking · take 5 min at top for Zugspitze platform view</t>
+          <t>⭐ 8:00am — Ehrwalder Almbahn — first cable car of the day · ~€26/adult · free parking · 5 min at top for Zugspitze platform view · ⚠️ July high season: opens 8:00am</t>
         </is>
       </c>
       <c r="F258" s="19" t="inlineStr">
@@ -5597,180 +5597,191 @@
         </is>
       </c>
     </row>
-    <row r="259" ht="31" customHeight="1">
-      <c r="A259" s="6" t="inlineStr"/>
-      <c r="B259" s="7" t="inlineStr">
+    <row r="259" ht="50" customHeight="1">
+      <c r="A259" s="20" t="inlineStr"/>
+      <c r="B259" s="21" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C259" s="8" t="inlineStr">
+      <c r="C259" s="22" t="inlineStr">
+        <is>
+          <t>Hike</t>
+        </is>
+      </c>
+      <c r="D259" s="21" t="inlineStr"/>
+      <c r="E259" s="23" t="inlineStr">
+        <is>
+          <t>8:10am — Hike to Seebensee — 5.6km from top station · wide gravel path · 152m elevation gain · easy · allow 1.5hrs · arrive ~9:45am · ➕ E-bikes available at valley station — cuts hike to 25 min if family wants to save le</t>
+        </is>
+      </c>
+      <c r="F259" s="24" t="inlineStr">
+        <is>
+          <t>6km / 5hr / 25 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="50" customHeight="1">
+      <c r="A260" s="6" t="inlineStr"/>
+      <c r="B260" s="7" t="inlineStr">
+        <is>
+          <t>Jul 3</t>
+        </is>
+      </c>
+      <c r="C260" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D259" s="7" t="inlineStr"/>
-      <c r="E259" s="9" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ 9:15am — Seebensee — 1.5km flat path · mirror reflection before 10:30am (winds pick up after)</t>
-        </is>
-      </c>
-      <c r="F259" s="10" t="inlineStr">
-        <is>
-          <t>5km</t>
-        </is>
-      </c>
-    </row>
-    <row r="260" ht="32" customHeight="1">
-      <c r="A260" s="20" t="inlineStr"/>
-      <c r="B260" s="21" t="inlineStr">
+      <c r="D260" s="7" t="inlineStr"/>
+      <c r="E260" s="9" t="inlineStr">
+        <is>
+          <t>⭐ ⭐ 9:45am — Seebensee mirror reflection — crystal-clear turquoise water · Zugspitze reflected · winds pick up after 10:30am — 9:45am arrival is perfectly timed · allow 30 min · benches along the southern shore</t>
+        </is>
+      </c>
+      <c r="F260" s="10" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="44" customHeight="1">
+      <c r="A261" s="20" t="inlineStr"/>
+      <c r="B261" s="21" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C260" s="22" t="inlineStr">
+      <c r="C261" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D260" s="21" t="inlineStr"/>
-      <c r="E260" s="23" t="inlineStr">
-        <is>
-          <t>10:15am — Drachensee ascent — 1km steep · 260m gain · ⚠️ slippery if rained Jul 2 · best-grip boots</t>
-        </is>
-      </c>
-      <c r="F260" s="24" t="inlineStr">
-        <is>
-          <t>1km</t>
-        </is>
-      </c>
-    </row>
-    <row r="261" ht="33" customHeight="1">
-      <c r="A261" s="16" t="inlineStr"/>
-      <c r="B261" s="17" t="inlineStr">
+      <c r="D261" s="21" t="inlineStr"/>
+      <c r="E261" s="23" t="inlineStr">
+        <is>
+          <t>10:15am — Drachensee ascent — 1.4km · 217m elevation gain · 30–45 min · ⚠️ slippery if rained Jul 2 · best-grip boots · steeper than Seebensee section but short</t>
+        </is>
+      </c>
+      <c r="F261" s="24" t="inlineStr">
+        <is>
+          <t>4km / 45 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="46" customHeight="1">
+      <c r="A262" s="16" t="inlineStr"/>
+      <c r="B262" s="17" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C261" s="16" t="inlineStr">
+      <c r="C262" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D261" s="17" t="inlineStr"/>
-      <c r="E261" s="18" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ 11:30am — Coburger Hütte (2,026m) — legendary Kaiserschmarrn — MUST · cash only — bring €60–80 family</t>
-        </is>
-      </c>
-      <c r="F261" s="19" t="inlineStr">
-        <is>
-          <t>€60</t>
-        </is>
-      </c>
-    </row>
-    <row r="262" ht="39" customHeight="1">
-      <c r="A262" s="6" t="inlineStr"/>
-      <c r="B262" s="7" t="inlineStr">
+      <c r="D262" s="17" t="inlineStr"/>
+      <c r="E262" s="18" t="inlineStr">
+        <is>
+          <t>⭐ ⭐ 11:00am — Coburger Hütte (1,917m) — legendary Kaiserschmarrn — MUST · cash only — bring €60–80 family · outdoor table facing deep blue Drachensee below · allow 1hr 45min</t>
+        </is>
+      </c>
+      <c r="F262" s="19" t="inlineStr">
+        <is>
+          <t>€60 / 1hr / 45min</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="40" customHeight="1">
+      <c r="A263" s="20" t="inlineStr"/>
+      <c r="B263" s="21" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C262" s="8" t="inlineStr">
+      <c r="C263" s="22" t="inlineStr">
+        <is>
+          <t>Hike</t>
+        </is>
+      </c>
+      <c r="D263" s="21" t="inlineStr"/>
+      <c r="E263" s="23" t="inlineStr">
+        <is>
+          <t>12:45pm — Descent to cable car station — ~1.5hrs back down · same trail · arrive top station ~2:15pm · cable car down · back at car ~2:45pm</t>
+        </is>
+      </c>
+      <c r="F263" s="24" t="inlineStr">
+        <is>
+          <t>5hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="39" customHeight="1">
+      <c r="A264" s="6" t="inlineStr"/>
+      <c r="B264" s="7" t="inlineStr">
+        <is>
+          <t>Jul 3</t>
+        </is>
+      </c>
+      <c r="C264" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D262" s="7" t="inlineStr"/>
-      <c r="E262" s="9" t="inlineStr">
-        <is>
-          <t>1:00pm — Descent to cable car station — back down the ridge · ~1.5hrs · back at Ehrwald valley station ~2:30pm · drive 5 min to Bichlbach</t>
-        </is>
-      </c>
-      <c r="F262" s="10" t="inlineStr">
-        <is>
-          <t>5hr / 5 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="263" ht="39" customHeight="1">
-      <c r="A263" s="6" t="inlineStr"/>
-      <c r="B263" s="7" t="inlineStr">
+      <c r="D264" s="7" t="inlineStr"/>
+      <c r="E264" s="9" t="inlineStr">
+        <is>
+          <t>3:00pm — Back at Landhaus Bichlbach — shower · rest legs · pack bags for tomorrow · checkout 8am — Neuschwanstein 9:30am · alarm 7:00am</t>
+        </is>
+      </c>
+      <c r="F264" s="10" t="inlineStr"/>
+    </row>
+    <row r="265" ht="46" customHeight="1">
+      <c r="A265" s="16" t="inlineStr"/>
+      <c r="B265" s="17" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C263" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D263" s="7" t="inlineStr"/>
-      <c r="E263" s="9" t="inlineStr">
-        <is>
-          <t>2:30pm — Back at Landhaus Bichlbach — relax · shower · pack bags for tomorrow · checkout is 8am — Neuschwanstein 9:30am · alarm 7:00am</t>
-        </is>
-      </c>
-      <c r="F263" s="10" t="inlineStr"/>
-    </row>
-    <row r="264" ht="29" customHeight="1">
-      <c r="A264" s="16" t="inlineStr"/>
-      <c r="B264" s="17" t="inlineStr">
+      <c r="C265" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D265" s="17" t="inlineStr"/>
+      <c r="E265" s="18" t="inlineStr">
+        <is>
+          <t>⭐ 7:30pm — Heiterwanger See sunset walk — 20 min walk from Landhaus along the Panoramaweg · flat · easy · clears the lactic acid · alpenglow after sunset on the higher path</t>
+        </is>
+      </c>
+      <c r="F265" s="19" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" ht="39" customHeight="1">
+      <c r="A266" s="11" t="inlineStr"/>
+      <c r="B266" s="12" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C264" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D264" s="17" t="inlineStr"/>
-      <c r="E264" s="18" t="inlineStr">
-        <is>
-          <t>⭐ 7:30pm — Heiterwanger See sunset walk — 20 min walk from Landhaus along the Panoramaweg</t>
-        </is>
-      </c>
-      <c r="F264" s="19" t="inlineStr">
-        <is>
-          <t>20 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="265" ht="39" customHeight="1">
-      <c r="A265" s="11" t="inlineStr"/>
-      <c r="B265" s="12" t="inlineStr">
-        <is>
-          <t>Jul 3</t>
-        </is>
-      </c>
-      <c r="C265" s="13" t="inlineStr">
+      <c r="C266" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D265" s="12" t="inlineStr"/>
-      <c r="E265" s="14" t="inlineStr">
-        <is>
-          <t>Dinner — Gasthof Bichlbach or hotel restaurant · early dinner + early bed · alarm 7:00am tomorrow · Neuschwanstein 9:30am — last big day</t>
-        </is>
-      </c>
-      <c r="F265" s="15" t="inlineStr"/>
-    </row>
-    <row r="266" ht="33" customHeight="1">
-      <c r="A266" s="30" t="inlineStr"/>
-      <c r="B266" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C266" s="32" t="inlineStr">
-        <is>
-          <t>Coburger Hütte cash only — withdraw €60–80 at Raiffeisenbank ATM in Ehrwald village tonight · budget: Kaiserschmarrn ~€12 · Tiroler Gröstl ~€14 · drinks ~€4–6 each</t>
-        </is>
-      </c>
-    </row>
-    <row r="267" ht="34" customHeight="1">
+      <c r="D266" s="12" t="inlineStr"/>
+      <c r="E266" s="14" t="inlineStr">
+        <is>
+          <t>Dinner — Gasthof Bichlbach or hotel restaurant — early dinner + early bed · alarm 7:00am tomorrow · Neuschwanstein 9:30am — last big day</t>
+        </is>
+      </c>
+      <c r="F266" s="15" t="inlineStr"/>
+    </row>
+    <row r="267" ht="33" customHeight="1">
       <c r="A267" s="30" t="inlineStr"/>
       <c r="B267" s="31" t="inlineStr">
         <is>
@@ -5779,7 +5790,7 @@
       </c>
       <c r="C267" s="32" t="inlineStr">
         <is>
-          <t>Seebensee mirror reflection — must arrive before 10:30am · mountain winds create ripples by midday · morning start from Bichlbach (8:30am) guarantees the calm water window</t>
+          <t>Coburger Hütte cash only — withdraw €60–80 at Raiffeisenbank ATM in Ehrwald village tonight · budget: Kaiserschmarrn ~€12 · Tiroler Gröstl ~€14 · drinks ~€4–6 each</t>
         </is>
       </c>
     </row>
@@ -5792,7 +5803,7 @@
       </c>
       <c r="C268" s="32" t="inlineStr">
         <is>
-          <t>️ Zugspitze platform at top station — take 5 min before walking to Seebensee · look north toward Germany · see the "other side" of the Zugspitze (2,962m) — same peak visible from Garmisch-Partenkirchen</t>
+          <t>Seebensee mirror reflection — must arrive before 10:30am · mountain winds create ripples by midday · morning start from Bichlbach (8:30am) guarantees the calm water window</t>
         </is>
       </c>
     </row>
@@ -5805,88 +5816,77 @@
       </c>
       <c r="C269" s="32" t="inlineStr">
         <is>
+          <t>️ Zugspitze platform at top station — take 5 min before walking to Seebensee · look north toward Germany · see the "other side" of the Zugspitze (2,962m) — same peak visible from Garmisch-Partenkirchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="34" customHeight="1">
+      <c r="A270" s="30" t="inlineStr"/>
+      <c r="B270" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C270" s="32" t="inlineStr">
+        <is>
           <t>Panoramaweg for Heiterwanger See — take the higher Panoramaweg trail not the lakeside path · stays above the valley floor to catch alpenglow after sunset · 20 min from hotel · flat + easy</t>
         </is>
       </c>
     </row>
-    <row r="270" ht="3" customHeight="1">
-      <c r="A270" s="33" t="n"/>
-      <c r="B270" s="33" t="n"/>
-      <c r="C270" s="33" t="n"/>
-      <c r="D270" s="33" t="n"/>
-      <c r="E270" s="33" t="n"/>
-      <c r="F270" s="33" t="n"/>
-    </row>
-    <row r="271" ht="20" customHeight="1">
-      <c r="A271" s="3" t="inlineStr">
+    <row r="271" ht="3" customHeight="1">
+      <c r="A271" s="33" t="n"/>
+      <c r="B271" s="33" t="n"/>
+      <c r="C271" s="33" t="n"/>
+      <c r="D271" s="33" t="n"/>
+      <c r="E271" s="33" t="n"/>
+      <c r="F271" s="33" t="n"/>
+    </row>
+    <row r="272" ht="20" customHeight="1">
+      <c r="A272" s="3" t="inlineStr">
         <is>
           <t>DAY 15  |  Jul 4  |  The Fairy Tale Finale — Neuschwanstein · Ebenalp · Aescher → ZRH  |  ~280 km / 174 mi  ~3h 30m · Neuschwanstein → Ebenalp → ZRH</t>
         </is>
       </c>
     </row>
-    <row r="272" ht="15" customHeight="1">
-      <c r="A272" s="4" t="inlineStr">
+    <row r="273" ht="15" customHeight="1">
+      <c r="A273" s="4" t="inlineStr">
         <is>
           <t>Timeline: 7:30am Bichlbach checkout ▸ 8:15am P4 Neuschwanstein ▸ 8:30am Marienbrücke FIRST ▸ 9:20am castle gate ▸ 9:30am tour ▸ 11:30am drive Bregenz tunnel ▸ 1:15pm Wasserauen ▸ 1:30pm Ebenalp cable car ▸ 2pm Aescher (before Swing event 5pm) ▸ 4pm descent ▸ 6pm ZRH hotel + return car tonight ▸ 5am alarm tomorrow</t>
         </is>
       </c>
     </row>
-    <row r="273" ht="22" customHeight="1">
-      <c r="A273" s="5" t="inlineStr">
+    <row r="274" ht="22" customHeight="1">
+      <c r="A274" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ Marienbrücke BEFORE the tour — go at 8:30am · virtually no queue · by 10am it's packed  |  ⚠️ Castle gate by 9:20am — NOT the ticket centre · guide will not wait for latecomers  |   Return car TONIGHT — drop bags at hotel · 5 min to Europcar ZRH · open until midnight · eliminates 5:30am stress</t>
         </is>
       </c>
     </row>
-    <row r="274" ht="34" customHeight="1">
-      <c r="A274" s="6" t="inlineStr"/>
-      <c r="B274" s="7" t="inlineStr">
+    <row r="275" ht="34" customHeight="1">
+      <c r="A275" s="6" t="inlineStr"/>
+      <c r="B275" s="7" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C274" s="8" t="inlineStr">
+      <c r="C275" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D274" s="7" t="inlineStr"/>
-      <c r="E274" s="9" t="inlineStr">
+      <c r="D275" s="7" t="inlineStr"/>
+      <c r="E275" s="9" t="inlineStr">
         <is>
           <t>⏰ 7:30am — Checkout Landhaus Bichlbach + depart — 30 min earlier than original plan · 45 min drive to Schwangau</t>
         </is>
       </c>
-      <c r="F274" s="10" t="inlineStr">
+      <c r="F275" s="10" t="inlineStr">
         <is>
           <t>30 min / 45 min</t>
         </is>
       </c>
     </row>
-    <row r="275" ht="25" customHeight="1">
-      <c r="A275" s="16" t="inlineStr"/>
-      <c r="B275" s="17" t="inlineStr">
-        <is>
-          <t>Jul 4</t>
-        </is>
-      </c>
-      <c r="C275" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D275" s="17" t="inlineStr"/>
-      <c r="E275" s="18" t="inlineStr">
-        <is>
-          <t>Swiss vignette check — cameras trigger a CHF 200 fine if missing</t>
-        </is>
-      </c>
-      <c r="F275" s="19" t="inlineStr">
-        <is>
-          <t>CHF 200</t>
-        </is>
-      </c>
-    </row>
-    <row r="276" ht="31" customHeight="1">
+    <row r="276" ht="25" customHeight="1">
       <c r="A276" s="16" t="inlineStr"/>
       <c r="B276" s="17" t="inlineStr">
         <is>
@@ -5901,16 +5901,16 @@
       <c r="D276" s="17" t="inlineStr"/>
       <c r="E276" s="18" t="inlineStr">
         <is>
-          <t>8:15am — Park P4, Schwangau — €7 · 10 min walk to ticket centre · go straight to Marienbrücke</t>
+          <t>Swiss vignette check — cameras trigger a CHF 200 fine if missing</t>
         </is>
       </c>
       <c r="F276" s="19" t="inlineStr">
         <is>
-          <t>€7 / 10 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="277" ht="35" customHeight="1">
+          <t>CHF 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="277" ht="31" customHeight="1">
       <c r="A277" s="16" t="inlineStr"/>
       <c r="B277" s="17" t="inlineStr">
         <is>
@@ -5925,16 +5925,16 @@
       <c r="D277" s="17" t="inlineStr"/>
       <c r="E277" s="18" t="inlineStr">
         <is>
-          <t>⭐ ⭐ 8:30am — Marienbrücke (Mary's Bridge) — go here FIRST — 10 min walk above the castle · allow 20–30 min for photos</t>
+          <t>8:15am — Park P4, Schwangau — €7 · 10 min walk to ticket centre · go straight to Marienbrücke</t>
         </is>
       </c>
       <c r="F277" s="19" t="inlineStr">
         <is>
-          <t>10 min / 30 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="278" ht="29" customHeight="1">
+          <t>€7 / 10 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="278" ht="35" customHeight="1">
       <c r="A278" s="16" t="inlineStr"/>
       <c r="B278" s="17" t="inlineStr">
         <is>
@@ -5949,12 +5949,16 @@
       <c r="D278" s="17" t="inlineStr"/>
       <c r="E278" s="18" t="inlineStr">
         <is>
-          <t>⚠️ 9:20am — Castle GATE (not ticket centre) — entry strictly timed · guide will not wait</t>
-        </is>
-      </c>
-      <c r="F278" s="19" t="inlineStr"/>
-    </row>
-    <row r="279" ht="34" customHeight="1">
+          <t>⭐ ⭐ 8:30am — Marienbrücke (Mary's Bridge) — go here FIRST — 10 min walk above the castle · allow 20–30 min for photos</t>
+        </is>
+      </c>
+      <c r="F278" s="19" t="inlineStr">
+        <is>
+          <t>10 min / 30 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="279" ht="29" customHeight="1">
       <c r="A279" s="16" t="inlineStr"/>
       <c r="B279" s="17" t="inlineStr">
         <is>
@@ -5969,217 +5973,224 @@
       <c r="D279" s="17" t="inlineStr"/>
       <c r="E279" s="18" t="inlineStr">
         <is>
+          <t>⚠️ 9:20am — Castle GATE (not ticket centre) — entry strictly timed · guide will not wait</t>
+        </is>
+      </c>
+      <c r="F279" s="19" t="inlineStr"/>
+    </row>
+    <row r="280" ht="34" customHeight="1">
+      <c r="A280" s="16" t="inlineStr"/>
+      <c r="B280" s="17" t="inlineStr">
+        <is>
+          <t>Jul 4</t>
+        </is>
+      </c>
+      <c r="C280" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D280" s="17" t="inlineStr"/>
+      <c r="E280" s="18" t="inlineStr">
+        <is>
           <t>⭐ ⭐ 9:30am — Neuschwanstein Castle interior tour — guided tour 35–40 min inside · photography not allowed inside</t>
         </is>
       </c>
-      <c r="F279" s="19" t="inlineStr">
+      <c r="F280" s="19" t="inlineStr">
         <is>
           <t>40 min</t>
         </is>
       </c>
     </row>
-    <row r="280" ht="37" customHeight="1">
-      <c r="A280" s="6" t="inlineStr"/>
-      <c r="B280" s="7" t="inlineStr">
+    <row r="281" ht="37" customHeight="1">
+      <c r="A281" s="6" t="inlineStr"/>
+      <c r="B281" s="7" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C280" s="8" t="inlineStr">
+      <c r="C281" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D280" s="7" t="inlineStr"/>
-      <c r="E280" s="9" t="inlineStr">
+      <c r="D281" s="7" t="inlineStr"/>
+      <c r="E281" s="9" t="inlineStr">
         <is>
           <t>11:30am — Depart Neuschwanstein → Wasserauen — 1hr 30min drive · ⚠️ Saturday = absolute peak crowds on all German/Swiss roads</t>
         </is>
       </c>
-      <c r="F280" s="10" t="inlineStr">
+      <c r="F281" s="10" t="inlineStr">
         <is>
           <t>1hr / 30min</t>
         </is>
       </c>
     </row>
-    <row r="281" ht="30" customHeight="1">
-      <c r="A281" s="16" t="inlineStr"/>
-      <c r="B281" s="17" t="inlineStr">
+    <row r="282" ht="30" customHeight="1">
+      <c r="A282" s="16" t="inlineStr"/>
+      <c r="B282" s="17" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C281" s="16" t="inlineStr">
+      <c r="C282" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D281" s="17" t="inlineStr"/>
-      <c r="E281" s="18" t="inlineStr">
+      <c r="D282" s="17" t="inlineStr"/>
+      <c r="E282" s="18" t="inlineStr">
         <is>
           <t>1:15pm — Park at Wasserauen cable car — CHF 36/adult return (2026 rate) · runs every 15 min</t>
         </is>
       </c>
-      <c r="F281" s="19" t="inlineStr">
+      <c r="F282" s="19" t="inlineStr">
         <is>
           <t>CHF 36 / 15 min</t>
         </is>
       </c>
     </row>
-    <row r="282" ht="32" customHeight="1">
-      <c r="A282" s="20" t="inlineStr"/>
-      <c r="B282" s="21" t="inlineStr">
+    <row r="283" ht="32" customHeight="1">
+      <c r="A283" s="20" t="inlineStr"/>
+      <c r="B283" s="21" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C282" s="22" t="inlineStr">
+      <c r="C283" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D282" s="21" t="inlineStr"/>
-      <c r="E282" s="23" t="inlineStr">
+      <c r="D283" s="21" t="inlineStr"/>
+      <c r="E283" s="23" t="inlineStr">
         <is>
           <t>⭐ 1:30pm — Ebenalp cable car — CHF 36/adult · 6 min · last descent 6pm · ⚠️ caves 10°C — pack a layer</t>
         </is>
       </c>
-      <c r="F282" s="24" t="inlineStr">
+      <c r="F283" s="24" t="inlineStr">
         <is>
           <t>CHF 36 / 6 min</t>
         </is>
       </c>
     </row>
-    <row r="283" ht="35" customHeight="1">
-      <c r="A283" s="16" t="inlineStr"/>
-      <c r="B283" s="17" t="inlineStr">
+    <row r="284" ht="35" customHeight="1">
+      <c r="A284" s="16" t="inlineStr"/>
+      <c r="B284" s="17" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C283" s="16" t="inlineStr">
+      <c r="C284" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D283" s="17" t="inlineStr"/>
-      <c r="E283" s="18" t="inlineStr">
+      <c r="D284" s="17" t="inlineStr"/>
+      <c r="E284" s="18" t="inlineStr">
         <is>
           <t>⭐ ⭐ 2:00pm — Berggasthaus Aescher — arrive before 4pm ·  Swing event 5pm · Chäs-Chnöpfli or Rösti · Siedwurst if full</t>
         </is>
       </c>
-      <c r="F283" s="19" t="inlineStr"/>
-    </row>
-    <row r="284" ht="39" customHeight="1">
-      <c r="A284" s="6" t="inlineStr"/>
-      <c r="B284" s="7" t="inlineStr">
+      <c r="F284" s="19" t="inlineStr"/>
+    </row>
+    <row r="285" ht="39" customHeight="1">
+      <c r="A285" s="6" t="inlineStr"/>
+      <c r="B285" s="7" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C284" s="8" t="inlineStr">
+      <c r="C285" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D284" s="7" t="inlineStr"/>
-      <c r="E284" s="9" t="inlineStr">
+      <c r="D285" s="7" t="inlineStr"/>
+      <c r="E285" s="9" t="inlineStr">
         <is>
           <t>4:00pm — Cable car down + drive to ZRH — walk 25 min back up to Ebenalp top station · cable car down · ~2hr drive to Zurich Airport area</t>
         </is>
       </c>
-      <c r="F284" s="10" t="inlineStr">
+      <c r="F285" s="10" t="inlineStr">
         <is>
           <t>25 min / ~2hr</t>
         </is>
       </c>
     </row>
-    <row r="285" ht="33" customHeight="1">
-      <c r="A285" s="16" t="inlineStr"/>
-      <c r="B285" s="17" t="inlineStr">
+    <row r="286" ht="33" customHeight="1">
+      <c r="A286" s="16" t="inlineStr"/>
+      <c r="B286" s="17" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C285" s="16" t="inlineStr">
+      <c r="C286" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D285" s="17" t="inlineStr"/>
-      <c r="E285" s="18" t="inlineStr">
+      <c r="D286" s="17" t="inlineStr"/>
+      <c r="E286" s="18" t="inlineStr">
         <is>
           <t>❌ Rhine Falls — SKIP TODAY — adding 45 min detour north on a peak Saturday risks missing car return window</t>
         </is>
       </c>
-      <c r="F285" s="19" t="inlineStr">
+      <c r="F286" s="19" t="inlineStr">
         <is>
           <t>45 min</t>
         </is>
       </c>
     </row>
-    <row r="286" ht="50" customHeight="1">
-      <c r="A286" s="6" t="inlineStr"/>
-      <c r="B286" s="7" t="inlineStr">
+    <row r="287" ht="50" customHeight="1">
+      <c r="A287" s="6" t="inlineStr"/>
+      <c r="B287" s="7" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C286" s="8" t="inlineStr">
+      <c r="C287" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D286" s="7" t="inlineStr"/>
-      <c r="E286" s="9" t="inlineStr">
+      <c r="D287" s="7" t="inlineStr"/>
+      <c r="E287" s="9" t="inlineStr">
         <is>
           <t>Return Europcar ZRH tonight — drop bags at Airport Hotel Zurich · drive 5 min to Europcar ZRH return · return by 11:30pm · Hilton shuttle back · check Booking.com email for return confirmation</t>
         </is>
       </c>
-      <c r="F286" s="10" t="inlineStr">
+      <c r="F287" s="10" t="inlineStr">
         <is>
           <t>5 min</t>
         </is>
       </c>
     </row>
-    <row r="287" ht="28" customHeight="1">
-      <c r="A287" s="25" t="inlineStr"/>
-      <c r="B287" s="26" t="inlineStr">
+    <row r="288" ht="28" customHeight="1">
+      <c r="A288" s="25" t="inlineStr"/>
+      <c r="B288" s="26" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C287" s="27" t="inlineStr">
+      <c r="C288" s="27" t="inlineStr">
         <is>
           <t>Stay</t>
         </is>
       </c>
-      <c r="D287" s="26" t="inlineStr"/>
-      <c r="E287" s="28" t="inlineStr">
+      <c r="D288" s="26" t="inlineStr"/>
+      <c r="E288" s="28" t="inlineStr">
         <is>
           <t>⚠️ Tonight — final checks — check-in opens 5:30am · hotel is 5 min walk to terminal</t>
         </is>
       </c>
-      <c r="F287" s="29" t="inlineStr">
+      <c r="F288" s="29" t="inlineStr">
         <is>
           <t>5 min</t>
         </is>
       </c>
     </row>
-    <row r="288" ht="31" customHeight="1">
-      <c r="A288" s="30" t="inlineStr"/>
-      <c r="B288" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C288" s="32" t="inlineStr">
-        <is>
-          <t>⚠️ Castle gate 9:20am — be at the GATE not the ticket centre by 9:20am · €17.50/adult incl. booking fee · guide does not wait · strictly timed entry</t>
-        </is>
-      </c>
-    </row>
-    <row r="289" ht="34" customHeight="1">
+    <row r="289" ht="31" customHeight="1">
       <c r="A289" s="30" t="inlineStr"/>
       <c r="B289" s="31" t="inlineStr">
         <is>
@@ -6188,11 +6199,11 @@
       </c>
       <c r="C289" s="32" t="inlineStr">
         <is>
-          <t>Aescher Swing event Jul 4 from 5pm — restaurant will be extremely crowded for the evening event · arrive 1:30–2:00pm · eat + leave before 4pm · if terrace full: Siedwurst at the kiosk + wooden bench · same views</t>
-        </is>
-      </c>
-    </row>
-    <row r="290" ht="30" customHeight="1">
+          <t>⚠️ Castle gate 9:20am — be at the GATE not the ticket centre by 9:20am · €17.50/adult incl. booking fee · guide does not wait · strictly timed entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="34" customHeight="1">
       <c r="A290" s="30" t="inlineStr"/>
       <c r="B290" s="31" t="inlineStr">
         <is>
@@ -6201,11 +6212,11 @@
       </c>
       <c r="C290" s="32" t="inlineStr">
         <is>
-          <t>Wildkirchli caves — 30°C outside · 10°C inside the caves · pack a light layer in your daypack · 5 min walk through the cave on the path to Aescher</t>
-        </is>
-      </c>
-    </row>
-    <row r="291" ht="34" customHeight="1">
+          <t>Aescher Swing event Jul 4 from 5pm — restaurant will be extremely crowded for the evening event · arrive 1:30–2:00pm · eat + leave before 4pm · if terrace full: Siedwurst at the kiosk + wooden bench · same views</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="30" customHeight="1">
       <c r="A291" s="30" t="inlineStr"/>
       <c r="B291" s="31" t="inlineStr">
         <is>
@@ -6214,7 +6225,7 @@
       </c>
       <c r="C291" s="32" t="inlineStr">
         <is>
-          <t>Return car tonight — drop bags at Airport Hotel Zurich · drive 5 min to Europcar ZRH car return · take Hilton shuttle back · Europcar open until midnight · eliminates 5:30am stress tomorrow</t>
+          <t>Wildkirchli caves — 30°C outside · 10°C inside the caves · pack a light layer in your daypack · 5 min walk through the cave on the path to Aescher</t>
         </is>
       </c>
     </row>
@@ -6227,11 +6238,11 @@
       </c>
       <c r="C292" s="32" t="inlineStr">
         <is>
-          <t>Aescher food — Chäs-Chnöpfli (Swiss mac and cheese with Appenzeller) · or Rösti · or Siedwurst at the kiosk if terrace full · same cliff view from the wooden benches outside</t>
-        </is>
-      </c>
-    </row>
-    <row r="293" ht="32" customHeight="1">
+          <t>Return car tonight — drop bags at Airport Hotel Zurich · drive 5 min to Europcar ZRH car return · take Hilton shuttle back · Europcar open until midnight · eliminates 5:30am stress tomorrow</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="34" customHeight="1">
       <c r="A293" s="30" t="inlineStr"/>
       <c r="B293" s="31" t="inlineStr">
         <is>
@@ -6240,148 +6251,137 @@
       </c>
       <c r="C293" s="32" t="inlineStr">
         <is>
+          <t>Aescher food — Chäs-Chnöpfli (Swiss mac and cheese with Appenzeller) · or Rösti · or Siedwurst at the kiosk if terrace full · same cliff view from the wooden benches outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="32" customHeight="1">
+      <c r="A294" s="30" t="inlineStr"/>
+      <c r="B294" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C294" s="32" t="inlineStr">
+        <is>
           <t>⚠️ 5:00am alarm Jul 5 — set two alarms · FI571 departs 7:55am · check-in opens 5:30am · hotel is 5 min walk to terminal · boarding passes on phone tonight</t>
         </is>
       </c>
     </row>
-    <row r="294" ht="3" customHeight="1">
-      <c r="A294" s="33" t="n"/>
-      <c r="B294" s="33" t="n"/>
-      <c r="C294" s="33" t="n"/>
-      <c r="D294" s="33" t="n"/>
-      <c r="E294" s="33" t="n"/>
-      <c r="F294" s="33" t="n"/>
-    </row>
-    <row r="295" ht="20" customHeight="1">
-      <c r="A295" s="3" t="inlineStr">
+    <row r="295" ht="3" customHeight="1">
+      <c r="A295" s="33" t="n"/>
+      <c r="B295" s="33" t="n"/>
+      <c r="C295" s="33" t="n"/>
+      <c r="D295" s="33" t="n"/>
+      <c r="E295" s="33" t="n"/>
+      <c r="F295" s="33" t="n"/>
+    </row>
+    <row r="296" ht="20" customHeight="1">
+      <c r="A296" s="3" t="inlineStr">
         <is>
           <t>DAY 16  |  Jul 5  |  Homebound — ZRH → KEF → MCO · The Final Leg  |  —  —</t>
         </is>
       </c>
     </row>
-    <row r="296" ht="15" customHeight="1">
-      <c r="A296" s="4" t="inlineStr">
+    <row r="297" ht="15" customHeight="1">
+      <c r="A297" s="4" t="inlineStr">
         <is>
           <t>Timeline: Sat night: app check-in ▸ confirm shuttle ▸ 5am wake ▸ 5:30am Hilton shuttle (NOT walk) ▸ 5:45am Terminal 2 · Check-in Row 3 ▸ 6am security + E Gate Skymetro ▸ 7:55am FI571 ZRH→KEF ▸ KEF Pylsur layover ▸ 8:50pm MCO home</t>
         </is>
       </c>
     </row>
-    <row r="297" ht="22" customHeight="1">
-      <c r="A297" s="5" t="inlineStr">
+    <row r="298" ht="22" customHeight="1">
+      <c r="A298" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ Take hotel shuttle NOT walk — Hilton is 2km from terminal · not walkable with luggage · CHF 7/person  |  ✅ Icelandair app check-in Saturday night — digital boarding pass · fast bag drop at Check-in 2 Row 3  |  ✅ US Customs at MCO not KEF — do not leave transit area in Iceland</t>
         </is>
       </c>
     </row>
-    <row r="298" ht="39" customHeight="1">
-      <c r="A298" s="34" t="inlineStr"/>
-      <c r="B298" s="35" t="inlineStr">
+    <row r="299" ht="39" customHeight="1">
+      <c r="A299" s="34" t="inlineStr"/>
+      <c r="B299" s="35" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C298" s="36" t="inlineStr">
+      <c r="C299" s="36" t="inlineStr">
         <is>
           <t>Alert</t>
         </is>
       </c>
-      <c r="D298" s="35" t="inlineStr"/>
-      <c r="E298" s="37" t="inlineStr">
+      <c r="D299" s="35" t="inlineStr"/>
+      <c r="E299" s="37" t="inlineStr">
         <is>
           <t>✅ Night before (Jul 4 Saturday evening) — final prep — (2) Check Europcar/Booking.com email — confirm car return was closed out correctly</t>
         </is>
       </c>
-      <c r="F298" s="38" t="inlineStr"/>
-    </row>
-    <row r="299" ht="40" customHeight="1">
-      <c r="A299" s="11" t="inlineStr"/>
-      <c r="B299" s="12" t="inlineStr">
+      <c r="F299" s="38" t="inlineStr"/>
+    </row>
+    <row r="300" ht="40" customHeight="1">
+      <c r="A300" s="11" t="inlineStr"/>
+      <c r="B300" s="12" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C299" s="13" t="inlineStr">
+      <c r="C300" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D299" s="12" t="inlineStr"/>
-      <c r="E299" s="14" t="inlineStr">
+      <c r="D300" s="12" t="inlineStr"/>
+      <c r="E300" s="14" t="inlineStr">
         <is>
           <t>⏰ 5:00am — Wake up — perfect timing · do not wake earlier unless extra bags need special handling · hotel breakfast starts at 5:30am if needed</t>
         </is>
       </c>
-      <c r="F299" s="15" t="inlineStr"/>
-    </row>
-    <row r="300" ht="31" customHeight="1">
-      <c r="A300" s="16" t="inlineStr"/>
-      <c r="B300" s="17" t="inlineStr">
+      <c r="F300" s="15" t="inlineStr"/>
+    </row>
+    <row r="301" ht="31" customHeight="1">
+      <c r="A301" s="16" t="inlineStr"/>
+      <c r="B301" s="17" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C300" s="16" t="inlineStr">
+      <c r="C301" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D300" s="17" t="inlineStr"/>
-      <c r="E300" s="18" t="inlineStr">
+      <c r="D301" s="17" t="inlineStr"/>
+      <c r="E301" s="18" t="inlineStr">
         <is>
           <t>⚠️ 5:30am — Hilton shuttle — ❌ do NOT walk · 2km to terminal · CHF 7/person · confirm seat tonight</t>
         </is>
       </c>
-      <c r="F300" s="19" t="inlineStr">
+      <c r="F301" s="19" t="inlineStr">
         <is>
           <t>2km / CHF 7</t>
         </is>
       </c>
     </row>
-    <row r="301" ht="31" customHeight="1">
-      <c r="A301" s="25" t="inlineStr"/>
-      <c r="B301" s="26" t="inlineStr">
+    <row r="302" ht="31" customHeight="1">
+      <c r="A302" s="25" t="inlineStr"/>
+      <c r="B302" s="26" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C301" s="27" t="inlineStr">
+      <c r="C302" s="27" t="inlineStr">
         <is>
           <t>Stay</t>
         </is>
       </c>
-      <c r="D301" s="26" t="inlineStr"/>
-      <c r="E301" s="28" t="inlineStr">
+      <c r="D302" s="26" t="inlineStr"/>
+      <c r="E302" s="28" t="inlineStr">
         <is>
           <t>✈️ 5:45am — Terminal 2, Check-in Row 3 — bag drop opens 5:25am · digital boarding pass on phone</t>
         </is>
       </c>
-      <c r="F301" s="29" t="inlineStr"/>
-    </row>
-    <row r="302" ht="30" customHeight="1">
-      <c r="A302" s="16" t="inlineStr"/>
-      <c r="B302" s="17" t="inlineStr">
-        <is>
-          <t>Jul 5</t>
-        </is>
-      </c>
-      <c r="C302" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D302" s="17" t="inlineStr"/>
-      <c r="E302" s="18" t="inlineStr">
-        <is>
-          <t>6:00am — Security + E Gates — Skymetro train from main terminal · allow 45 min · Sunday busy</t>
-        </is>
-      </c>
-      <c r="F302" s="19" t="inlineStr">
-        <is>
-          <t>45 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="303" ht="38" customHeight="1">
+      <c r="F302" s="29" t="inlineStr"/>
+    </row>
+    <row r="303" ht="30" customHeight="1">
       <c r="A303" s="16" t="inlineStr"/>
       <c r="B303" s="17" t="inlineStr">
         <is>
@@ -6396,56 +6396,56 @@
       <c r="D303" s="17" t="inlineStr"/>
       <c r="E303" s="18" t="inlineStr">
         <is>
+          <t>6:00am — Security + E Gates — Skymetro train from main terminal · allow 45 min · Sunday busy</t>
+        </is>
+      </c>
+      <c r="F303" s="19" t="inlineStr">
+        <is>
+          <t>45 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="38" customHeight="1">
+      <c r="A304" s="16" t="inlineStr"/>
+      <c r="B304" s="17" t="inlineStr">
+        <is>
+          <t>Jul 5</t>
+        </is>
+      </c>
+      <c r="C304" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D304" s="17" t="inlineStr"/>
+      <c r="E304" s="18" t="inlineStr">
+        <is>
           <t>Spend remaining Swiss Francs — airport shops + cafés open by 6:00am · CHF coins and small bills are hard to exchange back in the US</t>
         </is>
       </c>
-      <c r="F303" s="19" t="inlineStr"/>
-    </row>
-    <row r="304" ht="19" customHeight="1">
-      <c r="A304" s="6" t="inlineStr"/>
-      <c r="B304" s="7" t="inlineStr">
+      <c r="F304" s="19" t="inlineStr"/>
+    </row>
+    <row r="305" ht="19" customHeight="1">
+      <c r="A305" s="6" t="inlineStr"/>
+      <c r="B305" s="7" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C304" s="8" t="inlineStr">
+      <c r="C305" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D304" s="7" t="inlineStr"/>
-      <c r="E304" s="9" t="inlineStr">
+      <c r="D305" s="7" t="inlineStr"/>
+      <c r="E305" s="9" t="inlineStr">
         <is>
           <t>✈️ 7:55am — FI571 departs ZRH → KEF</t>
         </is>
       </c>
-      <c r="F304" s="10" t="inlineStr"/>
-    </row>
-    <row r="305" ht="37" customHeight="1">
-      <c r="A305" s="16" t="inlineStr"/>
-      <c r="B305" s="17" t="inlineStr">
-        <is>
-          <t>Jul 5</t>
-        </is>
-      </c>
-      <c r="C305" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D305" s="17" t="inlineStr"/>
-      <c r="E305" s="18" t="inlineStr">
-        <is>
-          <t>KEF layover tip — 1.5–2hr layover is just enough time · grab a Pylsur — duty-free is excellent here if you missed anything</t>
-        </is>
-      </c>
-      <c r="F305" s="19" t="inlineStr">
-        <is>
-          <t>2hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="306" ht="35" customHeight="1">
+      <c r="F305" s="10" t="inlineStr"/>
+    </row>
+    <row r="306" ht="37" customHeight="1">
       <c r="A306" s="16" t="inlineStr"/>
       <c r="B306" s="17" t="inlineStr">
         <is>
@@ -6460,25 +6460,36 @@
       <c r="D306" s="17" t="inlineStr"/>
       <c r="E306" s="18" t="inlineStr">
         <is>
+          <t>KEF layover tip — 1.5–2hr layover is just enough time · grab a Pylsur — duty-free is excellent here if you missed anything</t>
+        </is>
+      </c>
+      <c r="F306" s="19" t="inlineStr">
+        <is>
+          <t>2hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="35" customHeight="1">
+      <c r="A307" s="16" t="inlineStr"/>
+      <c r="B307" s="17" t="inlineStr">
+        <is>
+          <t>Jul 5</t>
+        </is>
+      </c>
+      <c r="C307" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D307" s="17" t="inlineStr"/>
+      <c r="E307" s="18" t="inlineStr">
+        <is>
           <t>8:50pm — Arrive Orlando MCO — clear US Customs + Immigration at MCO · allow 45–60 min for customs on Sunday evening</t>
         </is>
       </c>
-      <c r="F306" s="19" t="inlineStr">
+      <c r="F307" s="19" t="inlineStr">
         <is>
           <t>60 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="307" ht="34" customHeight="1">
-      <c r="A307" s="30" t="inlineStr"/>
-      <c r="B307" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C307" s="32" t="inlineStr">
-        <is>
-          <t>⚠️ Do NOT walk to terminal — Hilton Zurich Airport is ~2km from Terminal 2 in Glattbrugg · take the hotel shuttle · CHF 7/person · confirm 5:30am seat at front desk on Saturday evening</t>
         </is>
       </c>
     </row>
@@ -6491,7 +6502,7 @@
       </c>
       <c r="C308" s="32" t="inlineStr">
         <is>
-          <t>Saturday night app check-in — Icelandair app · download boarding passes to Apple/Google Wallet · check Europcar email for car return confirmation · passports in hand-carry bag · two alarms set</t>
+          <t>⚠️ Do NOT walk to terminal — Hilton Zurich Airport is ~2km from Terminal 2 in Glattbrugg · take the hotel shuttle · CHF 7/person · confirm 5:30am seat at front desk on Saturday evening</t>
         </is>
       </c>
     </row>
@@ -6504,11 +6515,11 @@
       </c>
       <c r="C309" s="32" t="inlineStr">
         <is>
-          <t>ZRH Terminal 2 details — Icelandair Check-in 2, Row 3 · E Gates for US-bound flights · Skymetro train from main terminal · extra security check at E Gate is standard · allow 45 min total at airport before gate</t>
-        </is>
-      </c>
-    </row>
-    <row r="310" ht="31" customHeight="1">
+          <t>Saturday night app check-in — Icelandair app · download boarding passes to Apple/Google Wallet · check Europcar email for car return confirmation · passports in hand-carry bag · two alarms set</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="34" customHeight="1">
       <c r="A310" s="30" t="inlineStr"/>
       <c r="B310" s="31" t="inlineStr">
         <is>
@@ -6517,17 +6528,30 @@
       </c>
       <c r="C310" s="32" t="inlineStr">
         <is>
+          <t>ZRH Terminal 2 details — Icelandair Check-in 2, Row 3 · E Gates for US-bound flights · Skymetro train from main terminal · extra security check at E Gate is standard · allow 45 min total at airport before gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="31" customHeight="1">
+      <c r="A311" s="30" t="inlineStr"/>
+      <c r="B311" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C311" s="32" t="inlineStr">
+        <is>
           <t>KEF layover — 1.5–2hrs · Pylsur hot dog (best in the world) · Skyr yoghurt · duty-free is excellent · US customs at MCO not here · do not leave transit</t>
         </is>
       </c>
     </row>
-    <row r="311" ht="3" customHeight="1">
-      <c r="A311" s="33" t="n"/>
-      <c r="B311" s="33" t="n"/>
-      <c r="C311" s="33" t="n"/>
-      <c r="D311" s="33" t="n"/>
-      <c r="E311" s="33" t="n"/>
-      <c r="F311" s="33" t="n"/>
+    <row r="312" ht="3" customHeight="1">
+      <c r="A312" s="33" t="n"/>
+      <c r="B312" s="33" t="n"/>
+      <c r="C312" s="33" t="n"/>
+      <c r="D312" s="33" t="n"/>
+      <c r="E312" s="33" t="n"/>
+      <c r="F312" s="33" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="110">
@@ -6546,6 +6570,7 @@
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="C172:F172"/>
     <mergeCell ref="A121:F121"/>
+    <mergeCell ref="A274:F274"/>
     <mergeCell ref="C73:F73"/>
     <mergeCell ref="C250:F250"/>
     <mergeCell ref="C231:F231"/>
@@ -6565,7 +6590,6 @@
     <mergeCell ref="A254:F254"/>
     <mergeCell ref="C175:F175"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="C288:F288"/>
     <mergeCell ref="A122:F122"/>
     <mergeCell ref="A215:F215"/>
     <mergeCell ref="C98:F98"/>
@@ -6597,9 +6621,9 @@
     <mergeCell ref="A100:F100"/>
     <mergeCell ref="A253:F253"/>
     <mergeCell ref="A180:F180"/>
+    <mergeCell ref="C294:F294"/>
     <mergeCell ref="C97:F97"/>
     <mergeCell ref="A102:F102"/>
-    <mergeCell ref="A295:F295"/>
     <mergeCell ref="C94:F94"/>
     <mergeCell ref="C152:F152"/>
     <mergeCell ref="A157:F157"/>
@@ -6610,7 +6634,6 @@
     <mergeCell ref="C51:F51"/>
     <mergeCell ref="C95:F95"/>
     <mergeCell ref="A78:F78"/>
-    <mergeCell ref="A271:F271"/>
     <mergeCell ref="A255:F255"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="A273:F273"/>
@@ -6621,11 +6644,10 @@
     <mergeCell ref="A235:F235"/>
     <mergeCell ref="C154:F154"/>
     <mergeCell ref="C267:F267"/>
-    <mergeCell ref="C307:F307"/>
     <mergeCell ref="C49:F49"/>
+    <mergeCell ref="A298:F298"/>
     <mergeCell ref="A194:F194"/>
     <mergeCell ref="A234:F234"/>
-    <mergeCell ref="C266:F266"/>
     <mergeCell ref="C33:F33"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="C269:F269"/>
@@ -6636,8 +6658,10 @@
     <mergeCell ref="C117:F117"/>
     <mergeCell ref="A77:F77"/>
     <mergeCell ref="C230:F230"/>
+    <mergeCell ref="C270:F270"/>
     <mergeCell ref="C118:F118"/>
     <mergeCell ref="C75:F75"/>
+    <mergeCell ref="C311:F311"/>
     <mergeCell ref="A138:F138"/>
     <mergeCell ref="C232:F232"/>
     <mergeCell ref="A196:F196"/>

</xml_diff>

<commit_message>
Day 15 redesigned: skip Neuschwanstein + Ebenalp · Bichlbach direct to ZRH ~185km ~2hrs · Zurich Old Town (Lindenhof + Grossmünster + Fraumünster) · Bahnhofstrasse + Sprüngli · Lake Zurich · Caliente! Latin Festival (Jul 4 final day) · dinner by lake · Neuschwanstein removed from checklist
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -5979,25 +5979,25 @@
     <row r="279" ht="20" customHeight="1">
       <c r="A279" s="3" t="inlineStr">
         <is>
-          <t>DAY 15  |  Jul 4  |  The Fairy Tale Finale — Neuschwanstein · Ebenalp · Aescher → ZRH  |  ~280 km / 174 mi  ~3h 30m · Neuschwanstein → Ebenalp → ZRH</t>
+          <t>DAY 15  |  Jul 4  |  Zurich Day — Old Town · Lake · Caliente Festival → ZRH  |  ~185 km / 115 mi  ~2h direct · saves 100km vs castle route</t>
         </is>
       </c>
     </row>
     <row r="280" ht="15" customHeight="1">
       <c r="A280" s="4" t="inlineStr">
         <is>
-          <t>Timeline: 7:30am Bichlbach checkout ▸ 8:15am P4 Neuschwanstein ▸ 8:30am Marienbrücke FIRST ▸ 9:20am castle gate ▸ 9:30am tour ▸ 11:30am drive Bregenz tunnel ▸ 1:15pm Wasserauen ▸ 1:30pm Ebenalp cable car ▸ 2pm Aescher (before Swing event 5pm) ▸ 4pm descent ▸ 6pm ZRH hotel + return car tonight ▸ 5am alarm tomorrow</t>
+          <t>Timeline: 8:00am Bichlbach checkout ▸ ~10:00am Airport Hotel ZRH ▸ 10:30am return Europcar ▸ 11:00am train to Zurich HB ▸ 11:15am Lindenhof + Grossmünster + Fraumünster ▸ 1:00pm Bahnhofstrasse + Sprüngli ▸ 1:45pm Lake Zurich waterfront ▸ 2:30pm Caliente! Latin Festival ▸ 4:30pm dinner by the lake ▸ 6:00pm train back ▸ early bed</t>
         </is>
       </c>
     </row>
     <row r="281" ht="22" customHeight="1">
       <c r="A281" s="5" t="inlineStr">
         <is>
-          <t>Key: ✅ Marienbrücke BEFORE the tour — go at 8:30am · virtually no queue · by 10am it's packed  |  ⚠️ Castle gate by 9:20am — NOT the ticket centre · guide will not wait for latecomers  |   Return car TONIGHT — drop bags at hotel · 5 min to Europcar ZRH · open until midnight · eliminates 5:30am stress</t>
-        </is>
-      </c>
-    </row>
-    <row r="282" ht="34" customHeight="1">
+          <t>Key: ✅ Return Europcar ZRH first thing — 10:30am · 5 min drive · done before Zurich  |  ✅ Caliente! Latin Festival Jul 4 — final day · Europe's largest Latin festival · lakefront · family-friendly  |  ✅ Confirm Hilton shuttle 5:30am at front desk tonight — CHF 7/person · NOT walk (2km)  |  ⚠️ Swiss vignette — verify on windscreen before crossing border</t>
+        </is>
+      </c>
+    </row>
+    <row r="282" ht="44" customHeight="1">
       <c r="A282" s="6" t="inlineStr"/>
       <c r="B282" s="7" t="inlineStr">
         <is>
@@ -6012,16 +6012,16 @@
       <c r="D282" s="7" t="inlineStr"/>
       <c r="E282" s="9" t="inlineStr">
         <is>
-          <t>⏰ 7:30am — Checkout Landhaus Bichlbach + depart — 30 min earlier than original plan · 45 min drive to Schwangau</t>
+          <t>8:00am — Checkout Landhaus Bichlbach + depart — ~185km direct to Zurich Airport · ~2hrs via A17/A12/A14 · no border stress · no peak Saturday mountain parking</t>
         </is>
       </c>
       <c r="F282" s="10" t="inlineStr">
         <is>
-          <t>30 min / 45 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="283" ht="25" customHeight="1">
+          <t>~185km / ~2hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="283" ht="35" customHeight="1">
       <c r="A283" s="16" t="inlineStr"/>
       <c r="B283" s="17" t="inlineStr">
         <is>
@@ -6036,7 +6036,7 @@
       <c r="D283" s="17" t="inlineStr"/>
       <c r="E283" s="18" t="inlineStr">
         <is>
-          <t>Swiss vignette check — cameras trigger a CHF 200 fine if missing</t>
+          <t>Swiss vignette check — cameras trigger a CHF 200 fine if missing · verify on windscreen before entering Switzerland</t>
         </is>
       </c>
       <c r="F283" s="19" t="inlineStr">
@@ -6045,55 +6045,51 @@
         </is>
       </c>
     </row>
-    <row r="284" ht="31" customHeight="1">
-      <c r="A284" s="16" t="inlineStr"/>
-      <c r="B284" s="17" t="inlineStr">
+    <row r="284" ht="41" customHeight="1">
+      <c r="A284" s="25" t="inlineStr"/>
+      <c r="B284" s="26" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C284" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D284" s="17" t="inlineStr"/>
-      <c r="E284" s="18" t="inlineStr">
-        <is>
-          <t>8:15am — Park P4, Schwangau — €7 · 10 min walk to ticket centre · go straight to Marienbrücke</t>
-        </is>
-      </c>
-      <c r="F284" s="19" t="inlineStr">
-        <is>
-          <t>€7 / 10 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="285" ht="35" customHeight="1">
-      <c r="A285" s="16" t="inlineStr"/>
-      <c r="B285" s="17" t="inlineStr">
+      <c r="C284" s="27" t="inlineStr">
+        <is>
+          <t>Stay</t>
+        </is>
+      </c>
+      <c r="D284" s="26" t="inlineStr"/>
+      <c r="E284" s="28" t="inlineStr">
+        <is>
+          <t>~10:00am — Airport Hotel Zurich — drop bags at hotel · Lindbergh-Platz 1, 8152 Glattbrugg · check-in may not be ready — leave bags at reception</t>
+        </is>
+      </c>
+      <c r="F284" s="29" t="inlineStr"/>
+    </row>
+    <row r="285" ht="46" customHeight="1">
+      <c r="A285" s="6" t="inlineStr"/>
+      <c r="B285" s="7" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C285" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D285" s="17" t="inlineStr"/>
-      <c r="E285" s="18" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ 8:30am — Marienbrücke (Mary's Bridge) — go here FIRST — 10 min walk above the castle · allow 20–30 min for photos</t>
-        </is>
-      </c>
-      <c r="F285" s="19" t="inlineStr">
-        <is>
-          <t>10 min / 30 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="286" ht="29" customHeight="1">
+      <c r="C285" s="8" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="D285" s="7" t="inlineStr"/>
+      <c r="E285" s="9" t="inlineStr">
+        <is>
+          <t>10:30am — Return Europcar ZRH — 5 min drive from hotel · confirm return closed out correctly · take Hilton shuttle back · keep boarding passes + passports in hand-carry</t>
+        </is>
+      </c>
+      <c r="F285" s="10" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="286" ht="38" customHeight="1">
       <c r="A286" s="16" t="inlineStr"/>
       <c r="B286" s="17" t="inlineStr">
         <is>
@@ -6108,60 +6104,64 @@
       <c r="D286" s="17" t="inlineStr"/>
       <c r="E286" s="18" t="inlineStr">
         <is>
-          <t>⚠️ 9:20am — Castle GATE (not ticket centre) — entry strictly timed · guide will not wait</t>
-        </is>
-      </c>
-      <c r="F286" s="19" t="inlineStr"/>
-    </row>
-    <row r="287" ht="34" customHeight="1">
-      <c r="A287" s="16" t="inlineStr"/>
-      <c r="B287" s="17" t="inlineStr">
+          <t>11:00am — Train to Zurich HB — Zurich Airport → Zurich HB · 10 min · CHF 7 · runs every 10 min from the airport underground station</t>
+        </is>
+      </c>
+      <c r="F286" s="19" t="inlineStr">
+        <is>
+          <t>10 min / CHF 7 / 10 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="287" ht="37" customHeight="1">
+      <c r="A287" s="20" t="inlineStr"/>
+      <c r="B287" s="21" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C287" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D287" s="17" t="inlineStr"/>
-      <c r="E287" s="18" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ 9:30am — Neuschwanstein Castle interior tour — guided tour 35–40 min inside · photography not allowed inside</t>
-        </is>
-      </c>
-      <c r="F287" s="19" t="inlineStr">
-        <is>
-          <t>40 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="288" ht="37" customHeight="1">
-      <c r="A288" s="6" t="inlineStr"/>
-      <c r="B288" s="7" t="inlineStr">
+      <c r="C287" s="22" t="inlineStr">
+        <is>
+          <t>Hike</t>
+        </is>
+      </c>
+      <c r="D287" s="21" t="inlineStr"/>
+      <c r="E287" s="23" t="inlineStr">
+        <is>
+          <t>⭐ 11:15am — Lindenhof viewpoint — hilltop square · best city panorama without climbing · Romans used it as a fort · free · 15 min</t>
+        </is>
+      </c>
+      <c r="F287" s="24" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="288" ht="40" customHeight="1">
+      <c r="A288" s="20" t="inlineStr"/>
+      <c r="B288" s="21" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C288" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D288" s="7" t="inlineStr"/>
-      <c r="E288" s="9" t="inlineStr">
-        <is>
-          <t>11:30am — Depart Neuschwanstein → Wasserauen — 1hr 30min drive · ⚠️ Saturday = absolute peak crowds on all German/Swiss roads</t>
-        </is>
-      </c>
-      <c r="F288" s="10" t="inlineStr">
-        <is>
-          <t>1hr / 30min</t>
-        </is>
-      </c>
-    </row>
-    <row r="289" ht="50" customHeight="1">
+      <c r="C288" s="22" t="inlineStr">
+        <is>
+          <t>Hike</t>
+        </is>
+      </c>
+      <c r="D288" s="21" t="inlineStr"/>
+      <c r="E288" s="23" t="inlineStr">
+        <is>
+          <t>⭐ ⭐ 11:30am — Grossmünster — twin-towered landmark · climb to the top for panorama of city + Lake Zurich · kids love the tower climb · ~CHF 5</t>
+        </is>
+      </c>
+      <c r="F288" s="24" t="inlineStr">
+        <is>
+          <t>CHF 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="289" ht="37" customHeight="1">
       <c r="A289" s="16" t="inlineStr"/>
       <c r="B289" s="17" t="inlineStr">
         <is>
@@ -6176,40 +6176,40 @@
       <c r="D289" s="17" t="inlineStr"/>
       <c r="E289" s="18" t="inlineStr">
         <is>
-          <t>1:15pm — Park at Wasserauen cable car — CHF 36/adult return (2026 rate) · runs every 15 min · ⚠️ Peak Saturday: parking lot likely full — if full: park further down the valley on the roadside · local train/shuttle runs t</t>
+          <t>⭐ 12:15pm — Fraumünster — Marc Chagall stained glass windows — genuinely stunning · unlike anything else on the trip · ~CHF 5</t>
         </is>
       </c>
       <c r="F289" s="19" t="inlineStr">
         <is>
-          <t>CHF 36 / 15 min / 20 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="290" ht="32" customHeight="1">
-      <c r="A290" s="20" t="inlineStr"/>
-      <c r="B290" s="21" t="inlineStr">
+          <t>CHF 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="43" customHeight="1">
+      <c r="A290" s="16" t="inlineStr"/>
+      <c r="B290" s="17" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C290" s="22" t="inlineStr">
-        <is>
-          <t>Hike</t>
-        </is>
-      </c>
-      <c r="D290" s="21" t="inlineStr"/>
-      <c r="E290" s="23" t="inlineStr">
-        <is>
-          <t>⭐ 1:30pm — Ebenalp cable car — CHF 36/adult · 6 min · last descent 6pm · ⚠️ caves 10°C — pack a layer</t>
-        </is>
-      </c>
-      <c r="F290" s="24" t="inlineStr">
-        <is>
-          <t>CHF 36 / 6 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="291" ht="35" customHeight="1">
+      <c r="C290" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D290" s="17" t="inlineStr"/>
+      <c r="E290" s="18" t="inlineStr">
+        <is>
+          <t>1:00pm — Bahnhofstrasse — one of the world's great shopping streets · Confiserie Sprüngli for Swiss chocolate + Luxemburgerli macarons — MUST · 30 min stroll</t>
+        </is>
+      </c>
+      <c r="F290" s="19" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="39" customHeight="1">
       <c r="A291" s="16" t="inlineStr"/>
       <c r="B291" s="17" t="inlineStr">
         <is>
@@ -6224,84 +6224,84 @@
       <c r="D291" s="17" t="inlineStr"/>
       <c r="E291" s="18" t="inlineStr">
         <is>
-          <t>⭐ ⭐ 2:00pm — Berggasthaus Aescher — arrive before 4pm ·  Swing event 5pm · Chäs-Chnöpfli or Rösti · Siedwurst if full</t>
-        </is>
-      </c>
-      <c r="F291" s="19" t="inlineStr"/>
-    </row>
-    <row r="292" ht="39" customHeight="1">
-      <c r="A292" s="6" t="inlineStr"/>
-      <c r="B292" s="7" t="inlineStr">
+          <t>⭐ ⭐ 1:45pm — Lake Zurich waterfront — Bürkliplatz · swans · paddle boats · Alps visible in the background on a clear day · free · 45 min</t>
+        </is>
+      </c>
+      <c r="F291" s="19" t="inlineStr">
+        <is>
+          <t>45 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="292" ht="50" customHeight="1">
+      <c r="A292" s="16" t="inlineStr"/>
+      <c r="B292" s="17" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C292" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D292" s="7" t="inlineStr"/>
-      <c r="E292" s="9" t="inlineStr">
-        <is>
-          <t>4:00pm — Cable car down + drive to ZRH — walk 25 min back up to Ebenalp top station · cable car down · ~2hr drive to Zurich Airport area</t>
-        </is>
-      </c>
-      <c r="F292" s="10" t="inlineStr">
-        <is>
-          <t>25 min / ~2hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="293" ht="33" customHeight="1">
-      <c r="A293" s="16" t="inlineStr"/>
-      <c r="B293" s="17" t="inlineStr">
+      <c r="C292" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D292" s="17" t="inlineStr"/>
+      <c r="E292" s="18" t="inlineStr">
+        <is>
+          <t>⭐ ⭐ 2:30pm — Caliente! Latin Festival — Jul 3–5 2026 · Europe's largest Latin festival · Kasernenareal · South American music + dancing + food stalls · Jul 4 is the final day — biggest atmosphere · family-friendly · free</t>
+        </is>
+      </c>
+      <c r="F292" s="19" t="inlineStr"/>
+    </row>
+    <row r="293" ht="44" customHeight="1">
+      <c r="A293" s="11" t="inlineStr"/>
+      <c r="B293" s="12" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C293" s="16" t="inlineStr">
+      <c r="C293" s="13" t="inlineStr">
+        <is>
+          <t>Eat</t>
+        </is>
+      </c>
+      <c r="D293" s="12" t="inlineStr"/>
+      <c r="E293" s="14" t="inlineStr">
+        <is>
+          <t>4:30pm — Early dinner by Lake Zurich — Zeughauskeller (15th century armory beer hall · hearty Swiss meals) · or lakeside restaurant at Bürkliplatz · allow 1.5hrs</t>
+        </is>
+      </c>
+      <c r="F293" s="15" t="inlineStr">
+        <is>
+          <t>5hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="27" customHeight="1">
+      <c r="A294" s="16" t="inlineStr"/>
+      <c r="B294" s="17" t="inlineStr">
+        <is>
+          <t>Jul 4</t>
+        </is>
+      </c>
+      <c r="C294" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D293" s="17" t="inlineStr"/>
-      <c r="E293" s="18" t="inlineStr">
-        <is>
-          <t>❌ Rhine Falls — SKIP TODAY — adding 45 min detour north on a peak Saturday risks missing car return window</t>
-        </is>
-      </c>
-      <c r="F293" s="19" t="inlineStr">
-        <is>
-          <t>45 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="294" ht="50" customHeight="1">
-      <c r="A294" s="6" t="inlineStr"/>
-      <c r="B294" s="7" t="inlineStr">
-        <is>
-          <t>Jul 4</t>
-        </is>
-      </c>
-      <c r="C294" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D294" s="7" t="inlineStr"/>
-      <c r="E294" s="9" t="inlineStr">
-        <is>
-          <t>Return Europcar ZRH tonight — drop bags at Airport Hotel Zurich · drive 5 min to Europcar ZRH return · return by 11:30pm · Hilton shuttle back · check Booking.com email for return confirmation</t>
-        </is>
-      </c>
-      <c r="F294" s="10" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="295" ht="28" customHeight="1">
+      <c r="D294" s="17" t="inlineStr"/>
+      <c r="E294" s="18" t="inlineStr">
+        <is>
+          <t>6:00pm — Train back to airport — Zurich HB → Zurich Airport · 10 min · CHF 7</t>
+        </is>
+      </c>
+      <c r="F294" s="19" t="inlineStr">
+        <is>
+          <t>10 min / CHF 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="47" customHeight="1">
       <c r="A295" s="25" t="inlineStr"/>
       <c r="B295" s="26" t="inlineStr">
         <is>
@@ -6316,14 +6316,10 @@
       <c r="D295" s="26" t="inlineStr"/>
       <c r="E295" s="28" t="inlineStr">
         <is>
-          <t>⚠️ Tonight — final checks — check-in opens 5:30am · hotel is 5 min walk to terminal</t>
-        </is>
-      </c>
-      <c r="F295" s="29" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
+          <t>6:30pm — Airport Hotel Zurich — pack final bags · passports in hand-carry · boarding passes to phone wallet · confirm 5:30am shuttle at front desk · set two alarms · early bed</t>
+        </is>
+      </c>
+      <c r="F295" s="29" t="inlineStr"/>
     </row>
     <row r="296" ht="31" customHeight="1">
       <c r="A296" s="30" t="inlineStr"/>
@@ -7436,7 +7432,7 @@
       </c>
       <c r="F17" s="46" t="inlineStr">
         <is>
-          <t>~280 km / 174 mi ~3h 30m · Neuschwanstein → Ebenalp → ZRH</t>
+          <t>~185 km / 115 mi ~2h direct to ZRH</t>
         </is>
       </c>
       <c r="G17" s="48" t="inlineStr">
@@ -7519,7 +7515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7702,96 +7698,92 @@
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="68" t="inlineStr">
+      <c r="A9" s="66" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Seceda 360 cable car — Jun 30 · 4 tickets</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Receipt 1161/678/554260 · 2 adults €84.50 + 2 juniors €43.00 · Total €255 · Valid Jun 30, 2026 · Print at home</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>Booked ✅ — print tickets before departure</t>
+        </is>
+      </c>
+      <c r="E9" s="67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="68" t="inlineStr">
         <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="B9" s="69" t="inlineStr">
-        <is>
-          <t>Neuschwanstein Castle tickets — Jul 4 · 9:30am entry slot</t>
-        </is>
-      </c>
-      <c r="C9" s="38" t="inlineStr">
-        <is>
-          <t>€17.50/adult incl. booking fee · tickets.hohenschwangau.de · be at GATE (not ticket centre) by 9:20am</t>
-        </is>
-      </c>
-      <c r="D9" s="38" t="inlineStr">
-        <is>
-          <t>Book NOW — July sells out weeks ahead</t>
-        </is>
-      </c>
-      <c r="E9" s="70" t="inlineStr"/>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="66" t="inlineStr">
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>Austrian digital vignette</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr"/>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>Buy on Jun 22 at asfinag.at after picking up Europcar car · need licence plate · ~€16.50 · 10-day pass</t>
+        </is>
+      </c>
+      <c r="E10" s="70" t="inlineStr"/>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="66" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>Seceda 360 cable car — Jun 30 · 4 tickets</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>Receipt 1161/678/554260 · 2 adults €84.50 + 2 juniors €43.00 · Total €255 · Valid Jun 30, 2026 · Print at home</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>Booked ✅ — print tickets before departure</t>
-        </is>
-      </c>
-      <c r="E10" s="67" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Oeschinensee timed slot — Jun 23 · 8:30am</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Order 254-SK2MH6 · CHF 125 · 08:30–10:00 Jun 23</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr"/>
+      <c r="E11" s="67" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="68" t="inlineStr">
-        <is>
-          <t>Urgent</t>
-        </is>
-      </c>
-      <c r="B11" s="69" t="inlineStr">
-        <is>
-          <t>Austrian digital vignette</t>
-        </is>
-      </c>
-      <c r="C11" s="38" t="inlineStr"/>
-      <c r="D11" s="38" t="inlineStr">
-        <is>
-          <t>Buy on Jun 22 at asfinag.at after picking up Europcar car · need licence plate · ~€16.50 · 10-day pass</t>
-        </is>
-      </c>
-      <c r="E11" s="70" t="inlineStr"/>
-    </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="66" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B12" s="23" t="inlineStr">
-        <is>
-          <t>Oeschinensee timed slot — Jun 23 · 8:30am</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t>Order 254-SK2MH6 · CHF 125 · 08:30–10:00 Jun 23</t>
-        </is>
-      </c>
-      <c r="D12" s="24" t="inlineStr"/>
-      <c r="E12" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="A12" s="71" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="B12" s="72" t="inlineStr">
+        <is>
+          <t>⛵ Königssee electric boat — Jun 25 · 9:15am</t>
+        </is>
+      </c>
+      <c r="C12" s="73" t="inlineStr"/>
+      <c r="D12" s="73" t="inlineStr">
+        <is>
+          <t>Book 1–2 weeks before Jun 25 (non-refundable · pick time you are confident about) · seenschifffahrt.de</t>
+        </is>
+      </c>
+      <c r="E12" s="74" t="inlineStr"/>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="71" t="inlineStr">
@@ -7801,66 +7793,70 @@
       </c>
       <c r="B13" s="72" t="inlineStr">
         <is>
-          <t>⛵ Königssee electric boat — Jun 25 · 9:15am</t>
-        </is>
-      </c>
-      <c r="C13" s="73" t="inlineStr"/>
+          <t>Gosaukammbahn cable car — Jun 27</t>
+        </is>
+      </c>
+      <c r="C13" s="73" t="inlineStr">
+        <is>
+          <t>~€28 return/adult · book at gosaukammbahn.at · afternoon after Krippenstein</t>
+        </is>
+      </c>
       <c r="D13" s="73" t="inlineStr">
         <is>
-          <t>Book 1–2 weeks before Jun 25 (non-refundable · pick time you are confident about) · seenschifffahrt.de</t>
+          <t>Book soon — Jun 27 Saturday peak season</t>
         </is>
       </c>
       <c r="E13" s="74" t="inlineStr"/>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="71" t="inlineStr">
+      <c r="A14" s="66" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>⛏ Hallstatt Salt Mine — CLOSED Jun 27 (renovation)</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>Closed for renovation · reopens Jun 30 · Salzwelten Altaussee is the alternative (25 min away)</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>N/A — closed during our visit</t>
+        </is>
+      </c>
+      <c r="E14" s="67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="71" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="B14" s="72" t="inlineStr">
-        <is>
-          <t>Gosaukammbahn cable car — Jun 27</t>
-        </is>
-      </c>
-      <c r="C14" s="73" t="inlineStr">
-        <is>
-          <t>~€28 return/adult · book at gosaukammbahn.at · afternoon after Krippenstein</t>
-        </is>
-      </c>
-      <c r="D14" s="73" t="inlineStr">
-        <is>
-          <t>Book soon — Jun 27 Saturday peak season</t>
-        </is>
-      </c>
-      <c r="E14" s="74" t="inlineStr"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="66" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B15" s="23" t="inlineStr">
-        <is>
-          <t>⛏ Hallstatt Salt Mine — CLOSED Jun 27 (renovation)</t>
-        </is>
-      </c>
-      <c r="C15" s="24" t="inlineStr">
-        <is>
-          <t>Closed for renovation · reopens Jun 30 · Salzwelten Altaussee is the alternative (25 min away)</t>
-        </is>
-      </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>N/A — closed during our visit</t>
-        </is>
-      </c>
-      <c r="E15" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="B15" s="72" t="inlineStr">
+        <is>
+          <t>Dachstein Krippenstein cable car + 5 Fingers — Jun 27</t>
+        </is>
+      </c>
+      <c r="C15" s="73" t="inlineStr">
+        <is>
+          <t>Book at dachstein.at · Sections 1+2 ~€44.90/adult · 5 Fingers free at top · arrive Obertraun 8:15am</t>
+        </is>
+      </c>
+      <c r="D15" s="73" t="inlineStr">
+        <is>
+          <t>Book before departure</t>
+        </is>
+      </c>
+      <c r="E15" s="74" t="inlineStr"/>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="71" t="inlineStr">
@@ -7870,17 +7866,13 @@
       </c>
       <c r="B16" s="72" t="inlineStr">
         <is>
-          <t>Dachstein Krippenstein cable car + 5 Fingers — Jun 27</t>
-        </is>
-      </c>
-      <c r="C16" s="73" t="inlineStr">
-        <is>
-          <t>Book at dachstein.at · Sections 1+2 ~€44.90/adult · 5 Fingers free at top · arrive Obertraun 8:15am</t>
-        </is>
-      </c>
+          <t>⛴ Achensee steamboat — Jul 2</t>
+        </is>
+      </c>
+      <c r="C16" s="73" t="inlineStr"/>
       <c r="D16" s="73" t="inlineStr">
         <is>
-          <t>Book before departure</t>
+          <t>Day-of or day-before fine · large boats · no timed slots · achensee.com</t>
         </is>
       </c>
       <c r="E16" s="74" t="inlineStr"/>
@@ -7893,13 +7885,17 @@
       </c>
       <c r="B17" s="72" t="inlineStr">
         <is>
-          <t>⛴ Achensee steamboat — Jul 2</t>
-        </is>
-      </c>
-      <c r="C17" s="73" t="inlineStr"/>
+          <t>Eagle's Nest bus — Jun 25 · ~1pm from Obersalzberg</t>
+        </is>
+      </c>
+      <c r="C17" s="73" t="inlineStr">
+        <is>
+          <t>~€32/person (bus + elevator) · buy at Obersalzberg car park · no advance booking · register return bus time immediately at top</t>
+        </is>
+      </c>
       <c r="D17" s="73" t="inlineStr">
         <is>
-          <t>Day-of or day-before fine · large boats · no timed slots · achensee.com</t>
+          <t>Buy on day — no pre-booking needed</t>
         </is>
       </c>
       <c r="E17" s="74" t="inlineStr"/>
@@ -7912,17 +7908,13 @@
       </c>
       <c r="B18" s="72" t="inlineStr">
         <is>
-          <t>Eagle's Nest bus — Jun 25 · ~1pm from Obersalzberg</t>
-        </is>
-      </c>
-      <c r="C18" s="73" t="inlineStr">
-        <is>
-          <t>~€32/person (bus + elevator) · buy at Obersalzberg car park · no advance booking · register return bus time immediately at top</t>
-        </is>
-      </c>
+          <t>Travel insurance × 4</t>
+        </is>
+      </c>
+      <c r="C18" s="73" t="inlineStr"/>
       <c r="D18" s="73" t="inlineStr">
         <is>
-          <t>Buy on day — no pre-booking needed</t>
+          <t>Before departure</t>
         </is>
       </c>
       <c r="E18" s="74" t="inlineStr"/>
@@ -7935,13 +7927,17 @@
       </c>
       <c r="B19" s="72" t="inlineStr">
         <is>
-          <t>Travel insurance × 4</t>
-        </is>
-      </c>
-      <c r="C19" s="73" t="inlineStr"/>
+          <t>️ P2 Compatsch parking — Jul 1 (fully booked · keep checking)</t>
+        </is>
+      </c>
+      <c r="C19" s="73" t="inlineStr">
+        <is>
+          <t>seiseralm.it · €30 · must arrive before 9am · cancellations appear · check daily · Plan B: Seis cable car €30/adult RT</t>
+        </is>
+      </c>
       <c r="D19" s="73" t="inlineStr">
         <is>
-          <t>Before departure</t>
+          <t>Keep checking daily — cancellations appear · Plan B = Seis–Compatsch cable car (no booking needed)</t>
         </is>
       </c>
       <c r="E19" s="74" t="inlineStr"/>
@@ -7954,43 +7950,47 @@
       </c>
       <c r="B20" s="72" t="inlineStr">
         <is>
-          <t>️ P2 Compatsch parking — Jul 1 (fully booked · keep checking)</t>
+          <t>Brenner Pass Digital Flex toll — buy online</t>
         </is>
       </c>
       <c r="C20" s="73" t="inlineStr">
         <is>
-          <t>seiseralm.it · €30 · must arrive before 9am · cancellations appear · check daily · Plan B: Seis cable car €30/adult RT</t>
+          <t>autobrennero.it · cameras read plate · skip queue · needed Jun 30→Jul 1</t>
         </is>
       </c>
       <c r="D20" s="73" t="inlineStr">
         <is>
-          <t>Keep checking daily — cancellations appear · Plan B = Seis–Compatsch cable car (no booking needed)</t>
+          <t>Buy before Jun 30</t>
         </is>
       </c>
       <c r="E20" s="74" t="inlineStr"/>
     </row>
     <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B21" s="72" t="inlineStr">
-        <is>
-          <t>Brenner Pass Digital Flex toll — buy online</t>
-        </is>
-      </c>
-      <c r="C21" s="73" t="inlineStr">
-        <is>
-          <t>autobrennero.it · cameras read plate · skip queue · needed Jun 30→Jul 1</t>
-        </is>
-      </c>
-      <c r="D21" s="73" t="inlineStr">
-        <is>
-          <t>Buy before Jun 30</t>
-        </is>
-      </c>
-      <c r="E21" s="74" t="inlineStr"/>
+      <c r="A21" s="66" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>️ Rifugio Auronzo parking — Jun 29 · Tre Cime</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>Transaction PASS3CIME_26017885 · Ticket P26134547 · €40 · 9:00am–8:59pm Jun 29 · update plate Jun 28 at pass.auronzo.info</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>Booked ✅ · update licence plate night before (Jun 28 in Sillian)</t>
+        </is>
+      </c>
+      <c r="E21" s="67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="66" t="inlineStr">
@@ -8000,47 +8000,20 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>️ Rifugio Auronzo parking — Jun 29 · Tre Cime</t>
+          <t>Siusi Alm e-bikes — Jul 1 · optional</t>
         </is>
       </c>
       <c r="C22" s="24" t="inlineStr">
         <is>
-          <t>Transaction PASS3CIME_26017885 · Ticket P26134547 · €40 · 9:00am–8:59pm Jun 29 · update plate Jun 28 at pass.auronzo.info</t>
+          <t>Removed from itinerary — time constraints on Jul 1</t>
         </is>
       </c>
       <c r="D22" s="24" t="inlineStr">
         <is>
-          <t>Booked ✅ · update licence plate night before (Jun 28 in Sillian)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E22" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="66" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>Siusi Alm e-bikes — Jul 1 · optional</t>
-        </is>
-      </c>
-      <c r="C23" s="24" t="inlineStr">
-        <is>
-          <t>Removed from itinerary — time constraints on Jul 1</t>
-        </is>
-      </c>
-      <c r="D23" s="24" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E23" s="67" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Königssee booked ✅ · OB6A2C80290DB89 · Vorgangs-Nr 95019 · 9:15am Jun 25 · €89.40 · 2 adults + 2 children · arrive dock 8:55am · return flexible
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -2786,7 +2786,7 @@
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>Timeline: 8:15am Königssee park ▸ 8:30am boat to Salet ▸ Obersee + Röthbachfall 9:45am ▸ St. Bartholomä lunch 12pm ▸ 1:30pm Eagle's Nest Kehlsteinbus ▸ 4pm Rossfeld Road ▸ 4:45pm Hintersee/Zauberwald ▸ 6:30pm Berchtesgaden dinner</t>
+          <t>Timeline: 8:55am Königssee dock ▸ 9:15am boat to Salet ▸ Obersee + Röthbachfall + Malerwinkel 10:10am ▸ St. Bartholomä lunch 12pm ▸ 12:45pm boat back ▸ 1:30pm Eagle's Nest (clear) or Salt Mine (cloudy) ▸ 4pm Rossfeld ▸ 4:45pm Hintersee/Zauberwald ▸ 6:30pm Berchtesgaden dinner</t>
         </is>
       </c>
     </row>
@@ -2836,12 +2836,12 @@
       <c r="D105" s="17" t="inlineStr"/>
       <c r="E105" s="18" t="inlineStr">
         <is>
-          <t>⭐ ⭐ 8:30am — Königssee electric boat — completely silent electric boats — only powered vessels allowed on this lake · ⚠️ Go all the way to Salet — 55 min to Salet · ~€28–30 return to Salet per adult</t>
+          <t xml:space="preserve">⭐ ⭐ 9:15am — Königssee electric boat — ✅ Booked · OB6A2C80290DB89 · Fahrt-Nr. 16 · arrive dock by 8:55am (20 min before) · completely silent electric boats — only powered vessels allowed on this lake · 55 min to Salet · </t>
         </is>
       </c>
       <c r="F105" s="19" t="inlineStr">
         <is>
-          <t>55 min / €28</t>
+          <t>20 min / 55 min / €29.80</t>
         </is>
       </c>
     </row>
@@ -7767,23 +7767,31 @@
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B12" s="72" t="inlineStr">
-        <is>
-          <t>⛵ Königssee electric boat — Jun 25 · 9:15am</t>
-        </is>
-      </c>
-      <c r="C12" s="73" t="inlineStr"/>
-      <c r="D12" s="73" t="inlineStr">
-        <is>
-          <t>Book 1–2 weeks before Jun 25 (non-refundable · pick time you are confident about) · seenschifffahrt.de</t>
-        </is>
-      </c>
-      <c r="E12" s="74" t="inlineStr"/>
+      <c r="A12" s="66" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>Königssee electric boat — Jun 25 · 9:15am</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>Booking OB6A2C80290DB89 · Vorgangs-Nr. 95019 · €89.40 · 2 adults + 2 children · Fahrt-Nr. 16 · Seelände → Salet return · 4 individual tickets</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>Booked ✅ · Arrive Seelände dock by 8:55am (20 min before) · Keep return tickets separately</t>
+        </is>
+      </c>
+      <c r="E12" s="67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="71" t="inlineStr">

</xml_diff>

<commit_message>
Checklist reordered: urgent top · done bottom · removed 4 items (Salt Mine closed, Achensee day-of, Eagles Nest day-of, Siusi e-bikes optional) · travel insurance + Brenner + Dachstein + Gosaukammbahn promoted to urgent
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -151,12 +151,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="004A7C2F"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00C0392B"/>
       <sz val="10"/>
     </font>
@@ -169,6 +163,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="0092400E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="004A7C2F"/>
       <sz val="10"/>
     </font>
     <font>
@@ -533,22 +533,16 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -557,7 +551,13 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -572,13 +572,13 @@
     <xf numFmtId="0" fontId="19" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -587,7 +587,7 @@
     <xf numFmtId="0" fontId="9" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -7515,7 +7515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7562,466 +7562,370 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="66" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B3" s="23" t="inlineStr">
-        <is>
-          <t>All accommodation — 10 properties confirmed</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="inlineStr">
-        <is>
-          <t>All 10 nights booked · see Accommodation section below</t>
-        </is>
-      </c>
-      <c r="D3" s="24" t="inlineStr"/>
-      <c r="E3" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>Travel insurance × 4</t>
+        </is>
+      </c>
+      <c r="C3" s="38" t="inlineStr"/>
+      <c r="D3" s="38" t="inlineStr">
+        <is>
+          <t>BOOK TODAY — trip departs Jun 19 · only 7 days away</t>
+        </is>
+      </c>
+      <c r="E3" s="68" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="66" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B4" s="23" t="inlineStr">
-        <is>
-          <t>✈️ Icelandair flights × 4</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
-        <is>
-          <t>Ref A77762 · $4,087.92</t>
-        </is>
-      </c>
-      <c r="D4" s="24" t="inlineStr"/>
-      <c r="E4" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="B4" s="67" t="inlineStr">
+        <is>
+          <t>Dachstein Krippenstein cable car + 5 Fingers — Jun 27</t>
+        </is>
+      </c>
+      <c r="C4" s="38" t="inlineStr">
+        <is>
+          <t>Book at dachstein.at · Sections 1+2 ~€44.90/adult · 5 Fingers free at top · arrive Obertraun 8:15am</t>
+        </is>
+      </c>
+      <c r="D4" s="38" t="inlineStr">
+        <is>
+          <t>Book before departure</t>
+        </is>
+      </c>
+      <c r="E4" s="68" t="inlineStr"/>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="66" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="inlineStr">
-        <is>
-          <t>Europcar ZRH — Volkswagen Tiguan 4x4 · Jun 22–Jul 4</t>
-        </is>
-      </c>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>Booking #738796923 · Booking.com · $746.30 · Pickup 1:30pm · Return 11:30pm Jul 4 · Unlimited mileage</t>
-        </is>
-      </c>
-      <c r="D5" s="24" t="inlineStr"/>
-      <c r="E5" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="B5" s="67" t="inlineStr">
+        <is>
+          <t>Gosaukammbahn cable car — Jun 27</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>~€28 return/adult · book at gosaukammbahn.at · afternoon after Krippenstein</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>Book soon — Jun 27 Saturday peak season</t>
+        </is>
+      </c>
+      <c r="E5" s="68" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="66" t="inlineStr">
         <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B6" s="23" t="inlineStr">
-        <is>
-          <t>Budget car — Keflavik KEF · Jun 20–22</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>Conf. #42334482US1 · $289 · pay at pickup</t>
-        </is>
-      </c>
-      <c r="D6" s="24" t="inlineStr"/>
-      <c r="E6" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="B6" s="67" t="inlineStr">
+        <is>
+          <t>Brenner Pass Digital Flex toll — buy online</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>autobrennero.it · cameras read plate · skip queue · needed Jun 30→Jul 1</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>Buy before Jun 30 (Day 12) · autobrennero.it · €11.50</t>
+        </is>
+      </c>
+      <c r="E6" s="68" t="inlineStr"/>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="66" t="inlineStr">
         <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="B7" s="67" t="inlineStr">
+        <is>
+          <t>Austrian digital vignette</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="inlineStr"/>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>Buy on Jun 22 at asfinag.at after picking up Europcar car · need licence plate · ~€16.50 · 10-day pass</t>
+        </is>
+      </c>
+      <c r="E7" s="68" t="inlineStr"/>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="69" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="B8" s="70" t="inlineStr">
+        <is>
+          <t>️ P2 Compatsch parking — Jul 1 (fully booked · keep checking)</t>
+        </is>
+      </c>
+      <c r="C8" s="71" t="inlineStr">
+        <is>
+          <t>seiseralm.it · €30 · must arrive before 9am · cancellations appear · check daily · Plan B: Seis cable car €30/adult RT</t>
+        </is>
+      </c>
+      <c r="D8" s="71" t="inlineStr">
+        <is>
+          <t>Keep checking daily — cancellations appear · Plan B = Seis–Compatsch cable car (no booking needed)</t>
+        </is>
+      </c>
+      <c r="E8" s="72" t="inlineStr"/>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="73" t="inlineStr">
+        <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>All accommodation — 10 properties confirmed</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>All 10 nights booked · see Accommodation section below</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr"/>
+      <c r="E9" s="74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>✈️ Icelandair flights × 4</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Ref A77762 · $4,087.92</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr"/>
+      <c r="E10" s="74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="73" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Europcar ZRH — Volkswagen Tiguan 4x4 · Jun 22–Jul 4</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Booking #738796923 · Booking.com · $746.30 · Pickup 1:30pm · Return 11:30pm Jul 4 · Unlimited mileage</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr"/>
+      <c r="E11" s="74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="73" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>Budget car — Keflavik KEF · Jun 20–22</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>Conf. #42334482US1 · $289 · pay at pickup</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr"/>
+      <c r="E12" s="74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="73" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Grindelwald First gondola — Jun 23</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Booking #238070</t>
         </is>
       </c>
-      <c r="D7" s="24" t="inlineStr"/>
-      <c r="E7" s="67" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr"/>
+      <c r="E13" s="74" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="66" t="inlineStr">
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="73" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>Check 4 passports (valid Oct 2026+)</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr"/>
-      <c r="E8" s="67" t="inlineStr">
+      <c r="D14" s="24" t="inlineStr"/>
+      <c r="E14" s="74" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="66" t="inlineStr">
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="73" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>Seceda 360 cable car — Jun 30 · 4 tickets</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C15" s="24" t="inlineStr">
         <is>
           <t>Receipt 1161/678/554260 · 2 adults €84.50 + 2 juniors €43.00 · Total €255 · Valid Jun 30, 2026 · Print at home</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>Booked ✅ — print tickets before departure</t>
         </is>
       </c>
-      <c r="E9" s="67" t="inlineStr">
+      <c r="E15" s="74" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="68" t="inlineStr">
-        <is>
-          <t>Urgent</t>
-        </is>
-      </c>
-      <c r="B10" s="69" t="inlineStr">
-        <is>
-          <t>Austrian digital vignette</t>
-        </is>
-      </c>
-      <c r="C10" s="38" t="inlineStr"/>
-      <c r="D10" s="38" t="inlineStr">
-        <is>
-          <t>Buy on Jun 22 at asfinag.at after picking up Europcar car · need licence plate · ~€16.50 · 10-day pass</t>
-        </is>
-      </c>
-      <c r="E10" s="70" t="inlineStr"/>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="66" t="inlineStr">
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="73" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>Oeschinensee timed slot — Jun 23 · 8:30am</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C16" s="24" t="inlineStr">
         <is>
           <t>Order 254-SK2MH6 · CHF 125 · 08:30–10:00 Jun 23</t>
         </is>
       </c>
-      <c r="D11" s="24" t="inlineStr"/>
-      <c r="E11" s="67" t="inlineStr">
+      <c r="D16" s="24" t="inlineStr"/>
+      <c r="E16" s="74" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="66" t="inlineStr">
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="73" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>Königssee electric boat — Jun 25 · 9:15am</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
         <is>
           <t>Booking OB6A2C80290DB89 · Vorgangs-Nr. 95019 · €89.40 · 2 adults + 2 children · Fahrt-Nr. 16 · Seelände → Salet return · 4 individual tickets</t>
         </is>
       </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>Booked ✅ · Arrive Seelände dock by 8:55am (20 min before) · Keep return tickets separately</t>
         </is>
       </c>
-      <c r="E12" s="67" t="inlineStr">
+      <c r="E17" s="74" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B13" s="72" t="inlineStr">
-        <is>
-          <t>Gosaukammbahn cable car — Jun 27</t>
-        </is>
-      </c>
-      <c r="C13" s="73" t="inlineStr">
-        <is>
-          <t>~€28 return/adult · book at gosaukammbahn.at · afternoon after Krippenstein</t>
-        </is>
-      </c>
-      <c r="D13" s="73" t="inlineStr">
-        <is>
-          <t>Book soon — Jun 27 Saturday peak season</t>
-        </is>
-      </c>
-      <c r="E13" s="74" t="inlineStr"/>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="66" t="inlineStr">
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="73" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
-        <is>
-          <t>⛏ Hallstatt Salt Mine — CLOSED Jun 27 (renovation)</t>
-        </is>
-      </c>
-      <c r="C14" s="24" t="inlineStr">
-        <is>
-          <t>Closed for renovation · reopens Jun 30 · Salzwelten Altaussee is the alternative (25 min away)</t>
-        </is>
-      </c>
-      <c r="D14" s="24" t="inlineStr">
-        <is>
-          <t>N/A — closed during our visit</t>
-        </is>
-      </c>
-      <c r="E14" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B15" s="72" t="inlineStr">
-        <is>
-          <t>Dachstein Krippenstein cable car + 5 Fingers — Jun 27</t>
-        </is>
-      </c>
-      <c r="C15" s="73" t="inlineStr">
-        <is>
-          <t>Book at dachstein.at · Sections 1+2 ~€44.90/adult · 5 Fingers free at top · arrive Obertraun 8:15am</t>
-        </is>
-      </c>
-      <c r="D15" s="73" t="inlineStr">
-        <is>
-          <t>Book before departure</t>
-        </is>
-      </c>
-      <c r="E15" s="74" t="inlineStr"/>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B16" s="72" t="inlineStr">
-        <is>
-          <t>⛴ Achensee steamboat — Jul 2</t>
-        </is>
-      </c>
-      <c r="C16" s="73" t="inlineStr"/>
-      <c r="D16" s="73" t="inlineStr">
-        <is>
-          <t>Day-of or day-before fine · large boats · no timed slots · achensee.com</t>
-        </is>
-      </c>
-      <c r="E16" s="74" t="inlineStr"/>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B17" s="72" t="inlineStr">
-        <is>
-          <t>Eagle's Nest bus — Jun 25 · ~1pm from Obersalzberg</t>
-        </is>
-      </c>
-      <c r="C17" s="73" t="inlineStr">
-        <is>
-          <t>~€32/person (bus + elevator) · buy at Obersalzberg car park · no advance booking · register return bus time immediately at top</t>
-        </is>
-      </c>
-      <c r="D17" s="73" t="inlineStr">
-        <is>
-          <t>Buy on day — no pre-booking needed</t>
-        </is>
-      </c>
-      <c r="E17" s="74" t="inlineStr"/>
-    </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B18" s="72" t="inlineStr">
-        <is>
-          <t>Travel insurance × 4</t>
-        </is>
-      </c>
-      <c r="C18" s="73" t="inlineStr"/>
-      <c r="D18" s="73" t="inlineStr">
-        <is>
-          <t>Before departure</t>
-        </is>
-      </c>
-      <c r="E18" s="74" t="inlineStr"/>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B19" s="72" t="inlineStr">
-        <is>
-          <t>️ P2 Compatsch parking — Jul 1 (fully booked · keep checking)</t>
-        </is>
-      </c>
-      <c r="C19" s="73" t="inlineStr">
-        <is>
-          <t>seiseralm.it · €30 · must arrive before 9am · cancellations appear · check daily · Plan B: Seis cable car €30/adult RT</t>
-        </is>
-      </c>
-      <c r="D19" s="73" t="inlineStr">
-        <is>
-          <t>Keep checking daily — cancellations appear · Plan B = Seis–Compatsch cable car (no booking needed)</t>
-        </is>
-      </c>
-      <c r="E19" s="74" t="inlineStr"/>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="71" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B20" s="72" t="inlineStr">
-        <is>
-          <t>Brenner Pass Digital Flex toll — buy online</t>
-        </is>
-      </c>
-      <c r="C20" s="73" t="inlineStr">
-        <is>
-          <t>autobrennero.it · cameras read plate · skip queue · needed Jun 30→Jul 1</t>
-        </is>
-      </c>
-      <c r="D20" s="73" t="inlineStr">
-        <is>
-          <t>Buy before Jun 30</t>
-        </is>
-      </c>
-      <c r="E20" s="74" t="inlineStr"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="66" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>️ Rifugio Auronzo parking — Jun 29 · Tre Cime</t>
         </is>
       </c>
-      <c r="C21" s="24" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>Transaction PASS3CIME_26017885 · Ticket P26134547 · €40 · 9:00am–8:59pm Jun 29 · update plate Jun 28 at pass.auronzo.info</t>
         </is>
       </c>
-      <c r="D21" s="24" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>Booked ✅ · update licence plate night before (Jun 28 in Sillian)</t>
         </is>
       </c>
-      <c r="E21" s="67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="66" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>Siusi Alm e-bikes — Jul 1 · optional</t>
-        </is>
-      </c>
-      <c r="C22" s="24" t="inlineStr">
-        <is>
-          <t>Removed from itinerary — time constraints on Jul 1</t>
-        </is>
-      </c>
-      <c r="D22" s="24" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E22" s="67" t="inlineStr">
+      <c r="E18" s="74" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Kaiserblick Goisern: platform corrected to Booking.com (not Airbnb) · cost updated to ~60 · check-in 14:00-20:00 · check-out 08:00-10:00 · key box with code at entrance
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -8100,7 +8100,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="75" t="inlineStr">
         <is>
-          <t>7–8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B7" s="76" t="inlineStr">
@@ -8120,7 +8120,7 @@
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>+43 xxx · Airbnb message host · key box on arrival</t>
+          <t>Key box with code at apartment entrance · schedule time with host via Booking.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 Compatsch: booking system not open yet · opens end of June 2026 · check seiseralm.it from Jun 25 · book immediately when live · within 6-day window from Collalbo · Plan B Seis cable car
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -7674,17 +7674,17 @@
       </c>
       <c r="B8" s="70" t="inlineStr">
         <is>
-          <t>️ P2 Compatsch parking — Jul 1 (fully booked · keep checking)</t>
+          <t>P2 Compatsch parking — Jul 1</t>
         </is>
       </c>
       <c r="C8" s="71" t="inlineStr">
         <is>
-          <t>seiseralm.it · €30 · must arrive before 9am · cancellations appear · check daily · Plan B: Seis cable car €30/adult RT</t>
+          <t>seiseralm.it · €30/day · must arrive before 9am · QR code scan at barrier above Hotel Zorzi · booking system opens end of June 2026</t>
         </is>
       </c>
       <c r="D8" s="71" t="inlineStr">
         <is>
-          <t>Keep checking daily — cancellations appear · Plan B = Seis–Compatsch cable car (no booking needed)</t>
+          <t>Booking NOT open yet — system opens ~Jun 25 · check seiseralm.it daily from Jun 25 · book immediately when live · within 6-day window from Collalbo · Plan B: Seis cable car (no booking needed)</t>
         </is>
       </c>
       <c r="E8" s="72" t="inlineStr"/>

</xml_diff>

<commit_message>
Day 7: Salzachöfen Gorge added · Day 7 map link updated (Berchtesgaden→Liechtensteinklamm→Gschwandtanger→Salzachöfen→St.Gilgen→Hallstatt→Bad Goisern) · timeline + glance updated · Excel regenerated
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -970,7 +970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F319"/>
+  <dimension ref="A1:F320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3195,14 +3195,14 @@
     <row r="124" ht="15" customHeight="1">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>Timeline: 8:15am depart Berchtesgaden ▸ 9:00am Liechtensteinklamm ▸ 11am drive Salzburg ▸ 12pm P+R South + Altstadt ▸ Hohensalzburg Panorama Tour ▸ 3pm drive Wolfgangsee ▸ 4pm St. Gilgen→St. Wolfgang ferry ▸ 5:30pm Hallstatt golden hour ▸ 7:30pm Kaiserblick Goisern</t>
+          <t>Timeline: 8:15am Berchtesgaden ▸ 9:00am Liechtensteinklamm ▸ 10:30am Gschwandtanger meadow ▸ 10:45am Salzachöfen Gorge ▸ 12:15pm drive ▸ 1:15pm St. Gilgen lunch ▸ 2:15pm Hallstatt ▸ 6:00pm Bad Goisern</t>
         </is>
       </c>
     </row>
     <row r="125" ht="22" customHeight="1">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>Key: ✅ Liechtensteinklamm 9:00am sharp — be first at the gate · €16/adult · wear sturdy shoes  |  ✅ Salzburg: P+R South (Alpenstraße) €15 family combo — do NOT park in city centre · 2026 restricted zone  |  ⚠️ Hallstatt tunnel signs: if "Full" — go straight to Goisern · park Obertraun + ferry instead</t>
+          <t>Key: ✅ Salzachöfen Gorge after Gschwandtanger — €5/adult · 1.5hrs · free parking · no booking needed  |  ✅ Liechtensteinklamm 9:00am sharp — be first at the gate · €16/adult · wear sturdy shoes  |  ⚠️ Hallstatt tunnel signs: if "Full" — go straight to Goisern · park Obertraun + ferry instead</t>
         </is>
       </c>
     </row>
@@ -3275,50 +3275,54 @@
       </c>
     </row>
     <row r="129" ht="50" customHeight="1">
-      <c r="A129" s="6" t="inlineStr"/>
-      <c r="B129" s="7" t="inlineStr">
+      <c r="A129" s="16" t="inlineStr"/>
+      <c r="B129" s="17" t="inlineStr">
         <is>
           <t>Jun 26</t>
         </is>
       </c>
-      <c r="C129" s="8" t="inlineStr">
+      <c r="C129" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D129" s="17" t="inlineStr"/>
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>⭐ ⭐ Salzachöfen Gorge — Paß-Lueg-Straße 82, Golling · 5 min away · €5/adult · €3/child · free parking · 90m deep gorge · narrow cathedral cave section · different experience to Liechtensteinklamm · allow 1.5hrs</t>
+        </is>
+      </c>
+      <c r="F129" s="19" t="inlineStr">
+        <is>
+          <t>5 min / €5 / €3</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="50" customHeight="1">
+      <c r="A130" s="6" t="inlineStr"/>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D129" s="7" t="inlineStr"/>
-      <c r="E129" s="9" t="inlineStr">
+      <c r="D130" s="7" t="inlineStr"/>
+      <c r="E130" s="9" t="inlineStr">
         <is>
           <t>11:00am — Drive north to Salzburg — ~1hr on A10 · arrive ~12:00pm · ⚠️ Do NOT park in the city centre — 2026 restricted traffic zone + construction everywhere · use P+R South (Alpenstraße) — €15 combo-ticket covers parki</t>
         </is>
       </c>
-      <c r="F129" s="10" t="inlineStr">
+      <c r="F130" s="10" t="inlineStr">
         <is>
           <t>~1hr / €15</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="18" customHeight="1">
-      <c r="A130" s="16" t="inlineStr"/>
-      <c r="B130" s="17" t="inlineStr">
-        <is>
-          <t>Jun 26</t>
-        </is>
-      </c>
-      <c r="C130" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D130" s="17" t="inlineStr"/>
-      <c r="E130" s="18" t="inlineStr">
-        <is>
-          <t>⭐ 12:00pm — Salzburg old town</t>
-        </is>
-      </c>
-      <c r="F130" s="19" t="inlineStr"/>
-    </row>
-    <row r="131" ht="38" customHeight="1">
+    <row r="131" ht="18" customHeight="1">
       <c r="A131" s="16" t="inlineStr"/>
       <c r="B131" s="17" t="inlineStr">
         <is>
@@ -3333,64 +3337,60 @@
       <c r="D131" s="17" t="inlineStr"/>
       <c r="E131" s="18" t="inlineStr">
         <is>
+          <t>⭐ 12:00pm — Salzburg old town</t>
+        </is>
+      </c>
+      <c r="F131" s="19" t="inlineStr"/>
+    </row>
+    <row r="132" ht="38" customHeight="1">
+      <c r="A132" s="16" t="inlineStr"/>
+      <c r="B132" s="17" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="C132" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D132" s="17" t="inlineStr"/>
+      <c r="E132" s="18" t="inlineStr">
+        <is>
           <t>⭐ 12:30pm — Hohensalzburg Fortress — funicular up from Kapitelplatz · stick to the Panorama Tour — ➕ Interior: €16/adult · allow 1hr</t>
         </is>
       </c>
-      <c r="F131" s="19" t="inlineStr">
+      <c r="F132" s="19" t="inlineStr">
         <is>
           <t>€16 / 1hr</t>
         </is>
       </c>
     </row>
-    <row r="132" ht="34" customHeight="1">
-      <c r="A132" s="6" t="inlineStr"/>
-      <c r="B132" s="7" t="inlineStr">
+    <row r="133" ht="34" customHeight="1">
+      <c r="A133" s="6" t="inlineStr"/>
+      <c r="B133" s="7" t="inlineStr">
         <is>
           <t>Jun 26</t>
         </is>
       </c>
-      <c r="C132" s="8" t="inlineStr">
+      <c r="C133" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D132" s="7" t="inlineStr"/>
-      <c r="E132" s="9" t="inlineStr">
+      <c r="D133" s="7" t="inlineStr"/>
+      <c r="E133" s="9" t="inlineStr">
         <is>
           <t>3:00pm — Drive east to Wolfgangsee — 45 min to St. Gilgen · arrive ~3:45pm · park in St. Gilgen village car park</t>
         </is>
       </c>
-      <c r="F132" s="10" t="inlineStr">
+      <c r="F133" s="10" t="inlineStr">
         <is>
           <t>45 min</t>
         </is>
       </c>
     </row>
-    <row r="133" ht="39" customHeight="1">
-      <c r="A133" s="16" t="inlineStr"/>
-      <c r="B133" s="17" t="inlineStr">
-        <is>
-          <t>Jun 26</t>
-        </is>
-      </c>
-      <c r="C133" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D133" s="17" t="inlineStr"/>
-      <c r="E133" s="18" t="inlineStr">
-        <is>
-          <t>⭐ 4:00pm — Wolfgangsee ferry: St. Gilgen → St. Wolfgang → back — take the ferry to St. Wolfgang (~20 min) · most relaxing 90 min of the day</t>
-        </is>
-      </c>
-      <c r="F133" s="19" t="inlineStr">
-        <is>
-          <t>~20 min / 90 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="22" customHeight="1">
+    <row r="134" ht="39" customHeight="1">
       <c r="A134" s="16" t="inlineStr"/>
       <c r="B134" s="17" t="inlineStr">
         <is>
@@ -3405,16 +3405,16 @@
       <c r="D134" s="17" t="inlineStr"/>
       <c r="E134" s="18" t="inlineStr">
         <is>
-          <t>⭐ ⭐ 5:30pm — Hallstatt golden hour — allow 1.5–2hrs</t>
+          <t>⭐ 4:00pm — Wolfgangsee ferry: St. Gilgen → St. Wolfgang → back — take the ferry to St. Wolfgang (~20 min) · most relaxing 90 min of the day</t>
         </is>
       </c>
       <c r="F134" s="19" t="inlineStr">
         <is>
-          <t>2hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="38" customHeight="1">
+          <t>~20 min / 90 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="22" customHeight="1">
       <c r="A135" s="16" t="inlineStr"/>
       <c r="B135" s="17" t="inlineStr">
         <is>
@@ -3429,49 +3429,60 @@
       <c r="D135" s="17" t="inlineStr"/>
       <c r="E135" s="18" t="inlineStr">
         <is>
+          <t>⭐ ⭐ 5:30pm — Hallstatt golden hour — allow 1.5–2hrs</t>
+        </is>
+      </c>
+      <c r="F135" s="19" t="inlineStr">
+        <is>
+          <t>2hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="38" customHeight="1">
+      <c r="A136" s="16" t="inlineStr"/>
+      <c r="B136" s="17" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="C136" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D136" s="17" t="inlineStr"/>
+      <c r="E136" s="18" t="inlineStr">
+        <is>
           <t>⚠️ Hallstatt 2026 camera parking system — alternative: park at Obertraun (5 min drive) + take the ferry to Hallstatt (€4 · 10 min)</t>
         </is>
       </c>
-      <c r="F135" s="19" t="inlineStr">
+      <c r="F136" s="19" t="inlineStr">
         <is>
           <t>5 min / €4 / 10 min</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="28" customHeight="1">
-      <c r="A136" s="6" t="inlineStr"/>
-      <c r="B136" s="7" t="inlineStr">
+    <row r="137" ht="28" customHeight="1">
+      <c r="A137" s="6" t="inlineStr"/>
+      <c r="B137" s="7" t="inlineStr">
         <is>
           <t>Jun 26</t>
         </is>
       </c>
-      <c r="C136" s="8" t="inlineStr">
+      <c r="C137" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D136" s="7" t="inlineStr"/>
-      <c r="E136" s="9" t="inlineStr">
+      <c r="D137" s="7" t="inlineStr"/>
+      <c r="E137" s="9" t="inlineStr">
         <is>
           <t>7:30pm — Kaiserblick Goisern, Bad Goisern — 15 min drive from Hallstatt · $333</t>
         </is>
       </c>
-      <c r="F136" s="10" t="inlineStr">
+      <c r="F137" s="10" t="inlineStr">
         <is>
           <t>15 min / $333</t>
-        </is>
-      </c>
-    </row>
-    <row r="137" ht="34" customHeight="1">
-      <c r="A137" s="30" t="inlineStr"/>
-      <c r="B137" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C137" s="32" t="inlineStr">
-        <is>
-          <t>⚠️ Salzburg parking 2026 — Old Town becoming restricted traffic zone · construction barriers everywhere · use P+R South (Alpenstraße) · €15 combo = parking + shuttle bus for whole family · much faster than city garage hunting</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3495,7 @@
       </c>
       <c r="C138" s="32" t="inlineStr">
         <is>
-          <t>⚠️ Hallstatt 2026 camera system — electronic signs at tunnel entrance · if "Full": do not enter · drive straight to Kaiserblick Goisern · return via ferry from Obertraun (€4 · 10 min) or bus on Day 8</t>
+          <t>⚠️ Salzburg parking 2026 — Old Town becoming restricted traffic zone · construction barriers everywhere · use P+R South (Alpenstraße) · €15 combo = parking + shuttle bus for whole family · much faster than city garage hunting</t>
         </is>
       </c>
     </row>
@@ -3497,112 +3508,101 @@
       </c>
       <c r="C139" s="32" t="inlineStr">
         <is>
+          <t>⚠️ Hallstatt 2026 camera system — electronic signs at tunnel entrance · if "Full": do not enter · drive straight to Kaiserblick Goisern · return via ferry from Obertraun (€4 · 10 min) or bus on Day 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="34" customHeight="1">
+      <c r="A140" s="30" t="inlineStr"/>
+      <c r="B140" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C140" s="32" t="inlineStr">
+        <is>
           <t>☕ Hohensalzburg tip — stick to Panorama Tour only (courtyards + bastions) · skip the individual museums to stay on schedule · the view is the reason to go up · allow 1hr max</t>
         </is>
       </c>
     </row>
-    <row r="140" ht="3" customHeight="1">
-      <c r="A140" s="33" t="n"/>
-      <c r="B140" s="33" t="n"/>
-      <c r="C140" s="33" t="n"/>
-      <c r="D140" s="33" t="n"/>
-      <c r="E140" s="33" t="n"/>
-      <c r="F140" s="33" t="n"/>
-    </row>
-    <row r="141" ht="20" customHeight="1">
-      <c r="A141" s="3" t="inlineStr">
+    <row r="141" ht="3" customHeight="1">
+      <c r="A141" s="33" t="n"/>
+      <c r="B141" s="33" t="n"/>
+      <c r="C141" s="33" t="n"/>
+      <c r="D141" s="33" t="n"/>
+      <c r="E141" s="33" t="n"/>
+      <c r="F141" s="33" t="n"/>
+    </row>
+    <row r="142" ht="20" customHeight="1">
+      <c r="A142" s="3" t="inlineStr">
         <is>
           <t>DAY 8  |  Jun 27  |  Dachstein Krippenstein · Gosausee · Hallstatt Evening — The High-Alpine Day  |  ~40 km / 25 mi  ~1h total · very local day</t>
         </is>
       </c>
     </row>
-    <row r="142" ht="15" customHeight="1">
-      <c r="A142" s="4" t="inlineStr">
+    <row r="143" ht="15" customHeight="1">
+      <c r="A143" s="4" t="inlineStr">
         <is>
           <t>Timeline: 8:15am depart Bad Goisern ▸ 8:45am Krippenstein cable car ▸ 9:30am 5 Fingers viewpoint ▸ Ice Cave optional ▸ 1:30pm Gosausee Mirror Lake ▸ 2:00pm Gosaukammbahn ▸ 4:30pm Hallstatt golden hour + dinner ▸ Beinhaus ▸ ~7pm Kaiserblick Goisern</t>
         </is>
       </c>
     </row>
-    <row r="143" ht="22" customHeight="1">
-      <c r="A143" s="5" t="inlineStr">
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="5" t="inlineStr">
         <is>
           <t>Key: Salt Mine + Skywalk CLOSED Jun 27 — reopens Jun 30 · do not book these  |  ✅ Dachstein Krippenstein 8:45am → 5 Fingers → Gosausee 1:30pm → Gosaukammbahn → Hallstatt 4:30pm  |  ⚠️ Saturday = busy Hallstatt · check digital signs · if Full → park Obertraun + NAVIA ferry €4</t>
         </is>
       </c>
     </row>
-    <row r="144" ht="50" customHeight="1">
-      <c r="A144" s="34" t="inlineStr"/>
-      <c r="B144" s="35" t="inlineStr">
+    <row r="145" ht="50" customHeight="1">
+      <c r="A145" s="34" t="inlineStr"/>
+      <c r="B145" s="35" t="inlineStr">
         <is>
           <t>Jun 27</t>
         </is>
       </c>
-      <c r="C144" s="36" t="inlineStr">
+      <c r="C145" s="36" t="inlineStr">
         <is>
           <t>Alert</t>
         </is>
       </c>
-      <c r="D144" s="35" t="inlineStr"/>
-      <c r="E144" s="37" t="inlineStr">
+      <c r="D145" s="35" t="inlineStr"/>
+      <c r="E145" s="37" t="inlineStr">
         <is>
           <t>2026 Alert: Hallstatt Salt Mine + Skywalk CLOSED Jun 27 — major renovation underway · scheduled to reopen June 30, 2026 · do not attempt to book these for today · alternative: Salzwelten Altaussee — (25 min from Bad Gois</t>
         </is>
       </c>
-      <c r="F144" s="38" t="inlineStr">
+      <c r="F145" s="38" t="inlineStr">
         <is>
           <t>25 min</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="41" customHeight="1">
-      <c r="A145" s="6" t="inlineStr"/>
-      <c r="B145" s="7" t="inlineStr">
+    <row r="146" ht="41" customHeight="1">
+      <c r="A146" s="6" t="inlineStr"/>
+      <c r="B146" s="7" t="inlineStr">
         <is>
           <t>Jun 27</t>
         </is>
       </c>
-      <c r="C145" s="8" t="inlineStr">
+      <c r="C146" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D145" s="7" t="inlineStr"/>
-      <c r="E145" s="9" t="inlineStr">
+      <c r="D146" s="7" t="inlineStr"/>
+      <c r="E146" s="9" t="inlineStr">
         <is>
           <t>⏰ 8:15am — Depart Bad Goisern — 20 min drive to Obertraun · arrive by 8:40am · park at the Dachstein Krippenstein cable car base station in Obertraun</t>
         </is>
       </c>
-      <c r="F145" s="10" t="inlineStr">
+      <c r="F146" s="10" t="inlineStr">
         <is>
           <t>20 min</t>
         </is>
       </c>
     </row>
-    <row r="146" ht="30" customHeight="1">
-      <c r="A146" s="16" t="inlineStr"/>
-      <c r="B146" s="17" t="inlineStr">
-        <is>
-          <t>Jun 27</t>
-        </is>
-      </c>
-      <c r="C146" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D146" s="17" t="inlineStr"/>
-      <c r="E146" s="18" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ 8:45am — Dachstein Krippenstein cable car — Sections 1 + 2 up to 2,109m · €44.90/adult</t>
-        </is>
-      </c>
-      <c r="F146" s="19" t="inlineStr">
-        <is>
-          <t>€44.90</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="32" customHeight="1">
+    <row r="147" ht="30" customHeight="1">
       <c r="A147" s="16" t="inlineStr"/>
       <c r="B147" s="17" t="inlineStr">
         <is>
@@ -3617,12 +3617,12 @@
       <c r="D147" s="17" t="inlineStr"/>
       <c r="E147" s="18" t="inlineStr">
         <is>
-          <t>⭐ ⭐ 9:30am — 5 Fingers Viewpoint — 20 min walk from the Section 2 top station · allow 45 min at the top</t>
+          <t>⭐ ⭐ 8:45am — Dachstein Krippenstein cable car — Sections 1 + 2 up to 2,109m · €44.90/adult</t>
         </is>
       </c>
       <c r="F147" s="19" t="inlineStr">
         <is>
-          <t>20 min / 45 min</t>
+          <t>€44.90</t>
         </is>
       </c>
     </row>
@@ -3641,64 +3641,64 @@
       <c r="D148" s="17" t="inlineStr"/>
       <c r="E148" s="18" t="inlineStr">
         <is>
+          <t>⭐ ⭐ 9:30am — 5 Fingers Viewpoint — 20 min walk from the Section 2 top station · allow 45 min at the top</t>
+        </is>
+      </c>
+      <c r="F148" s="19" t="inlineStr">
+        <is>
+          <t>20 min / 45 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="32" customHeight="1">
+      <c r="A149" s="16" t="inlineStr"/>
+      <c r="B149" s="17" t="inlineStr">
+        <is>
+          <t>Jun 27</t>
+        </is>
+      </c>
+      <c r="C149" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D149" s="17" t="inlineStr"/>
+      <c r="E149" s="18" t="inlineStr">
+        <is>
           <t>➕ Optional: Giant Ice Cave (Section 1) — accessible from Section 1 midstation · extra cost ~€10/adult</t>
         </is>
       </c>
-      <c r="F148" s="19" t="inlineStr">
+      <c r="F149" s="19" t="inlineStr">
         <is>
           <t>€10</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="30" customHeight="1">
-      <c r="A149" s="6" t="inlineStr"/>
-      <c r="B149" s="7" t="inlineStr">
+    <row r="150" ht="30" customHeight="1">
+      <c r="A150" s="6" t="inlineStr"/>
+      <c r="B150" s="7" t="inlineStr">
         <is>
           <t>Jun 27</t>
         </is>
       </c>
-      <c r="C149" s="8" t="inlineStr">
+      <c r="C150" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D149" s="7" t="inlineStr"/>
-      <c r="E149" s="9" t="inlineStr">
+      <c r="D150" s="7" t="inlineStr"/>
+      <c r="E150" s="9" t="inlineStr">
         <is>
           <t>⭐ ⭐ 1:30pm — Vorderer Gosausee — the Mirror Lake — 25 min drive from Obertraun · allow 30 min</t>
         </is>
       </c>
-      <c r="F149" s="10" t="inlineStr">
+      <c r="F150" s="10" t="inlineStr">
         <is>
           <t>25 min / 30 min</t>
         </is>
       </c>
     </row>
-    <row r="150" ht="33" customHeight="1">
-      <c r="A150" s="16" t="inlineStr"/>
-      <c r="B150" s="17" t="inlineStr">
-        <is>
-          <t>Jun 27</t>
-        </is>
-      </c>
-      <c r="C150" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D150" s="17" t="inlineStr"/>
-      <c r="E150" s="18" t="inlineStr">
-        <is>
-          <t>⭐ 2:00pm — Gosaukammbahn cable car — ~€28 return/adult · panoramic view of the Dachstein glacier from above</t>
-        </is>
-      </c>
-      <c r="F150" s="19" t="inlineStr">
-        <is>
-          <t>€28</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="31" customHeight="1">
+    <row r="151" ht="33" customHeight="1">
       <c r="A151" s="16" t="inlineStr"/>
       <c r="B151" s="17" t="inlineStr">
         <is>
@@ -3713,16 +3713,16 @@
       <c r="D151" s="17" t="inlineStr"/>
       <c r="E151" s="18" t="inlineStr">
         <is>
-          <t>⭐ ⭐ 4:30pm — Hallstatt village evening — mine renovation crowds have gone by now · allow 1.5hrs</t>
+          <t>⭐ 2:00pm — Gosaukammbahn cable car — ~€28 return/adult · panoramic view of the Dachstein glacier from above</t>
         </is>
       </c>
       <c r="F151" s="19" t="inlineStr">
         <is>
-          <t>5hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="38" customHeight="1">
+          <t>€28</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="31" customHeight="1">
       <c r="A152" s="16" t="inlineStr"/>
       <c r="B152" s="17" t="inlineStr">
         <is>
@@ -3737,16 +3737,16 @@
       <c r="D152" s="17" t="inlineStr"/>
       <c r="E152" s="18" t="inlineStr">
         <is>
-          <t>⚠️ Saturday parking warning — if P1/P2 show "Full": park in Obertraun (5 min drive) + take the ferry across · NAVIA ferry: €4 cash</t>
+          <t>⭐ ⭐ 4:30pm — Hallstatt village evening — mine renovation crowds have gone by now · allow 1.5hrs</t>
         </is>
       </c>
       <c r="F152" s="19" t="inlineStr">
         <is>
-          <t>5 min / €4</t>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="21" customHeight="1">
+          <t>5hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="38" customHeight="1">
       <c r="A153" s="16" t="inlineStr"/>
       <c r="B153" s="17" t="inlineStr">
         <is>
@@ -3761,49 +3761,60 @@
       <c r="D153" s="17" t="inlineStr"/>
       <c r="E153" s="18" t="inlineStr">
         <is>
+          <t>⚠️ Saturday parking warning — if P1/P2 show "Full": park in Obertraun (5 min drive) + take the ferry across · NAVIA ferry: €4 cash</t>
+        </is>
+      </c>
+      <c r="F153" s="19" t="inlineStr">
+        <is>
+          <t>5 min / €4</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="21" customHeight="1">
+      <c r="A154" s="16" t="inlineStr"/>
+      <c r="B154" s="17" t="inlineStr">
+        <is>
+          <t>Jun 27</t>
+        </is>
+      </c>
+      <c r="C154" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D154" s="17" t="inlineStr"/>
+      <c r="E154" s="18" t="inlineStr">
+        <is>
           <t>⭐ Beinhaus (Bone Chapel) — €1.50/adult · 10 min</t>
         </is>
       </c>
-      <c r="F153" s="19" t="inlineStr">
+      <c r="F154" s="19" t="inlineStr">
         <is>
           <t>€1.50 / 10 min</t>
         </is>
       </c>
     </row>
-    <row r="154" ht="37" customHeight="1">
-      <c r="A154" s="6" t="inlineStr"/>
-      <c r="B154" s="7" t="inlineStr">
+    <row r="155" ht="37" customHeight="1">
+      <c r="A155" s="6" t="inlineStr"/>
+      <c r="B155" s="7" t="inlineStr">
         <is>
           <t>Jun 27</t>
         </is>
       </c>
-      <c r="C154" s="8" t="inlineStr">
+      <c r="C155" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D154" s="7" t="inlineStr"/>
-      <c r="E154" s="9" t="inlineStr">
+      <c r="D155" s="7" t="inlineStr"/>
+      <c r="E155" s="9" t="inlineStr">
         <is>
           <t>Night 2 — Kaiserblick Goisern — ✅ Already checked in ·  38 Unterjoch, 4822 Bad Goisern, Austria · 15 min drive from Hallstatt</t>
         </is>
       </c>
-      <c r="F154" s="10" t="inlineStr">
+      <c r="F155" s="10" t="inlineStr">
         <is>
           <t>15 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="34" customHeight="1">
-      <c r="A155" s="30" t="inlineStr"/>
-      <c r="B155" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C155" s="32" t="inlineStr">
-        <is>
-          <t>Salt Mine + Skywalk CLOSED Jun 27 — major renovation · reopens Jun 30, 2026 · alternative: Salzwelten Altaussee (25 min from Bad Goisern) · active mine · most authentic</t>
         </is>
       </c>
     </row>
@@ -3816,11 +3827,11 @@
       </c>
       <c r="C156" s="32" t="inlineStr">
         <is>
-          <t>⚠️ 5 Fingers vs Skywalk — 5 Fingers on Krippenstein is higher, more dramatic, free with cable car ticket · direct aerial view down into Hallstatt village · Skywalk is closed anyway — 5 Fingers is the better experience</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="33" customHeight="1">
+          <t>Salt Mine + Skywalk CLOSED Jun 27 — major renovation · reopens Jun 30, 2026 · alternative: Salzwelten Altaussee (25 min from Bad Goisern) · active mine · most authentic</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="34" customHeight="1">
       <c r="A157" s="30" t="inlineStr"/>
       <c r="B157" s="31" t="inlineStr">
         <is>
@@ -3829,11 +3840,11 @@
       </c>
       <c r="C157" s="32" t="inlineStr">
         <is>
-          <t>Gosausee afternoon tip — best photos happen when the sun hits the Dachstein glacier face-on in the afternoon · go at 3pm not morning for the mirror reflection shot</t>
-        </is>
-      </c>
-    </row>
-    <row r="158" ht="34" customHeight="1">
+          <t>⚠️ 5 Fingers vs Skywalk — 5 Fingers on Krippenstein is higher, more dramatic, free with cable car ticket · direct aerial view down into Hallstatt village · Skywalk is closed anyway — 5 Fingers is the better experience</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="33" customHeight="1">
       <c r="A158" s="30" t="inlineStr"/>
       <c r="B158" s="31" t="inlineStr">
         <is>
@@ -3842,7 +3853,7 @@
       </c>
       <c r="C158" s="32" t="inlineStr">
         <is>
-          <t>Hofer (Aldi) Bad Goisern — stock up this morning or evening · discount prices · buy for Jun 27–Jul 1: Grossglockner · Sillian · Dolomites 3 nights · Hofrat-Renner-Weg 1 · open Tue 7:15am</t>
+          <t>Gosausee afternoon tip — best photos happen when the sun hits the Dachstein glacier face-on in the afternoon · go at 3pm not morning for the mirror reflection shot</t>
         </is>
       </c>
     </row>
@@ -3855,88 +3866,77 @@
       </c>
       <c r="C159" s="32" t="inlineStr">
         <is>
+          <t>Hofer (Aldi) Bad Goisern — stock up this morning or evening · discount prices · buy for Jun 27–Jul 1: Grossglockner · Sillian · Dolomites 3 nights · Hofrat-Renner-Weg 1 · open Tue 7:15am</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="34" customHeight="1">
+      <c r="A160" s="30" t="inlineStr"/>
+      <c r="B160" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C160" s="32" t="inlineStr">
+        <is>
           <t>Löckenmoos alpine lake — Bad Goisern — minutes from Kaiserblick hotel · almost no international tourists · small alpine bog lake with mountain reflections · ☀️ clear weather only — magical when calm · perfect 20 min evening walk from the ho</t>
         </is>
       </c>
     </row>
-    <row r="160" ht="3" customHeight="1">
-      <c r="A160" s="33" t="n"/>
-      <c r="B160" s="33" t="n"/>
-      <c r="C160" s="33" t="n"/>
-      <c r="D160" s="33" t="n"/>
-      <c r="E160" s="33" t="n"/>
-      <c r="F160" s="33" t="n"/>
-    </row>
-    <row r="161" ht="20" customHeight="1">
-      <c r="A161" s="3" t="inlineStr">
+    <row r="161" ht="3" customHeight="1">
+      <c r="A161" s="33" t="n"/>
+      <c r="B161" s="33" t="n"/>
+      <c r="C161" s="33" t="n"/>
+      <c r="D161" s="33" t="n"/>
+      <c r="E161" s="33" t="n"/>
+      <c r="F161" s="33" t="n"/>
+    </row>
+    <row r="162" ht="20" customHeight="1">
+      <c r="A162" s="3" t="inlineStr">
         <is>
           <t>DAY 9  |  Jun 28  |  The Roof of Austria — Grossglockner High Alpine Road → Sillian  |  ~280 km / 174 mi  ~4h 30m incl. Grossglockner slow drive</t>
         </is>
       </c>
     </row>
-    <row r="162" ht="15" customHeight="1">
-      <c r="A162" s="4" t="inlineStr">
+    <row r="163" ht="15" customHeight="1">
+      <c r="A163" s="4" t="inlineStr">
         <is>
           <t>Timeline: 8:00am checkout ▸ 9:30am Ferleiten toll €46.50 ▸ 10:15am Edelweiß-Spitze ▸ 11:30am Hochtor tunnel ▸ 12:15pm KFJ-Höhe + marmots ▸ 1:30pm glacier lunch ▸ 3:30pm Heiligenblut church photo ▸ 5:30pm Sillian ▸ alarm 5am</t>
         </is>
       </c>
     </row>
-    <row r="163" ht="22" customHeight="1">
-      <c r="A163" s="5" t="inlineStr">
+    <row r="164" ht="22" customHeight="1">
+      <c r="A164" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ Edelweiß-Spitze FIRST — go before motorcycles arrive · dead-end road congests by afternoon  |  ✅ Gamsgrubenweg 10 min from KFJ-Höhe — best marmot spotting on the road · kids will love it  |  ⚠️ Descent: engine brake in low gear · do NOT ride the brakes · they will overheat</t>
         </is>
       </c>
     </row>
-    <row r="164" ht="43" customHeight="1">
-      <c r="A164" s="6" t="inlineStr"/>
-      <c r="B164" s="7" t="inlineStr">
+    <row r="165" ht="43" customHeight="1">
+      <c r="A165" s="6" t="inlineStr"/>
+      <c r="B165" s="7" t="inlineStr">
         <is>
           <t>Jun 28</t>
         </is>
       </c>
-      <c r="C164" s="8" t="inlineStr">
+      <c r="C165" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D164" s="7" t="inlineStr"/>
-      <c r="E164" s="9" t="inlineStr">
+      <c r="D165" s="7" t="inlineStr"/>
+      <c r="E165" s="9" t="inlineStr">
         <is>
           <t>⏰ 8:00am — Checkout Kaiserblick Goisern — 1.5hr drive to the Ferleiten toll gate via the B311 · download offline maps for the Dolomites tonight if not done yet</t>
         </is>
       </c>
-      <c r="F164" s="10" t="inlineStr">
+      <c r="F165" s="10" t="inlineStr">
         <is>
           <t>5hr</t>
         </is>
       </c>
     </row>
-    <row r="165" ht="46" customHeight="1">
-      <c r="A165" s="16" t="inlineStr"/>
-      <c r="B165" s="17" t="inlineStr">
-        <is>
-          <t>Jun 28</t>
-        </is>
-      </c>
-      <c r="C165" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D165" s="17" t="inlineStr"/>
-      <c r="E165" s="18" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ Grossglockner High Alpine Road — 48km of switchbacks across the highest surfaced alpine pass in Austria · road open from 5:30am — last entry 45 min before 9pm closing</t>
-        </is>
-      </c>
-      <c r="F165" s="19" t="inlineStr">
-        <is>
-          <t>48km / 45 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="166" ht="38" customHeight="1">
+    <row r="166" ht="46" customHeight="1">
       <c r="A166" s="16" t="inlineStr"/>
       <c r="B166" s="17" t="inlineStr">
         <is>
@@ -3951,60 +3951,64 @@
       <c r="D166" s="17" t="inlineStr"/>
       <c r="E166" s="18" t="inlineStr">
         <is>
+          <t>⭐ ⭐ Grossglockner High Alpine Road — 48km of switchbacks across the highest surfaced alpine pass in Austria · road open from 5:30am — last entry 45 min before 9pm closing</t>
+        </is>
+      </c>
+      <c r="F166" s="19" t="inlineStr">
+        <is>
+          <t>48km / 45 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="38" customHeight="1">
+      <c r="A167" s="16" t="inlineStr"/>
+      <c r="B167" s="17" t="inlineStr">
+        <is>
+          <t>Jun 28</t>
+        </is>
+      </c>
+      <c r="C167" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D167" s="17" t="inlineStr"/>
+      <c r="E167" s="18" t="inlineStr">
+        <is>
           <t>9:30am — Ferleiten Toll Gate — 2026 rate: €46.50/car — first stop: Edelweiß-Spitze — go there FIRST before the motorcycles arrive</t>
         </is>
       </c>
-      <c r="F166" s="19" t="inlineStr">
+      <c r="F167" s="19" t="inlineStr">
         <is>
           <t>€46.50</t>
         </is>
       </c>
     </row>
-    <row r="167" ht="34" customHeight="1">
-      <c r="A167" s="20" t="inlineStr"/>
-      <c r="B167" s="21" t="inlineStr">
+    <row r="168" ht="34" customHeight="1">
+      <c r="A168" s="20" t="inlineStr"/>
+      <c r="B168" s="21" t="inlineStr">
         <is>
           <t>Jun 28</t>
         </is>
       </c>
-      <c r="C167" s="22" t="inlineStr">
+      <c r="C168" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D167" s="21" t="inlineStr"/>
-      <c r="E167" s="23" t="inlineStr">
+      <c r="D168" s="21" t="inlineStr"/>
+      <c r="E168" s="23" t="inlineStr">
         <is>
           <t>Haus Alpine Naturschau — natural history museum — 15 min · great context for the kids before reaching the summit</t>
         </is>
       </c>
-      <c r="F167" s="24" t="inlineStr">
+      <c r="F168" s="24" t="inlineStr">
         <is>
           <t>15 min</t>
         </is>
       </c>
     </row>
-    <row r="168" ht="32" customHeight="1">
-      <c r="A168" s="16" t="inlineStr"/>
-      <c r="B168" s="17" t="inlineStr">
-        <is>
-          <t>Jun 28</t>
-        </is>
-      </c>
-      <c r="C168" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D168" s="17" t="inlineStr"/>
-      <c r="E168" s="18" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ 10:15am — Edelweiß-Spitze (2,571m) — MUST STOP · dead-end cobblestone branch road — go here FIRST</t>
-        </is>
-      </c>
-      <c r="F168" s="19" t="inlineStr"/>
-    </row>
-    <row r="169" ht="21" customHeight="1">
+    <row r="169" ht="32" customHeight="1">
       <c r="A169" s="16" t="inlineStr"/>
       <c r="B169" s="17" t="inlineStr">
         <is>
@@ -4019,132 +4023,128 @@
       <c r="D169" s="17" t="inlineStr"/>
       <c r="E169" s="18" t="inlineStr">
         <is>
+          <t>⭐ ⭐ 10:15am — Edelweiß-Spitze (2,571m) — MUST STOP · dead-end cobblestone branch road — go here FIRST</t>
+        </is>
+      </c>
+      <c r="F169" s="19" t="inlineStr"/>
+    </row>
+    <row r="170" ht="21" customHeight="1">
+      <c r="A170" s="16" t="inlineStr"/>
+      <c r="B170" s="17" t="inlineStr">
+        <is>
+          <t>Jun 28</t>
+        </is>
+      </c>
+      <c r="C170" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D170" s="17" t="inlineStr"/>
+      <c r="E170" s="18" t="inlineStr">
+        <is>
           <t>11:30am — Hochtor Tunnel (2,504m) — 10 min stop</t>
         </is>
       </c>
-      <c r="F169" s="19" t="inlineStr">
+      <c r="F170" s="19" t="inlineStr">
         <is>
           <t>10 min</t>
         </is>
       </c>
     </row>
-    <row r="170" ht="50" customHeight="1">
-      <c r="A170" s="20" t="inlineStr"/>
-      <c r="B170" s="21" t="inlineStr">
+    <row r="171" ht="50" customHeight="1">
+      <c r="A171" s="20" t="inlineStr"/>
+      <c r="B171" s="21" t="inlineStr">
         <is>
           <t>Jun 28</t>
         </is>
       </c>
-      <c r="C170" s="22" t="inlineStr">
+      <c r="C171" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D170" s="21" t="inlineStr"/>
-      <c r="E170" s="23" t="inlineStr">
+      <c r="D171" s="21" t="inlineStr"/>
+      <c r="E171" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">⭐ ⭐ 12:15pm — Kaiser-Franz-Josefs-Höhe (2,369m) — Austria's longest glacier (8km) stretching toward the Grossglockner · ⚠️ 2026: glacier has receded significantly — to touch the ice take the Gletscherbahn funicular down </t>
         </is>
       </c>
-      <c r="F170" s="24" t="inlineStr">
+      <c r="F171" s="24" t="inlineStr">
         <is>
           <t>8km / 45 min</t>
         </is>
       </c>
     </row>
-    <row r="171" ht="36" customHeight="1">
-      <c r="A171" s="16" t="inlineStr"/>
-      <c r="B171" s="17" t="inlineStr">
+    <row r="172" ht="36" customHeight="1">
+      <c r="A172" s="16" t="inlineStr"/>
+      <c r="B172" s="17" t="inlineStr">
         <is>
           <t>Jun 28</t>
         </is>
       </c>
-      <c r="C171" s="16" t="inlineStr">
+      <c r="C172" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D171" s="17" t="inlineStr"/>
-      <c r="E171" s="18" t="inlineStr">
+      <c r="D172" s="17" t="inlineStr"/>
+      <c r="E172" s="18" t="inlineStr">
         <is>
           <t>Marmot &amp; ibex spotting — Gamsgrubenweg — from Kaiser-Franz-Josefs-Höhe: follow the Gamsgrubenweg tunnel path for 10 min</t>
         </is>
       </c>
-      <c r="F171" s="19" t="inlineStr">
+      <c r="F172" s="19" t="inlineStr">
         <is>
           <t>10 min</t>
         </is>
       </c>
     </row>
-    <row r="172" ht="31" customHeight="1">
-      <c r="A172" s="11" t="inlineStr"/>
-      <c r="B172" s="12" t="inlineStr">
+    <row r="173" ht="31" customHeight="1">
+      <c r="A173" s="11" t="inlineStr"/>
+      <c r="B173" s="12" t="inlineStr">
         <is>
           <t>Jun 28</t>
         </is>
       </c>
-      <c r="C172" s="13" t="inlineStr">
+      <c r="C173" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D172" s="12" t="inlineStr"/>
-      <c r="E172" s="14" t="inlineStr">
+      <c r="D173" s="12" t="inlineStr"/>
+      <c r="E173" s="14" t="inlineStr">
         <is>
           <t>1:30pm — Lunch at Kaiser-Franz-Josefs-Höhe — panoramic terrace facing the glacier · allow 1hr</t>
         </is>
       </c>
-      <c r="F172" s="15" t="inlineStr">
+      <c r="F173" s="15" t="inlineStr">
         <is>
           <t>1hr</t>
         </is>
       </c>
     </row>
-    <row r="173" ht="21" customHeight="1">
-      <c r="A173" s="20" t="inlineStr"/>
-      <c r="B173" s="21" t="inlineStr">
+    <row r="174" ht="21" customHeight="1">
+      <c r="A174" s="20" t="inlineStr"/>
+      <c r="B174" s="21" t="inlineStr">
         <is>
           <t>Jun 28</t>
         </is>
       </c>
-      <c r="C173" s="22" t="inlineStr">
+      <c r="C174" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D173" s="21" t="inlineStr"/>
-      <c r="E173" s="23" t="inlineStr">
+      <c r="D174" s="21" t="inlineStr"/>
+      <c r="E174" s="23" t="inlineStr">
         <is>
           <t>⚠️ Descent toward Heiligenblut — brake warning</t>
         </is>
       </c>
-      <c r="F173" s="24" t="inlineStr"/>
-    </row>
-    <row r="174" ht="21" customHeight="1">
-      <c r="A174" s="16" t="inlineStr"/>
-      <c r="B174" s="17" t="inlineStr">
-        <is>
-          <t>Jun 28</t>
-        </is>
-      </c>
-      <c r="C174" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D174" s="17" t="inlineStr"/>
-      <c r="E174" s="18" t="inlineStr">
-        <is>
-          <t>⭐ 3:30pm — Heiligenblut village — allow 30 min</t>
-        </is>
-      </c>
-      <c r="F174" s="19" t="inlineStr">
-        <is>
-          <t>30 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="175" ht="50" customHeight="1">
+      <c r="F174" s="24" t="inlineStr"/>
+    </row>
+    <row r="175" ht="21" customHeight="1">
       <c r="A175" s="16" t="inlineStr"/>
       <c r="B175" s="17" t="inlineStr">
         <is>
@@ -4159,71 +4159,82 @@
       <c r="D175" s="17" t="inlineStr"/>
       <c r="E175" s="18" t="inlineStr">
         <is>
+          <t>⭐ 3:30pm — Heiligenblut village — allow 30 min</t>
+        </is>
+      </c>
+      <c r="F175" s="19" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="50" customHeight="1">
+      <c r="A176" s="16" t="inlineStr"/>
+      <c r="B176" s="17" t="inlineStr">
+        <is>
+          <t>Jun 28</t>
+        </is>
+      </c>
+      <c r="C176" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D176" s="17" t="inlineStr"/>
+      <c r="E176" s="18" t="inlineStr">
+        <is>
           <t>Gößnitzfall waterfall — Heiligenblut — right outside the village · easy 20 min walk through shaded forest to dramatic wooden viewing platform · thunderous alpine waterfall · stroller-friendly · free · perfect for shaking</t>
         </is>
       </c>
-      <c r="F175" s="19" t="inlineStr">
+      <c r="F176" s="19" t="inlineStr">
         <is>
           <t>20 min</t>
         </is>
       </c>
     </row>
-    <row r="176" ht="23" customHeight="1">
-      <c r="A176" s="25" t="inlineStr"/>
-      <c r="B176" s="26" t="inlineStr">
+    <row r="177" ht="23" customHeight="1">
+      <c r="A177" s="25" t="inlineStr"/>
+      <c r="B177" s="26" t="inlineStr">
         <is>
           <t>Jun 28</t>
         </is>
       </c>
-      <c r="C176" s="27" t="inlineStr">
+      <c r="C177" s="27" t="inlineStr">
         <is>
           <t>Stay</t>
         </is>
       </c>
-      <c r="D176" s="26" t="inlineStr"/>
-      <c r="E176" s="28" t="inlineStr">
+      <c r="D177" s="26" t="inlineStr"/>
+      <c r="E177" s="28" t="inlineStr">
         <is>
           <t>5:30pm — Hotel Schwarzer Adler, Sillian — $115 / €99.40</t>
         </is>
       </c>
-      <c r="F176" s="29" t="inlineStr">
+      <c r="F177" s="29" t="inlineStr">
         <is>
           <t>$115 / €99.40</t>
         </is>
       </c>
     </row>
-    <row r="177" ht="40" customHeight="1">
-      <c r="A177" s="11" t="inlineStr"/>
-      <c r="B177" s="12" t="inlineStr">
+    <row r="178" ht="40" customHeight="1">
+      <c r="A178" s="11" t="inlineStr"/>
+      <c r="B178" s="12" t="inlineStr">
         <is>
           <t>Jun 28</t>
         </is>
       </c>
-      <c r="C177" s="13" t="inlineStr">
+      <c r="C178" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D177" s="12" t="inlineStr"/>
-      <c r="E177" s="14" t="inlineStr">
+      <c r="D178" s="12" t="inlineStr"/>
+      <c r="E178" s="14" t="inlineStr">
         <is>
           <t>Dinner in Sillian —  Download offline Dolomites maps tonight (Maps.me or Google Maps) · check Rifugio Auronzo parking booking confirmation</t>
         </is>
       </c>
-      <c r="F177" s="15" t="inlineStr"/>
-    </row>
-    <row r="178" ht="34" customHeight="1">
-      <c r="A178" s="30" t="inlineStr"/>
-      <c r="B178" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C178" s="32" t="inlineStr">
-        <is>
-          <t>Grossglockner toll 2026: €46.50/car — buy Day Ticket online at grossglockner.at to skip queue · road open 5:30am–9pm · last entry 45 min before closing · check road status for snow/closures before departing</t>
-        </is>
-      </c>
+      <c r="F178" s="15" t="inlineStr"/>
     </row>
     <row r="179" ht="34" customHeight="1">
       <c r="A179" s="30" t="inlineStr"/>
@@ -4234,11 +4245,11 @@
       </c>
       <c r="C179" s="32" t="inlineStr">
         <is>
-          <t>⚠️ Pasterze Glacier 2026 — glacier has receded significantly · to touch the ice: Gletscherbahn funicular down + 30–45 min hike · terrace view is still spectacular without going down</t>
-        </is>
-      </c>
-    </row>
-    <row r="180" ht="33" customHeight="1">
+          <t>Grossglockner toll 2026: €46.50/car — buy Day Ticket online at grossglockner.at to skip queue · road open 5:30am–9pm · last entry 45 min before closing · check road status for snow/closures before departing</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="34" customHeight="1">
       <c r="A180" s="30" t="inlineStr"/>
       <c r="B180" s="31" t="inlineStr">
         <is>
@@ -4247,11 +4258,11 @@
       </c>
       <c r="C180" s="32" t="inlineStr">
         <is>
-          <t>⚠️ Brake warning on descent — Heiligenblut descent is steep and long · use 2nd/3rd gear engine braking · continuous brake use = overheating + brake fade = dangerous</t>
-        </is>
-      </c>
-    </row>
-    <row r="181" ht="34" customHeight="1">
+          <t>⚠️ Pasterze Glacier 2026 — glacier has receded significantly · to touch the ice: Gletscherbahn funicular down + 30–45 min hike · terrace view is still spectacular without going down</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="33" customHeight="1">
       <c r="A181" s="30" t="inlineStr"/>
       <c r="B181" s="31" t="inlineStr">
         <is>
@@ -4260,7 +4271,7 @@
       </c>
       <c r="C181" s="32" t="inlineStr">
         <is>
-          <t>Heiligenblut church photo — upper car park near the cemetery · Grossglockner peak frames behind the church spire · 4pm light is ideal · one of the most iconic shots in Austria</t>
+          <t>⚠️ Brake warning on descent — Heiligenblut descent is steep and long · use 2nd/3rd gear engine braking · continuous brake use = overheating + brake fade = dangerous</t>
         </is>
       </c>
     </row>
@@ -4273,112 +4284,101 @@
       </c>
       <c r="C182" s="32" t="inlineStr">
         <is>
+          <t>Heiligenblut church photo — upper car park near the cemetery · Grossglockner peak frames behind the church spire · 4pm light is ideal · one of the most iconic shots in Austria</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="34" customHeight="1">
+      <c r="A183" s="30" t="inlineStr"/>
+      <c r="B183" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C183" s="32" t="inlineStr">
+        <is>
           <t>Tonight: prep for Dolomites — download offline maps (Google Maps or Maps.me) for the Dolomites · confirm Rifugio Auronzo parking booking · 5am alarm tomorrow · Braies gate opens 7:30am</t>
         </is>
       </c>
     </row>
-    <row r="183" ht="3" customHeight="1">
-      <c r="A183" s="33" t="n"/>
-      <c r="B183" s="33" t="n"/>
-      <c r="C183" s="33" t="n"/>
-      <c r="D183" s="33" t="n"/>
-      <c r="E183" s="33" t="n"/>
-      <c r="F183" s="33" t="n"/>
-    </row>
-    <row r="184" ht="20" customHeight="1">
-      <c r="A184" s="3" t="inlineStr">
+    <row r="184" ht="3" customHeight="1">
+      <c r="A184" s="33" t="n"/>
+      <c r="B184" s="33" t="n"/>
+      <c r="C184" s="33" t="n"/>
+      <c r="D184" s="33" t="n"/>
+      <c r="E184" s="33" t="n"/>
+      <c r="F184" s="33" t="n"/>
+    </row>
+    <row r="185" ht="20" customHeight="1">
+      <c r="A185" s="3" t="inlineStr">
         <is>
           <t>DAY 10  |  Jun 29  |  The Iconic Dolomites — Braies Sunrise · Tre Cime · Prato Piazza · Gardena  |  ~200 km / 124 mi  ~5h total driving · many short hops</t>
         </is>
       </c>
     </row>
-    <row r="185" ht="15" customHeight="1">
-      <c r="A185" s="4" t="inlineStr">
+    <row r="186" ht="15" customHeight="1">
+      <c r="A186" s="4" t="inlineStr">
         <is>
           <t>Timeline: 8am Sillian ▸ 8:45am Braies P3 ▸ 10:15am depart ▸ Misurina coffee ▸ 11:15am Auronzo gate ▸ 11:45am Cadini Trail 117 ▸ 1:30pm lunch ▸ 2:30pm Tre Cime walk ▸ 3:45pm Gardena Pass ▸ 5pm Collalbo</t>
         </is>
       </c>
     </row>
-    <row r="186" ht="22" customHeight="1">
-      <c r="A186" s="5" t="inlineStr">
+    <row r="187" ht="22" customHeight="1">
+      <c r="A187" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ 8am departure — relaxed start · Braies 8:45am · still beautiful · P3 no reservation  |  ❌ Prato Piazza dropped — already have Alpe di Siusi Day 12 · same alpine meadow experience  |  ✅ Auronzo gate 11:15am — well within 9am–8:59pm slot · plate auto-read · no queue  |  ⚠️ Cadini final 50m narrow ridge — secondary viewpoint 20m back is 95% as good  |  ⚠️ Update Auronzo licence plate Jun 28 evening at pass.auronzo.info before Sillian dinner</t>
         </is>
       </c>
     </row>
-    <row r="187" ht="48" customHeight="1">
-      <c r="A187" s="6" t="inlineStr"/>
-      <c r="B187" s="7" t="inlineStr">
+    <row r="188" ht="48" customHeight="1">
+      <c r="A188" s="6" t="inlineStr"/>
+      <c r="B188" s="7" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C187" s="8" t="inlineStr">
+      <c r="C188" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D187" s="7" t="inlineStr"/>
-      <c r="E187" s="9" t="inlineStr">
+      <c r="D188" s="7" t="inlineStr"/>
+      <c r="E188" s="9" t="inlineStr">
         <is>
           <t>8:00am — Depart Sillian — 45 min straight across the Italian border · download offline Dolomites maps tonight if not done · update Auronzo plate at pass.auronzo.info tonight (Jun 28)</t>
         </is>
       </c>
-      <c r="F187" s="10" t="inlineStr">
+      <c r="F188" s="10" t="inlineStr">
         <is>
           <t>45 min</t>
         </is>
       </c>
     </row>
-    <row r="188" ht="49" customHeight="1">
-      <c r="A188" s="16" t="inlineStr"/>
-      <c r="B188" s="17" t="inlineStr">
+    <row r="189" ht="49" customHeight="1">
+      <c r="A189" s="16" t="inlineStr"/>
+      <c r="B189" s="17" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C188" s="16" t="inlineStr">
+      <c r="C189" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D188" s="17" t="inlineStr"/>
-      <c r="E188" s="18" t="inlineStr">
+      <c r="D189" s="17" t="inlineStr"/>
+      <c r="E189" s="18" t="inlineStr">
         <is>
           <t>⭐ ⭐ 8:45am — Lago di Braies — park P3 ~€12 · no reservation needed · walk the best half of the lakeside circuit · famous stilt boathouse · morning views · allow 1.5hrs · leave by 10:15am</t>
         </is>
       </c>
-      <c r="F188" s="19" t="inlineStr">
+      <c r="F189" s="19" t="inlineStr">
         <is>
           <t>€12 / 5hr</t>
         </is>
       </c>
     </row>
-    <row r="189" ht="44" customHeight="1">
-      <c r="A189" s="6" t="inlineStr"/>
-      <c r="B189" s="7" t="inlineStr">
-        <is>
-          <t>Jun 29</t>
-        </is>
-      </c>
-      <c r="C189" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D189" s="7" t="inlineStr"/>
-      <c r="E189" s="9" t="inlineStr">
-        <is>
-          <t>☕ 10:15am — Drive via Lago di Misurina — 1hr drive down the valley · stop at Rifugio Misurina café · 15 min coffee + mirror-reflection photo of Tre Cime in the lake</t>
-        </is>
-      </c>
-      <c r="F189" s="10" t="inlineStr">
-        <is>
-          <t>1hr / 15 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="190" ht="45" customHeight="1">
+    <row r="190" ht="44" customHeight="1">
       <c r="A190" s="6" t="inlineStr"/>
       <c r="B190" s="7" t="inlineStr">
         <is>
@@ -4393,64 +4393,64 @@
       <c r="D190" s="7" t="inlineStr"/>
       <c r="E190" s="9" t="inlineStr">
         <is>
+          <t>☕ 10:15am — Drive via Lago di Misurina — 1hr drive down the valley · stop at Rifugio Misurina café · 15 min coffee + mirror-reflection photo of Tre Cime in the lake</t>
+        </is>
+      </c>
+      <c r="F190" s="10" t="inlineStr">
+        <is>
+          <t>1hr / 15 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="45" customHeight="1">
+      <c r="A191" s="6" t="inlineStr"/>
+      <c r="B191" s="7" t="inlineStr">
+        <is>
+          <t>Jun 29</t>
+        </is>
+      </c>
+      <c r="C191" s="8" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="D191" s="7" t="inlineStr"/>
+      <c r="E191" s="9" t="inlineStr">
+        <is>
           <t>⚠️ 11:15am — Auronzo gate — ✅ Pre-booked · PASS3CIME_26017885 · Ticket P26134547 · 9am–8:59pm slot · plate reads automatically · drive straight up · €40 paid · no queue</t>
         </is>
       </c>
-      <c r="F190" s="10" t="inlineStr">
+      <c r="F191" s="10" t="inlineStr">
         <is>
           <t>€40</t>
         </is>
       </c>
     </row>
-    <row r="191" ht="50" customHeight="1">
-      <c r="A191" s="20" t="inlineStr"/>
-      <c r="B191" s="21" t="inlineStr">
+    <row r="192" ht="50" customHeight="1">
+      <c r="A192" s="20" t="inlineStr"/>
+      <c r="B192" s="21" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C191" s="22" t="inlineStr">
+      <c r="C192" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D191" s="21" t="inlineStr"/>
-      <c r="E191" s="23" t="inlineStr">
+      <c r="D192" s="21" t="inlineStr"/>
+      <c r="E192" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">⭐ ⭐ 11:45am — Cadini di Misurina Trail 117 — hike out to the iconic jagged peak viewpoint · 45 min RT at normal pace · ⚠️ final 50m is a narrow ridge · secondary viewpoint 20m back is 95% as good · allow 1hr 45min total </t>
         </is>
       </c>
-      <c r="F191" s="24" t="inlineStr">
+      <c r="F192" s="24" t="inlineStr">
         <is>
           <t>45 min / 1hr / 45min</t>
         </is>
       </c>
     </row>
-    <row r="192" ht="29" customHeight="1">
-      <c r="A192" s="11" t="inlineStr"/>
-      <c r="B192" s="12" t="inlineStr">
-        <is>
-          <t>Jun 29</t>
-        </is>
-      </c>
-      <c r="C192" s="13" t="inlineStr">
-        <is>
-          <t>Eat</t>
-        </is>
-      </c>
-      <c r="D192" s="12" t="inlineStr"/>
-      <c r="E192" s="14" t="inlineStr">
-        <is>
-          <t>1:30pm — Lunch at Rifugio Auronzo — cash is faster · hearty mountain lunch · allow 1hr</t>
-        </is>
-      </c>
-      <c r="F192" s="15" t="inlineStr">
-        <is>
-          <t>1hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="193" ht="40" customHeight="1">
+    <row r="193" ht="29" customHeight="1">
       <c r="A193" s="11" t="inlineStr"/>
       <c r="B193" s="12" t="inlineStr">
         <is>
@@ -4465,71 +4465,82 @@
       <c r="D193" s="12" t="inlineStr"/>
       <c r="E193" s="14" t="inlineStr">
         <is>
+          <t>1:30pm — Lunch at Rifugio Auronzo — cash is faster · hearty mountain lunch · allow 1hr</t>
+        </is>
+      </c>
+      <c r="F193" s="15" t="inlineStr">
+        <is>
+          <t>1hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="40" customHeight="1">
+      <c r="A194" s="11" t="inlineStr"/>
+      <c r="B194" s="12" t="inlineStr">
+        <is>
+          <t>Jun 29</t>
+        </is>
+      </c>
+      <c r="C194" s="13" t="inlineStr">
+        <is>
+          <t>Eat</t>
+        </is>
+      </c>
+      <c r="D194" s="12" t="inlineStr"/>
+      <c r="E194" s="14" t="inlineStr">
+        <is>
           <t>2:30pm — Tre Cime Highlights Walk — flat path to Rifugio Lavaredo (20 min each way) · see the towering north faces up close · allow 1hr 15min</t>
         </is>
       </c>
-      <c r="F193" s="15" t="inlineStr">
+      <c r="F194" s="15" t="inlineStr">
         <is>
           <t>20 min / 1hr / 15min</t>
         </is>
       </c>
     </row>
-    <row r="194" ht="50" customHeight="1">
-      <c r="A194" s="6" t="inlineStr"/>
-      <c r="B194" s="7" t="inlineStr">
+    <row r="195" ht="50" customHeight="1">
+      <c r="A195" s="6" t="inlineStr"/>
+      <c r="B195" s="7" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C194" s="8" t="inlineStr">
+      <c r="C195" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D194" s="7" t="inlineStr"/>
-      <c r="E194" s="9" t="inlineStr">
+      <c r="D195" s="7" t="inlineStr"/>
+      <c r="E195" s="9" t="inlineStr">
         <is>
           <t>3:45pm — Passo Gardena scenic drive — drive back down toll road · SS243 Gardena Pass (2,121m) · hairpin turns · low gear descent · ➕ Lagazuoi cable car optional if energy · ~1hr 15min drive</t>
         </is>
       </c>
-      <c r="F194" s="10" t="inlineStr">
+      <c r="F195" s="10" t="inlineStr">
         <is>
           <t>~1hr / 15min</t>
         </is>
       </c>
     </row>
-    <row r="195" ht="43" customHeight="1">
-      <c r="A195" s="25" t="inlineStr"/>
-      <c r="B195" s="26" t="inlineStr">
+    <row r="196" ht="43" customHeight="1">
+      <c r="A196" s="25" t="inlineStr"/>
+      <c r="B196" s="26" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C195" s="27" t="inlineStr">
+      <c r="C196" s="27" t="inlineStr">
         <is>
           <t>Stay</t>
         </is>
       </c>
-      <c r="D195" s="26" t="inlineStr"/>
-      <c r="E195" s="28" t="inlineStr">
+      <c r="D196" s="26" t="inlineStr"/>
+      <c r="E196" s="28" t="inlineStr">
         <is>
           <t>5:00pm — Kaiserau 1907, Collalbo — ✅ Check in · Via Peter Mayr 65, 39054 Collalbo · check-in 15:00–22:00 · unpack · rest · open a bottle of Italian wine</t>
         </is>
       </c>
-      <c r="F195" s="29" t="inlineStr"/>
-    </row>
-    <row r="196" ht="34" customHeight="1">
-      <c r="A196" s="30" t="inlineStr"/>
-      <c r="B196" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C196" s="32" t="inlineStr">
-        <is>
-          <t>⚠️ Braies 2026 access — road blocked 9am–4pm in peak season · arrive by 5:30am · P3 no reservation before 8am · €12 · leave before 8:30am · pivot to Prato Piazza if cloudy</t>
-        </is>
-      </c>
+      <c r="F196" s="29" t="inlineStr"/>
     </row>
     <row r="197" ht="34" customHeight="1">
       <c r="A197" s="30" t="inlineStr"/>
@@ -4540,7 +4551,7 @@
       </c>
       <c r="C197" s="32" t="inlineStr">
         <is>
-          <t>⚠️ Auronzo toll road 2026 — book at pass.auronzo.info · €40/car · 12-hour slot · book May 30 (exactly 30 days before) · rental plate: leave blank · update night before at Sillian hotel</t>
+          <t>⚠️ Braies 2026 access — road blocked 9am–4pm in peak season · arrive by 5:30am · P3 no reservation before 8am · €12 · leave before 8:30am · pivot to Prato Piazza if cloudy</t>
         </is>
       </c>
     </row>
@@ -4553,184 +4564,173 @@
       </c>
       <c r="C198" s="32" t="inlineStr">
         <is>
+          <t>⚠️ Auronzo toll road 2026 — book at pass.auronzo.info · €40/car · 12-hour slot · book May 30 (exactly 30 days before) · rental plate: leave blank · update night before at Sillian hotel</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="34" customHeight="1">
+      <c r="A199" s="30" t="inlineStr"/>
+      <c r="B199" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C199" s="32" t="inlineStr">
+        <is>
           <t>Cadini viewpoint tip — final 50m is a narrow ridge · secondary viewpoint 20m before the narrow section · 95% as good · go early — very crowded by midday · most dramatic jagged peak view in the Dolomites</t>
         </is>
       </c>
     </row>
-    <row r="199" ht="3" customHeight="1">
-      <c r="A199" s="33" t="n"/>
-      <c r="B199" s="33" t="n"/>
-      <c r="C199" s="33" t="n"/>
-      <c r="D199" s="33" t="n"/>
-      <c r="E199" s="33" t="n"/>
-      <c r="F199" s="33" t="n"/>
-    </row>
-    <row r="200" ht="20" customHeight="1">
-      <c r="A200" s="3" t="inlineStr">
+    <row r="200" ht="3" customHeight="1">
+      <c r="A200" s="33" t="n"/>
+      <c r="B200" s="33" t="n"/>
+      <c r="C200" s="33" t="n"/>
+      <c r="D200" s="33" t="n"/>
+      <c r="E200" s="33" t="n"/>
+      <c r="F200" s="33" t="n"/>
+    </row>
+    <row r="201" ht="20" customHeight="1">
+      <c r="A201" s="3" t="inlineStr">
         <is>
           <t>DAY 11  |  Jun 30  |  The Razor-Edge Peaks — Seceda · Val di Funes · Adolf Munkel Trail  |  ~80 km / 50 mi  ~2h total · Collalbo loop day</t>
         </is>
       </c>
     </row>
-    <row r="201" ht="15" customHeight="1">
-      <c r="A201" s="4" t="inlineStr">
+    <row r="202" ht="15" customHeight="1">
+      <c r="A202" s="4" t="inlineStr">
         <is>
           <t>Timeline: 8am Collalbo ▸ 8:45am Seceda cable car ▸ Trail 1 ridge + Rifugio Firenze lunch ▸ 1pm drive Val di Funes ▸ Santa Maddalena barrier + Panorama Trail ▸ St. Johann Ranui ▸ Zans traffic light ▸ 1:30pm Adolf Munkel Trail 35 ▸ Rifugio Odle lounge chairs ▸ 5:30pm descent ▸ 7pm Collalbo</t>
         </is>
       </c>
     </row>
-    <row r="202" ht="22" customHeight="1">
-      <c r="A202" s="5" t="inlineStr">
+    <row r="203" ht="22" customHeight="1">
+      <c r="A203" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ Seceda 8:45am — pre-booked · photos best 9–10:30am before clouds form · razor ridge Trail 1  |   Santa Maddalena 2026 barrier — park at Filler/Putzen lot · walk 25min Panorama Trail · cannot drive up  |   Zans traffic light Red → don't wait · park Ranui immediately + Bus 330 · saves hiking time</t>
         </is>
       </c>
     </row>
-    <row r="203" ht="50" customHeight="1">
-      <c r="A203" s="16" t="inlineStr"/>
-      <c r="B203" s="17" t="inlineStr">
+    <row r="204" ht="50" customHeight="1">
+      <c r="A204" s="16" t="inlineStr"/>
+      <c r="B204" s="17" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C203" s="16" t="inlineStr">
+      <c r="C204" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D203" s="17" t="inlineStr"/>
-      <c r="E203" s="18" t="inlineStr">
+      <c r="D204" s="17" t="inlineStr"/>
+      <c r="E204" s="18" t="inlineStr">
         <is>
           <t>️ Parking at Seceda valley station — no booking needed · €2.80/hr · 250+ spaces · arrive before 9am (your 8:45am slot guarantees this) · if full: Garage Central Ortisei €19.80/day · 10 min walk via La Curta escalator tun</t>
         </is>
       </c>
-      <c r="F203" s="19" t="inlineStr">
+      <c r="F204" s="19" t="inlineStr">
         <is>
           <t>€2.80 / €19.80 / 10 min</t>
         </is>
       </c>
     </row>
-    <row r="204" ht="49" customHeight="1">
-      <c r="A204" s="6" t="inlineStr"/>
-      <c r="B204" s="7" t="inlineStr">
+    <row r="205" ht="49" customHeight="1">
+      <c r="A205" s="6" t="inlineStr"/>
+      <c r="B205" s="7" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C204" s="8" t="inlineStr">
+      <c r="C205" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D204" s="7" t="inlineStr"/>
-      <c r="E204" s="9" t="inlineStr">
+      <c r="D205" s="7" t="inlineStr"/>
+      <c r="E205" s="9" t="inlineStr">
         <is>
           <t>⭐ ⭐ 8:45am — Seceda 360 cable car — ✅ Booked · Receipt 1161/678/554260 · €255 total · 2 adults €84.50 + 2 juniors €43 · print tickets before departure · best photos 9–10:30am before clouds</t>
         </is>
       </c>
-      <c r="F204" s="10" t="inlineStr">
+      <c r="F205" s="10" t="inlineStr">
         <is>
           <t>€255 / €84.50 / €43</t>
         </is>
       </c>
     </row>
-    <row r="205" ht="37" customHeight="1">
-      <c r="A205" s="20" t="inlineStr"/>
-      <c r="B205" s="21" t="inlineStr">
+    <row r="206" ht="37" customHeight="1">
+      <c r="A206" s="20" t="inlineStr"/>
+      <c r="B206" s="21" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C205" s="22" t="inlineStr">
+      <c r="C206" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D205" s="21" t="inlineStr"/>
-      <c r="E205" s="23" t="inlineStr">
+      <c r="D206" s="21" t="inlineStr"/>
+      <c r="E206" s="23" t="inlineStr">
         <is>
           <t>Trail 1 — Razor Edge ridge walk — from the cable car top follow Trail 1 to the summit cross · allow 1.5hrs for the ridge walk</t>
         </is>
       </c>
-      <c r="F205" s="24" t="inlineStr">
+      <c r="F206" s="24" t="inlineStr">
         <is>
           <t>5hr</t>
         </is>
       </c>
     </row>
-    <row r="206" ht="22" customHeight="1">
-      <c r="A206" s="11" t="inlineStr"/>
-      <c r="B206" s="12" t="inlineStr">
+    <row r="207" ht="22" customHeight="1">
+      <c r="A207" s="11" t="inlineStr"/>
+      <c r="B207" s="12" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C206" s="13" t="inlineStr">
+      <c r="C207" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D206" s="12" t="inlineStr"/>
-      <c r="E206" s="14" t="inlineStr">
+      <c r="D207" s="12" t="inlineStr"/>
+      <c r="E207" s="14" t="inlineStr">
         <is>
           <t>Lunch at Rifugio Firenze (2,039m) — allow 45 min</t>
         </is>
       </c>
-      <c r="F206" s="15" t="inlineStr">
+      <c r="F207" s="15" t="inlineStr">
         <is>
           <t>45 min</t>
         </is>
       </c>
     </row>
-    <row r="207" ht="38" customHeight="1">
-      <c r="A207" s="6" t="inlineStr"/>
-      <c r="B207" s="7" t="inlineStr">
+    <row r="208" ht="38" customHeight="1">
+      <c r="A208" s="6" t="inlineStr"/>
+      <c r="B208" s="7" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C207" s="8" t="inlineStr">
+      <c r="C208" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D207" s="7" t="inlineStr"/>
-      <c r="E207" s="9" t="inlineStr">
+      <c r="D208" s="7" t="inlineStr"/>
+      <c r="E208" s="9" t="inlineStr">
         <is>
           <t>1:00pm — Val di Funes (Santa Maddalena) —  2026 barrier — park Filler/Putzen lots · walk 25 min Panorama Trail · cannot drive up</t>
         </is>
       </c>
-      <c r="F207" s="10" t="inlineStr">
+      <c r="F208" s="10" t="inlineStr">
         <is>
           <t>25 min</t>
         </is>
       </c>
     </row>
-    <row r="208" ht="27" customHeight="1">
-      <c r="A208" s="16" t="inlineStr"/>
-      <c r="B208" s="17" t="inlineStr">
-        <is>
-          <t>Jun 30</t>
-        </is>
-      </c>
-      <c r="C208" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D208" s="17" t="inlineStr"/>
-      <c r="E208" s="18" t="inlineStr">
-        <is>
-          <t>⭐ St. Johann in Ranui — €4 turnstile for meadow access · card only · 15 min</t>
-        </is>
-      </c>
-      <c r="F208" s="19" t="inlineStr">
-        <is>
-          <t>€4 / 15 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="209" ht="31" customHeight="1">
+    <row r="209" ht="27" customHeight="1">
       <c r="A209" s="16" t="inlineStr"/>
       <c r="B209" s="17" t="inlineStr">
         <is>
@@ -4745,120 +4745,120 @@
       <c r="D209" s="17" t="inlineStr"/>
       <c r="E209" s="18" t="inlineStr">
         <is>
+          <t>⭐ St. Johann in Ranui — €4 turnstile for meadow access · card only · 15 min</t>
+        </is>
+      </c>
+      <c r="F209" s="19" t="inlineStr">
+        <is>
+          <t>€4 / 15 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="31" customHeight="1">
+      <c r="A210" s="16" t="inlineStr"/>
+      <c r="B210" s="17" t="inlineStr">
+        <is>
+          <t>Jun 30</t>
+        </is>
+      </c>
+      <c r="C210" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D210" s="17" t="inlineStr"/>
+      <c r="E210" s="18" t="inlineStr">
+        <is>
           <t>⭐ ⭐ Santa Maddalena viewpoint — most photographed scene in South Tyrol · best light: late afternoon</t>
         </is>
       </c>
-      <c r="F209" s="19" t="inlineStr"/>
-    </row>
-    <row r="210" ht="29" customHeight="1">
-      <c r="A210" s="6" t="inlineStr"/>
-      <c r="B210" s="7" t="inlineStr">
+      <c r="F210" s="19" t="inlineStr"/>
+    </row>
+    <row r="211" ht="29" customHeight="1">
+      <c r="A211" s="6" t="inlineStr"/>
+      <c r="B211" s="7" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C210" s="8" t="inlineStr">
+      <c r="C211" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D210" s="7" t="inlineStr"/>
-      <c r="E210" s="9" t="inlineStr">
+      <c r="D211" s="7" t="inlineStr"/>
+      <c r="E211" s="9" t="inlineStr">
         <is>
           <t>⚠️ Zans traffic light —  Green = drive up ·  Red = park Ranui + Bus 330 · don't wait</t>
         </is>
       </c>
-      <c r="F210" s="10" t="inlineStr"/>
-    </row>
-    <row r="211" ht="33" customHeight="1">
-      <c r="A211" s="20" t="inlineStr"/>
-      <c r="B211" s="21" t="inlineStr">
+      <c r="F211" s="10" t="inlineStr"/>
+    </row>
+    <row r="212" ht="33" customHeight="1">
+      <c r="A212" s="20" t="inlineStr"/>
+      <c r="B212" s="21" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C211" s="22" t="inlineStr">
+      <c r="C212" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D211" s="21" t="inlineStr"/>
-      <c r="E211" s="23" t="inlineStr">
+      <c r="D212" s="21" t="inlineStr"/>
+      <c r="E212" s="23" t="inlineStr">
         <is>
           <t>1:30pm — Adolf Munkel Trail 35 — from Parkplatz Zanser Alm (Zannes) trailhead · Trail 35 (Via delle Odle)</t>
         </is>
       </c>
-      <c r="F211" s="24" t="inlineStr"/>
-    </row>
-    <row r="212" ht="38" customHeight="1">
-      <c r="A212" s="11" t="inlineStr"/>
-      <c r="B212" s="12" t="inlineStr">
+      <c r="F212" s="24" t="inlineStr"/>
+    </row>
+    <row r="213" ht="38" customHeight="1">
+      <c r="A213" s="11" t="inlineStr"/>
+      <c r="B213" s="12" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C212" s="13" t="inlineStr">
+      <c r="C213" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D212" s="12" t="inlineStr"/>
-      <c r="E212" s="14" t="inlineStr">
+      <c r="D213" s="12" t="inlineStr"/>
+      <c r="E213" s="14" t="inlineStr">
         <is>
           <t>⭐ ⭐ Rifugio Odle / Geisler Alm (1,986m) — the Cinema of the Odle — the best seats in the Dolomites · cash is faster but cards accepted</t>
         </is>
       </c>
-      <c r="F212" s="15" t="inlineStr"/>
-    </row>
-    <row r="213" ht="36" customHeight="1">
-      <c r="A213" s="6" t="inlineStr"/>
-      <c r="B213" s="7" t="inlineStr">
+      <c r="F213" s="15" t="inlineStr"/>
+    </row>
+    <row r="214" ht="36" customHeight="1">
+      <c r="A214" s="6" t="inlineStr"/>
+      <c r="B214" s="7" t="inlineStr">
         <is>
           <t>Jun 30</t>
         </is>
       </c>
-      <c r="C213" s="8" t="inlineStr">
+      <c r="C214" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D213" s="7" t="inlineStr"/>
-      <c r="E213" s="9" t="inlineStr">
+      <c r="D214" s="7" t="inlineStr"/>
+      <c r="E214" s="9" t="inlineStr">
         <is>
           <t>5:30pm — Descent to Zannes car park — ~1hr back down · same trail · arrive Zannes ~6:30pm · drive 50 min back to Collalbo</t>
         </is>
       </c>
-      <c r="F213" s="10" t="inlineStr">
+      <c r="F214" s="10" t="inlineStr">
         <is>
           <t>~1hr / 50 min</t>
         </is>
       </c>
     </row>
-    <row r="214" ht="29" customHeight="1">
-      <c r="A214" s="25" t="inlineStr"/>
-      <c r="B214" s="26" t="inlineStr">
-        <is>
-          <t>Jun 30</t>
-        </is>
-      </c>
-      <c r="C214" s="27" t="inlineStr">
-        <is>
-          <t>Stay</t>
-        </is>
-      </c>
-      <c r="D214" s="26" t="inlineStr"/>
-      <c r="E214" s="28" t="inlineStr">
-        <is>
-          <t>⭐ Renon Earth Pyramids — evening walk — ➕ Optional if energy allows · 5 min from hotel</t>
-        </is>
-      </c>
-      <c r="F214" s="29" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="215" ht="19" customHeight="1">
+    <row r="215" ht="29" customHeight="1">
       <c r="A215" s="25" t="inlineStr"/>
       <c r="B215" s="26" t="inlineStr">
         <is>
@@ -4873,25 +4873,36 @@
       <c r="D215" s="26" t="inlineStr"/>
       <c r="E215" s="28" t="inlineStr">
         <is>
+          <t>⭐ Renon Earth Pyramids — evening walk — ➕ Optional if energy allows · 5 min from hotel</t>
+        </is>
+      </c>
+      <c r="F215" s="29" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="19" customHeight="1">
+      <c r="A216" s="25" t="inlineStr"/>
+      <c r="B216" s="26" t="inlineStr">
+        <is>
+          <t>Jun 30</t>
+        </is>
+      </c>
+      <c r="C216" s="27" t="inlineStr">
+        <is>
+          <t>Stay</t>
+        </is>
+      </c>
+      <c r="D216" s="26" t="inlineStr"/>
+      <c r="E216" s="28" t="inlineStr">
+        <is>
           <t>Night 2 — Kaiserau 1907, Collalbo</t>
         </is>
       </c>
-      <c r="F215" s="29" t="inlineStr"/>
-    </row>
-    <row r="216" ht="34" customHeight="1">
-      <c r="A216" s="30" t="inlineStr"/>
-      <c r="B216" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C216" s="32" t="inlineStr">
-        <is>
-          <t>Santa Maddalena 2026 barrier — physical barrier blocks non-resident cars since May 2026 · park Filler or Putzen lots in village · follow Panorama Trail signs · 25 min uphill walk to the viewpoint · you can no longer drive to the famous phot</t>
-        </is>
-      </c>
-    </row>
-    <row r="217" ht="30" customHeight="1">
+      <c r="F216" s="29" t="inlineStr"/>
+    </row>
+    <row r="217" ht="34" customHeight="1">
       <c r="A217" s="30" t="inlineStr"/>
       <c r="B217" s="31" t="inlineStr">
         <is>
@@ -4900,11 +4911,11 @@
       </c>
       <c r="C217" s="32" t="inlineStr">
         <is>
-          <t>Zans traffic light 2026 — Green = drive up · Red = park at Ranui immediately + Bus 330 every 30–60 min · do not wait at the gate — bus is faster</t>
-        </is>
-      </c>
-    </row>
-    <row r="218" ht="34" customHeight="1">
+          <t>Santa Maddalena 2026 barrier — physical barrier blocks non-resident cars since May 2026 · park Filler or Putzen lots in village · follow Panorama Trail signs · 25 min uphill walk to the viewpoint · you can no longer drive to the famous phot</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="30" customHeight="1">
       <c r="A218" s="30" t="inlineStr"/>
       <c r="B218" s="31" t="inlineStr">
         <is>
@@ -4913,112 +4924,101 @@
       </c>
       <c r="C218" s="32" t="inlineStr">
         <is>
+          <t>Zans traffic light 2026 — Green = drive up · Red = park at Ranui immediately + Bus 330 every 30–60 min · do not wait at the gate — bus is faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="34" customHeight="1">
+      <c r="A219" s="30" t="inlineStr"/>
+      <c r="B219" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C219" s="32" t="inlineStr">
+        <is>
           <t>Photography windows — Seceda ridge: 9:00–10:30am before clouds form · Santa Maddalena viewpoint: late afternoon — sun behind you · Odle peaks lit directly · morning light hits the wrong side of the peaks</t>
         </is>
       </c>
     </row>
-    <row r="219" ht="3" customHeight="1">
-      <c r="A219" s="33" t="n"/>
-      <c r="B219" s="33" t="n"/>
-      <c r="C219" s="33" t="n"/>
-      <c r="D219" s="33" t="n"/>
-      <c r="E219" s="33" t="n"/>
-      <c r="F219" s="33" t="n"/>
-    </row>
-    <row r="220" ht="20" customHeight="1">
-      <c r="A220" s="3" t="inlineStr">
+    <row r="220" ht="3" customHeight="1">
+      <c r="A220" s="33" t="n"/>
+      <c r="B220" s="33" t="n"/>
+      <c r="C220" s="33" t="n"/>
+      <c r="D220" s="33" t="n"/>
+      <c r="E220" s="33" t="n"/>
+      <c r="F220" s="33" t="n"/>
+    </row>
+    <row r="221" ht="20" customHeight="1">
+      <c r="A221" s="3" t="inlineStr">
         <is>
           <t>DAY 12  |  Jul 1  |  Alpe di Siusi + Brenner Pass → Finkenberg — The Plateau &amp; The Pass  |  ~120 km / 75 mi  ~1h 45m · Collalbo → Finkenberg via Brenner</t>
         </is>
       </c>
     </row>
-    <row r="221" ht="15" customHeight="1">
-      <c r="A221" s="4" t="inlineStr">
+    <row r="222" ht="15" customHeight="1">
+      <c r="A222" s="4" t="inlineStr">
         <is>
           <t>Timeline: 7:45am Collalbo ▸ 8:30am St. Valentin gate (must be before 9am) ▸ 8:45am P2 Compatsch ▸ 9:15am Bullaccia loop ▸ Hexenbänke viewpoint ▸ 12pm Tschötsch Alm lunch ▸ 1:30pm depart ▸ Brenner construction ▸ M-Preis Mayrhofen ▸ 4:30pm Keyone Rooms Finkenberg</t>
         </is>
       </c>
     </row>
-    <row r="222" ht="22" customHeight="1">
-      <c r="A222" s="5" t="inlineStr">
+    <row r="223" ht="22" customHeight="1">
+      <c r="A223" s="5" t="inlineStr">
         <is>
           <t>Key: ️ Plan A: P2 Compatsch — keep checking seiseralm.it for cancellations · must arrive before 9am · €30  |   Plan B: Seis cable car → Compatsch — park in Seis · ~€30/adult RT · no booking · no 9am rule · same trailhead  |   St. Valentin gate closes 9:00am SHARP — leave Collalbo 7:45am · arrive 8:30am · no exceptions  |  ❌ Skip Rifugio Zallinger — 4hr RT or 2 extra lifts · impractical · eat at Tschötsch Alm instead  |  ⚠️ Brenner Lueg Bridge construction 2026 — 30–45 min delay · Digital Flex toll essential</t>
         </is>
       </c>
     </row>
-    <row r="223" ht="40" customHeight="1">
-      <c r="A223" s="6" t="inlineStr"/>
-      <c r="B223" s="7" t="inlineStr">
+    <row r="224" ht="40" customHeight="1">
+      <c r="A224" s="6" t="inlineStr"/>
+      <c r="B224" s="7" t="inlineStr">
         <is>
           <t>Jul 1</t>
         </is>
       </c>
-      <c r="C223" s="8" t="inlineStr">
+      <c r="C224" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D223" s="7" t="inlineStr"/>
-      <c r="E223" s="9" t="inlineStr">
+      <c r="D224" s="7" t="inlineStr"/>
+      <c r="E224" s="9" t="inlineStr">
         <is>
           <t>⏰ 7:45am — Depart Collalbo — 40 min drive to the Alpe di Siusi St. Valentin gate · checkout Kaiserau 1907 before leaving · luggage in the car</t>
         </is>
       </c>
-      <c r="F223" s="10" t="inlineStr">
+      <c r="F224" s="10" t="inlineStr">
         <is>
           <t>40 min</t>
         </is>
       </c>
     </row>
-    <row r="224" ht="31" customHeight="1">
-      <c r="A224" s="34" t="inlineStr"/>
-      <c r="B224" s="35" t="inlineStr">
+    <row r="225" ht="31" customHeight="1">
+      <c r="A225" s="34" t="inlineStr"/>
+      <c r="B225" s="35" t="inlineStr">
         <is>
           <t>Jul 1</t>
         </is>
       </c>
-      <c r="C224" s="36" t="inlineStr">
+      <c r="C225" s="36" t="inlineStr">
         <is>
           <t>Alert</t>
         </is>
       </c>
-      <c r="D224" s="35" t="inlineStr"/>
-      <c r="E224" s="37" t="inlineStr">
+      <c r="D225" s="35" t="inlineStr"/>
+      <c r="E225" s="37" t="inlineStr">
         <is>
           <t>⚠️ CRITICAL: St. Valentin Gate — before 9:00am — 9:01am = turned back · €120+ cable car alternative</t>
         </is>
       </c>
-      <c r="F224" s="38" t="inlineStr">
+      <c r="F225" s="38" t="inlineStr">
         <is>
           <t>€120</t>
         </is>
       </c>
     </row>
-    <row r="225" ht="50" customHeight="1">
-      <c r="A225" s="20" t="inlineStr"/>
-      <c r="B225" s="21" t="inlineStr">
-        <is>
-          <t>Jul 1</t>
-        </is>
-      </c>
-      <c r="C225" s="22" t="inlineStr">
-        <is>
-          <t>Hike</t>
-        </is>
-      </c>
-      <c r="D225" s="21" t="inlineStr"/>
-      <c r="E225" s="23" t="inlineStr">
-        <is>
-          <t>P2 Compatsch parking — ⚠️ Currently fully booked · keep checking seiseralm.it for cancellations · slots open up to 6 days before · €30 cash · must arrive before 9am · cameras enforce the gate ·  Plan B: Seis–Compatsch ca</t>
-        </is>
-      </c>
-      <c r="F225" s="24" t="inlineStr">
-        <is>
-          <t>€30 / €30 / €65</t>
-        </is>
-      </c>
-    </row>
-    <row r="226" ht="34" customHeight="1">
+    <row r="226" ht="50" customHeight="1">
       <c r="A226" s="20" t="inlineStr"/>
       <c r="B226" s="21" t="inlineStr">
         <is>
@@ -5033,12 +5033,16 @@
       <c r="D226" s="21" t="inlineStr"/>
       <c r="E226" s="23" t="inlineStr">
         <is>
-          <t>9:15am — Bullaccia (Puflatsch) Loop — take the Telemix lift up from Compatsch · Trail PU (Puflatschumrundung)</t>
-        </is>
-      </c>
-      <c r="F226" s="24" t="inlineStr"/>
-    </row>
-    <row r="227" ht="23" customHeight="1">
+          <t>P2 Compatsch parking — ⚠️ Currently fully booked · keep checking seiseralm.it for cancellations · slots open up to 6 days before · €30 cash · must arrive before 9am · cameras enforce the gate ·  Plan B: Seis–Compatsch ca</t>
+        </is>
+      </c>
+      <c r="F226" s="24" t="inlineStr">
+        <is>
+          <t>€30 / €30 / €65</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="34" customHeight="1">
       <c r="A227" s="20" t="inlineStr"/>
       <c r="B227" s="21" t="inlineStr">
         <is>
@@ -5053,80 +5057,76 @@
       <c r="D227" s="21" t="inlineStr"/>
       <c r="E227" s="23" t="inlineStr">
         <is>
+          <t>9:15am — Bullaccia (Puflatsch) Loop — take the Telemix lift up from Compatsch · Trail PU (Puflatschumrundung)</t>
+        </is>
+      </c>
+      <c r="F227" s="24" t="inlineStr"/>
+    </row>
+    <row r="228" ht="23" customHeight="1">
+      <c r="A228" s="20" t="inlineStr"/>
+      <c r="B228" s="21" t="inlineStr">
+        <is>
+          <t>Jul 1</t>
+        </is>
+      </c>
+      <c r="C228" s="22" t="inlineStr">
+        <is>
+          <t>Hike</t>
+        </is>
+      </c>
+      <c r="D228" s="21" t="inlineStr"/>
+      <c r="E228" s="23" t="inlineStr">
+        <is>
           <t>⭐ Hexenbänke — Witches' Benches — signed from the trail</t>
         </is>
       </c>
-      <c r="F227" s="24" t="inlineStr"/>
-    </row>
-    <row r="228" ht="31" customHeight="1">
-      <c r="A228" s="11" t="inlineStr"/>
-      <c r="B228" s="12" t="inlineStr">
+      <c r="F228" s="24" t="inlineStr"/>
+    </row>
+    <row r="229" ht="31" customHeight="1">
+      <c r="A229" s="11" t="inlineStr"/>
+      <c r="B229" s="12" t="inlineStr">
         <is>
           <t>Jul 1</t>
         </is>
       </c>
-      <c r="C228" s="13" t="inlineStr">
+      <c r="C229" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D228" s="12" t="inlineStr"/>
-      <c r="E228" s="14" t="inlineStr">
+      <c r="D229" s="12" t="inlineStr"/>
+      <c r="E229" s="14" t="inlineStr">
         <is>
           <t>️ 12:00pm — Lunch: Tschötsch Alm or Arnika Hütte — ⚠️ Do NOT go to Rifugio Zallinger — allow 1hr</t>
         </is>
       </c>
-      <c r="F228" s="15" t="inlineStr">
+      <c r="F229" s="15" t="inlineStr">
         <is>
           <t>1hr</t>
         </is>
       </c>
     </row>
-    <row r="229" ht="27" customHeight="1">
-      <c r="A229" s="6" t="inlineStr"/>
-      <c r="B229" s="7" t="inlineStr">
+    <row r="230" ht="27" customHeight="1">
+      <c r="A230" s="6" t="inlineStr"/>
+      <c r="B230" s="7" t="inlineStr">
         <is>
           <t>Jul 1</t>
         </is>
       </c>
-      <c r="C229" s="8" t="inlineStr">
+      <c r="C230" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D229" s="7" t="inlineStr"/>
-      <c r="E229" s="9" t="inlineStr">
+      <c r="D230" s="7" t="inlineStr"/>
+      <c r="E230" s="9" t="inlineStr">
         <is>
           <t>1:30pm — Depart Alpe di Siusi — unrestricted descent · head north to Brenner</t>
         </is>
       </c>
-      <c r="F229" s="10" t="inlineStr"/>
-    </row>
-    <row r="230" ht="50" customHeight="1">
-      <c r="A230" s="16" t="inlineStr"/>
-      <c r="B230" s="17" t="inlineStr">
-        <is>
-          <t>Jul 1</t>
-        </is>
-      </c>
-      <c r="C230" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D230" s="17" t="inlineStr"/>
-      <c r="E230" s="18" t="inlineStr">
-        <is>
-          <t>⚠️ Brenner Pass — Lueg Bridge construction — 30–45 min delay expected · Digital Flex toll green lanes · €11.50 · ➡️ If standstill at A22/A13 toll plaza: take B182 Brenner Route Nationale — free state road running paralle</t>
-        </is>
-      </c>
-      <c r="F230" s="19" t="inlineStr">
-        <is>
-          <t>45 min / €11.50</t>
-        </is>
-      </c>
-    </row>
-    <row r="231" ht="18" customHeight="1">
+      <c r="F230" s="10" t="inlineStr"/>
+    </row>
+    <row r="231" ht="50" customHeight="1">
       <c r="A231" s="16" t="inlineStr"/>
       <c r="B231" s="17" t="inlineStr">
         <is>
@@ -5141,93 +5141,104 @@
       <c r="D231" s="17" t="inlineStr"/>
       <c r="E231" s="18" t="inlineStr">
         <is>
+          <t>⚠️ Brenner Pass — Lueg Bridge construction — 30–45 min delay expected · Digital Flex toll green lanes · €11.50 · ➡️ If standstill at A22/A13 toll plaza: take B182 Brenner Route Nationale — free state road running paralle</t>
+        </is>
+      </c>
+      <c r="F231" s="19" t="inlineStr">
+        <is>
+          <t>45 min / €11.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="18" customHeight="1">
+      <c r="A232" s="16" t="inlineStr"/>
+      <c r="B232" s="17" t="inlineStr">
+        <is>
+          <t>Jul 1</t>
+        </is>
+      </c>
+      <c r="C232" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D232" s="17" t="inlineStr"/>
+      <c r="E232" s="18" t="inlineStr">
+        <is>
           <t>Austrian vignette still valid?</t>
         </is>
       </c>
-      <c r="F231" s="19" t="inlineStr"/>
-    </row>
-    <row r="232" ht="35" customHeight="1">
-      <c r="A232" s="11" t="inlineStr"/>
-      <c r="B232" s="12" t="inlineStr">
+      <c r="F232" s="19" t="inlineStr"/>
+    </row>
+    <row r="233" ht="35" customHeight="1">
+      <c r="A233" s="11" t="inlineStr"/>
+      <c r="B233" s="12" t="inlineStr">
         <is>
           <t>Jul 1</t>
         </is>
       </c>
-      <c r="C232" s="13" t="inlineStr">
+      <c r="C233" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D232" s="12" t="inlineStr"/>
-      <c r="E232" s="14" t="inlineStr">
+      <c r="D233" s="12" t="inlineStr"/>
+      <c r="E233" s="14" t="inlineStr">
         <is>
           <t>M-Preis Supermarket, Mayrhofen — Finkenberg is up a winding road — nothing open nearby in the evening · allow 20 min</t>
         </is>
       </c>
-      <c r="F232" s="15" t="inlineStr">
+      <c r="F233" s="15" t="inlineStr">
         <is>
           <t>20 min</t>
         </is>
       </c>
     </row>
-    <row r="233" ht="34" customHeight="1">
-      <c r="A233" s="16" t="inlineStr"/>
-      <c r="B233" s="17" t="inlineStr">
+    <row r="234" ht="34" customHeight="1">
+      <c r="A234" s="16" t="inlineStr"/>
+      <c r="B234" s="17" t="inlineStr">
         <is>
           <t>Jul 1</t>
         </is>
       </c>
-      <c r="C233" s="16" t="inlineStr">
+      <c r="C234" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D233" s="17" t="inlineStr"/>
-      <c r="E233" s="18" t="inlineStr">
+      <c r="D234" s="17" t="inlineStr"/>
+      <c r="E234" s="18" t="inlineStr">
         <is>
           <t>4:30pm — Keyone Rooms, Finkenberg — $176 / €152.92 · ⚠️ Driveway can be steep — take it slowly on the approach</t>
         </is>
       </c>
-      <c r="F233" s="19" t="inlineStr">
+      <c r="F234" s="19" t="inlineStr">
         <is>
           <t>$176 / €152.92</t>
         </is>
       </c>
     </row>
-    <row r="234" ht="29" customHeight="1">
-      <c r="A234" s="6" t="inlineStr"/>
-      <c r="B234" s="7" t="inlineStr">
+    <row r="235" ht="29" customHeight="1">
+      <c r="A235" s="6" t="inlineStr"/>
+      <c r="B235" s="7" t="inlineStr">
         <is>
           <t>Jul 1</t>
         </is>
       </c>
-      <c r="C234" s="8" t="inlineStr">
+      <c r="C235" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D234" s="7" t="inlineStr"/>
-      <c r="E234" s="9" t="inlineStr">
+      <c r="D235" s="7" t="inlineStr"/>
+      <c r="E235" s="9" t="inlineStr">
         <is>
           <t>Dinner in Finkenberg or Mayrhofen — or drive 5 min down to Mayrhofen for more options</t>
         </is>
       </c>
-      <c r="F234" s="10" t="inlineStr">
+      <c r="F235" s="10" t="inlineStr">
         <is>
           <t>5 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="235" ht="34" customHeight="1">
-      <c r="A235" s="30" t="inlineStr"/>
-      <c r="B235" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C235" s="32" t="inlineStr">
-        <is>
-          <t>9:00am St. Valentin gate — non-negotiable — electronic barrier closes to private cars at exactly 9am · 9:01am = turned back · €120+ family cable car alternative · leave Collalbo by 7:45am</t>
         </is>
       </c>
     </row>
@@ -5240,7 +5251,7 @@
       </c>
       <c r="C236" s="32" t="inlineStr">
         <is>
-          <t>⚠️ Brenner Lueg Bridge 2026 — single-lane renovation · 30–45 min delay expected · Digital Flex toll at autobrennero.it · €11.50 · green Video Toll lanes · saves 1hr vs manual queue</t>
+          <t>9:00am St. Valentin gate — non-negotiable — electronic barrier closes to private cars at exactly 9am · 9:01am = turned back · €120+ family cable car alternative · leave Collalbo by 7:45am</t>
         </is>
       </c>
     </row>
@@ -5253,11 +5264,11 @@
       </c>
       <c r="C237" s="32" t="inlineStr">
         <is>
-          <t>Hexenbänke — Witches' Benches — giant stone formations on the Bullaccia ridge · highest point of the plateau · best 360° photo spot · signed from the trail · kids love the legend</t>
-        </is>
-      </c>
-    </row>
-    <row r="238" ht="32" customHeight="1">
+          <t>⚠️ Brenner Lueg Bridge 2026 — single-lane renovation · 30–45 min delay expected · Digital Flex toll at autobrennero.it · €11.50 · green Video Toll lanes · saves 1hr vs manual queue</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="34" customHeight="1">
       <c r="A238" s="30" t="inlineStr"/>
       <c r="B238" s="31" t="inlineStr">
         <is>
@@ -5266,333 +5277,333 @@
       </c>
       <c r="C238" s="32" t="inlineStr">
         <is>
+          <t>Hexenbänke — Witches' Benches — giant stone formations on the Bullaccia ridge · highest point of the plateau · best 360° photo spot · signed from the trail · kids love the legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="32" customHeight="1">
+      <c r="A239" s="30" t="inlineStr"/>
+      <c r="B239" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C239" s="32" t="inlineStr">
+        <is>
           <t>M-Preis Mayrhofen — stop before Finkenberg · buy breakfast for Day 13 · nothing open near Keyone in evenings · steep winding road to Finkenberg — take slowly</t>
         </is>
       </c>
     </row>
-    <row r="239" ht="3" customHeight="1">
-      <c r="A239" s="33" t="n"/>
-      <c r="B239" s="33" t="n"/>
-      <c r="C239" s="33" t="n"/>
-      <c r="D239" s="33" t="n"/>
-      <c r="E239" s="33" t="n"/>
-      <c r="F239" s="33" t="n"/>
-    </row>
-    <row r="240" ht="20" customHeight="1">
-      <c r="A240" s="3" t="inlineStr">
+    <row r="240" ht="3" customHeight="1">
+      <c r="A240" s="33" t="n"/>
+      <c r="B240" s="33" t="n"/>
+      <c r="C240" s="33" t="n"/>
+      <c r="D240" s="33" t="n"/>
+      <c r="E240" s="33" t="n"/>
+      <c r="F240" s="33" t="n"/>
+    </row>
+    <row r="241" ht="20" customHeight="1">
+      <c r="A241" s="3" t="inlineStr">
         <is>
           <t>DAY 13  |  Jul 2  |  High Bridges &amp; Deep Lakes — Olpererhütte · Achensee · Swarovski → Bichlbach  |  ~150 km / 93 mi  ~2h 30m incl. Achensee + Swarovski stops</t>
         </is>
       </c>
     </row>
-    <row r="241" ht="15" customHeight="1">
-      <c r="A241" s="4" t="inlineStr">
+    <row r="242" ht="15" customHeight="1">
+      <c r="A242" s="4" t="inlineStr">
         <is>
           <t>Timeline: 8am Finkenberg ▸ 8:30am Schlegeis toll €17 ▸ 9am Olpererhütte hike ▸ 10:30am Kebema bridge ▸ 11am lunch ▸ 1:30pm descent ▸ Swarovski (if rain) ▸ Achensee optional ▸ Fern Pass ▸ 7:30pm Bichlbach ▸ Heiterwanger See sunset</t>
         </is>
       </c>
     </row>
-    <row r="242" ht="22" customHeight="1">
-      <c r="A242" s="5" t="inlineStr">
+    <row r="243" ht="22" customHeight="1">
+      <c r="A243" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ Arrive dam by 8:45am — reach Kebema bridge 10:30am · beats 45min photo queue by midday  |  ☀️ Plan A (sunny): Achensee — steamboat ~€22/adult OR free Gaisalm promenade walk if kids tired  |  ️ Plan B (rain/cloudy): Swarovski Crystal Worlds — 5min off A12 · ~€22/adult · no booking needed</t>
         </is>
       </c>
     </row>
-    <row r="243" ht="31" customHeight="1">
-      <c r="A243" s="6" t="inlineStr"/>
-      <c r="B243" s="7" t="inlineStr">
+    <row r="244" ht="31" customHeight="1">
+      <c r="A244" s="6" t="inlineStr"/>
+      <c r="B244" s="7" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C243" s="8" t="inlineStr">
+      <c r="C244" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D243" s="7" t="inlineStr"/>
-      <c r="E243" s="9" t="inlineStr">
+      <c r="D244" s="7" t="inlineStr"/>
+      <c r="E244" s="9" t="inlineStr">
         <is>
           <t>⏰ 8:00am — Depart Finkenberg — 20 min to Schlegeis · ⚠️ tunnel traffic lights = up to 15 min wait</t>
         </is>
       </c>
-      <c r="F243" s="10" t="inlineStr">
+      <c r="F244" s="10" t="inlineStr">
         <is>
           <t>20 min / 15 min</t>
         </is>
       </c>
     </row>
-    <row r="244" ht="27" customHeight="1">
-      <c r="A244" s="16" t="inlineStr"/>
-      <c r="B244" s="17" t="inlineStr">
+    <row r="245" ht="27" customHeight="1">
+      <c r="A245" s="16" t="inlineStr"/>
+      <c r="B245" s="17" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C244" s="16" t="inlineStr">
+      <c r="C245" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D244" s="17" t="inlineStr"/>
-      <c r="E244" s="18" t="inlineStr">
+      <c r="D245" s="17" t="inlineStr"/>
+      <c r="E245" s="18" t="inlineStr">
         <is>
           <t>8:30am — Schlegeis Alpine Road toll — €17 · pay at the gate (cash or card)</t>
         </is>
       </c>
-      <c r="F244" s="19" t="inlineStr">
+      <c r="F245" s="19" t="inlineStr">
         <is>
           <t>€17</t>
         </is>
       </c>
     </row>
-    <row r="245" ht="29" customHeight="1">
-      <c r="A245" s="20" t="inlineStr"/>
-      <c r="B245" s="21" t="inlineStr">
+    <row r="246" ht="29" customHeight="1">
+      <c r="A246" s="20" t="inlineStr"/>
+      <c r="B246" s="21" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C245" s="22" t="inlineStr">
+      <c r="C246" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D245" s="21" t="inlineStr"/>
-      <c r="E245" s="23" t="inlineStr">
+      <c r="D246" s="21" t="inlineStr"/>
+      <c r="E246" s="23" t="inlineStr">
         <is>
           <t>9:00am — Olpererhütte Hike (Trail 502) — 3km / 1.9mi each way · well-maintained trail</t>
         </is>
       </c>
-      <c r="F245" s="24" t="inlineStr">
+      <c r="F246" s="24" t="inlineStr">
         <is>
           <t>3km</t>
         </is>
       </c>
     </row>
-    <row r="246" ht="41" customHeight="1">
-      <c r="A246" s="16" t="inlineStr"/>
-      <c r="B246" s="17" t="inlineStr">
+    <row r="247" ht="41" customHeight="1">
+      <c r="A247" s="16" t="inlineStr"/>
+      <c r="B247" s="17" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C246" s="16" t="inlineStr">
+      <c r="C247" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D246" s="17" t="inlineStr"/>
-      <c r="E246" s="18" t="inlineStr">
+      <c r="D247" s="17" t="inlineStr"/>
+      <c r="E247" s="18" t="inlineStr">
         <is>
           <t>⭐ ⭐ 10:30am — Kebema Suspension Bridge (Olperer Panoramabrücke) — 3–4 min past the hut · floats in mid-air above the turquoise reservoir 600m below</t>
         </is>
       </c>
-      <c r="F246" s="19" t="inlineStr">
+      <c r="F247" s="19" t="inlineStr">
         <is>
           <t>4 min</t>
         </is>
       </c>
     </row>
-    <row r="247" ht="36" customHeight="1">
-      <c r="A247" s="11" t="inlineStr"/>
-      <c r="B247" s="12" t="inlineStr">
+    <row r="248" ht="36" customHeight="1">
+      <c r="A248" s="11" t="inlineStr"/>
+      <c r="B248" s="12" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C247" s="13" t="inlineStr">
+      <c r="C248" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D247" s="12" t="inlineStr"/>
-      <c r="E247" s="14" t="inlineStr">
+      <c r="D248" s="12" t="inlineStr"/>
+      <c r="E248" s="14" t="inlineStr">
         <is>
           <t>️ 11:00am — Lunch at Olpererhütte — cash preferred (but Wi-Fi available — check your Neuschwanstein booking!) · allow 1hr</t>
         </is>
       </c>
-      <c r="F247" s="15" t="inlineStr">
+      <c r="F248" s="15" t="inlineStr">
         <is>
           <t>1hr</t>
         </is>
       </c>
     </row>
-    <row r="248" ht="35" customHeight="1">
-      <c r="A248" s="20" t="inlineStr"/>
-      <c r="B248" s="21" t="inlineStr">
+    <row r="249" ht="35" customHeight="1">
+      <c r="A249" s="20" t="inlineStr"/>
+      <c r="B249" s="21" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C248" s="22" t="inlineStr">
+      <c r="C249" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D248" s="21" t="inlineStr"/>
-      <c r="E248" s="23" t="inlineStr">
+      <c r="D249" s="21" t="inlineStr"/>
+      <c r="E249" s="23" t="inlineStr">
         <is>
           <t>1:30pm — Descent to the dam — ~1hr back down same trail · easier on the knees than going up · back at car ~2:30pm</t>
         </is>
       </c>
-      <c r="F248" s="24" t="inlineStr">
+      <c r="F249" s="24" t="inlineStr">
         <is>
           <t>~1hr</t>
         </is>
       </c>
     </row>
-    <row r="249" ht="50" customHeight="1">
-      <c r="A249" s="6" t="inlineStr"/>
-      <c r="B249" s="7" t="inlineStr">
+    <row r="250" ht="50" customHeight="1">
+      <c r="A250" s="6" t="inlineStr"/>
+      <c r="B250" s="7" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C249" s="8" t="inlineStr">
+      <c r="C250" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D249" s="7" t="inlineStr"/>
-      <c r="E249" s="9" t="inlineStr">
+      <c r="D250" s="7" t="inlineStr"/>
+      <c r="E250" s="9" t="inlineStr">
         <is>
           <t>☀️ Plan A — Sunny: Achensee — 50 min drive north from Schlegeis · park at Pertisau · Option 1: Achensee steamboat ~€22/adult · allow 1.5hrs · Option 2 (kids tired): Gaisalm promenade walk — free · same fjord-like views ·</t>
         </is>
       </c>
-      <c r="F249" s="10" t="inlineStr">
+      <c r="F250" s="10" t="inlineStr">
         <is>
           <t>50 min / €22 / 5hr</t>
         </is>
       </c>
     </row>
-    <row r="250" ht="50" customHeight="1">
-      <c r="A250" s="20" t="inlineStr"/>
-      <c r="B250" s="21" t="inlineStr">
+    <row r="251" ht="50" customHeight="1">
+      <c r="A251" s="20" t="inlineStr"/>
+      <c r="B251" s="21" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C250" s="22" t="inlineStr">
+      <c r="C251" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D250" s="21" t="inlineStr"/>
-      <c r="E250" s="23" t="inlineStr">
+      <c r="D251" s="21" t="inlineStr"/>
+      <c r="E251" s="23" t="inlineStr">
         <is>
           <t>️ Plan B — Rain/Cloudy: Swarovski Crystal Worlds — 5 min off A12 at Wattens · ~€22/adult · allow 1.5–2hrs · indoor immersive art installation · perfect rainy-day refuge after cold wet Olpererhütte hike · no booking neede</t>
         </is>
       </c>
-      <c r="F250" s="24" t="inlineStr">
+      <c r="F251" s="24" t="inlineStr">
         <is>
           <t>5 min / €22 / 2hr</t>
         </is>
       </c>
     </row>
-    <row r="251" ht="29" customHeight="1">
-      <c r="A251" s="6" t="inlineStr"/>
-      <c r="B251" s="7" t="inlineStr">
+    <row r="252" ht="29" customHeight="1">
+      <c r="A252" s="6" t="inlineStr"/>
+      <c r="B252" s="7" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C251" s="8" t="inlineStr">
+      <c r="C252" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D251" s="7" t="inlineStr"/>
-      <c r="E251" s="9" t="inlineStr">
+      <c r="D252" s="7" t="inlineStr"/>
+      <c r="E252" s="9" t="inlineStr">
         <is>
           <t>⚠️ Fern Pass warning on drive to Bichlbach — village Gasthäuser are relaxed about timing</t>
         </is>
       </c>
-      <c r="F251" s="10" t="inlineStr"/>
-    </row>
-    <row r="252" ht="33" customHeight="1">
-      <c r="A252" s="25" t="inlineStr"/>
-      <c r="B252" s="26" t="inlineStr">
+      <c r="F252" s="10" t="inlineStr"/>
+    </row>
+    <row r="253" ht="33" customHeight="1">
+      <c r="A253" s="25" t="inlineStr"/>
+      <c r="B253" s="26" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C252" s="27" t="inlineStr">
+      <c r="C253" s="27" t="inlineStr">
         <is>
           <t>Stay</t>
         </is>
       </c>
-      <c r="D252" s="26" t="inlineStr"/>
-      <c r="E252" s="28" t="inlineStr">
+      <c r="D253" s="26" t="inlineStr"/>
+      <c r="E253" s="28" t="inlineStr">
         <is>
           <t>~7:30pm — Landhaus Bichlbach — $467 / €405 · Heiterwanger See lake is a 20 min evening walk from the hotel</t>
         </is>
       </c>
-      <c r="F252" s="29" t="inlineStr">
+      <c r="F253" s="29" t="inlineStr">
         <is>
           <t>$467 / €405 / 20 min</t>
         </is>
       </c>
     </row>
-    <row r="253" ht="28" customHeight="1">
-      <c r="A253" s="16" t="inlineStr"/>
-      <c r="B253" s="17" t="inlineStr">
+    <row r="254" ht="28" customHeight="1">
+      <c r="A254" s="16" t="inlineStr"/>
+      <c r="B254" s="17" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C253" s="16" t="inlineStr">
+      <c r="C254" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D253" s="17" t="inlineStr"/>
-      <c r="E253" s="18" t="inlineStr">
+      <c r="D254" s="17" t="inlineStr"/>
+      <c r="E254" s="18" t="inlineStr">
         <is>
           <t>⭐ Heiterwanger See sunset walk — easy 20 min walk from Landhaus along Panoramaweg</t>
         </is>
       </c>
-      <c r="F253" s="19" t="inlineStr">
+      <c r="F254" s="19" t="inlineStr">
         <is>
           <t>20 min</t>
         </is>
       </c>
     </row>
-    <row r="254" ht="25" customHeight="1">
-      <c r="A254" s="6" t="inlineStr"/>
-      <c r="B254" s="7" t="inlineStr">
+    <row r="255" ht="25" customHeight="1">
+      <c r="A255" s="6" t="inlineStr"/>
+      <c r="B255" s="7" t="inlineStr">
         <is>
           <t>Jul 2</t>
         </is>
       </c>
-      <c r="C254" s="8" t="inlineStr">
+      <c r="C255" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D254" s="7" t="inlineStr"/>
-      <c r="E254" s="9" t="inlineStr">
+      <c r="D255" s="7" t="inlineStr"/>
+      <c r="E255" s="9" t="inlineStr">
         <is>
           <t>Dinner + pack bags — Gasthof Bichlbach · checkout 8am · alarm 7am</t>
         </is>
       </c>
-      <c r="F254" s="10" t="inlineStr"/>
-    </row>
-    <row r="255" ht="32" customHeight="1">
-      <c r="A255" s="30" t="inlineStr"/>
-      <c r="B255" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C255" s="32" t="inlineStr">
-        <is>
-          <t>⚠️ Schlegeis tunnel traffic lights — one-way sections · red light = up to 15 min wait · factor into morning timing · aim to be at the dam car park by 8:45am</t>
-        </is>
-      </c>
-    </row>
-    <row r="256" ht="34" customHeight="1">
+      <c r="F255" s="10" t="inlineStr"/>
+    </row>
+    <row r="256" ht="32" customHeight="1">
       <c r="A256" s="30" t="inlineStr"/>
       <c r="B256" s="31" t="inlineStr">
         <is>
@@ -5601,11 +5612,11 @@
       </c>
       <c r="C256" s="32" t="inlineStr">
         <is>
-          <t>⚠️ Fern Pass congestion 2026 — slow trucks · one of the most congested alpine roads · flexible dinner only — no reservations · Bichlbach Gasthäuser are relaxed about timing</t>
-        </is>
-      </c>
-    </row>
-    <row r="257" ht="32" customHeight="1">
+          <t>⚠️ Schlegeis tunnel traffic lights — one-way sections · red light = up to 15 min wait · factor into morning timing · aim to be at the dam car park by 8:45am</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="34" customHeight="1">
       <c r="A257" s="30" t="inlineStr"/>
       <c r="B257" s="31" t="inlineStr">
         <is>
@@ -5614,11 +5625,11 @@
       </c>
       <c r="C257" s="32" t="inlineStr">
         <is>
-          <t>At Olpererhütte: check Neuschwanstein booking — the hut has excellent Wi-Fi · confirm your 9:30am slot for tomorrow · cash preferred for food but cards accepted</t>
-        </is>
-      </c>
-    </row>
-    <row r="258" ht="34" customHeight="1">
+          <t>⚠️ Fern Pass congestion 2026 — slow trucks · one of the most congested alpine roads · flexible dinner only — no reservations · Bichlbach Gasthäuser are relaxed about timing</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="32" customHeight="1">
       <c r="A258" s="30" t="inlineStr"/>
       <c r="B258" s="31" t="inlineStr">
         <is>
@@ -5627,309 +5638,309 @@
       </c>
       <c r="C258" s="32" t="inlineStr">
         <is>
+          <t>At Olpererhütte: check Neuschwanstein booking — the hut has excellent Wi-Fi · confirm your 9:30am slot for tomorrow · cash preferred for food but cards accepted</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="34" customHeight="1">
+      <c r="A259" s="30" t="inlineStr"/>
+      <c r="B259" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C259" s="32" t="inlineStr">
+        <is>
           <t>Blindsee — 2km from Landhaus Bichlbach — one of Austria's most photogenic lakes · emerald green · often misty in the morning · short walk or 3 min drive from the hotel · many visitors prefer it over Achensee · perfect early morning walk bef</t>
         </is>
       </c>
     </row>
-    <row r="259" ht="3" customHeight="1">
-      <c r="A259" s="33" t="n"/>
-      <c r="B259" s="33" t="n"/>
-      <c r="C259" s="33" t="n"/>
-      <c r="D259" s="33" t="n"/>
-      <c r="E259" s="33" t="n"/>
-      <c r="F259" s="33" t="n"/>
-    </row>
-    <row r="260" ht="20" customHeight="1">
-      <c r="A260" s="3" t="inlineStr">
+    <row r="260" ht="3" customHeight="1">
+      <c r="A260" s="33" t="n"/>
+      <c r="B260" s="33" t="n"/>
+      <c r="C260" s="33" t="n"/>
+      <c r="D260" s="33" t="n"/>
+      <c r="E260" s="33" t="n"/>
+      <c r="F260" s="33" t="n"/>
+    </row>
+    <row r="261" ht="20" customHeight="1">
+      <c r="A261" s="3" t="inlineStr">
         <is>
           <t>DAY 14  |  Jul 3  |  The Lakes of the Dragon — Seebensee · Drachensee · Coburger Hütte  |  ~20 km / 12 mi  ~30m · just Bichlbach ↔ Ehrwald</t>
         </is>
       </c>
     </row>
-    <row r="261" ht="15" customHeight="1">
-      <c r="A261" s="4" t="inlineStr">
+    <row r="262" ht="15" customHeight="1">
+      <c r="A262" s="4" t="inlineStr">
         <is>
           <t>Timeline: Tonight: ATM Ehrwald €60–80 ▸ 7:45am Bichlbach ▸ 8:00am Ehrwalder Almbahn (first car) ▸ 8:10am hike ▸ 9:45am Seebensee mirror ▸ 10:15am Drachensee climb ▸ 11:00am Coburger Hütte Kaiserschmarrn ▸ 12:45pm descent ▸ 2:45pm back at car ▸ 3pm Bichlbach ▸ 7:30pm Heiterwanger See sunset</t>
         </is>
       </c>
     </row>
-    <row r="262" ht="22" customHeight="1">
-      <c r="A262" s="5" t="inlineStr">
+    <row r="263" ht="22" customHeight="1">
+      <c r="A263" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ ATM in Ehrwald tonight — €60–80 cash · Coburger Hütte cash only · no card reader  |  ✅ 7:45am departure — first cable car 8:00am · arrive Seebensee 9:45am · beats 10:30am winds  |  ⚠️ Seebensee mirror reflection before 10:30am — winds create ripples by midday · 9:45am arrival ✅  |  ⚠️ Drachensee path slippery if rained Jul 2 — best-grip boots · 217m steep climb · 30–45 min  |  ➕ E-bikes optional at valley station — cuts Seebensee hike from 1.5hrs to 25 min · saves legs for Drachensee</t>
         </is>
       </c>
     </row>
-    <row r="263" ht="50" customHeight="1">
-      <c r="A263" s="16" t="inlineStr"/>
-      <c r="B263" s="17" t="inlineStr">
+    <row r="264" ht="50" customHeight="1">
+      <c r="A264" s="16" t="inlineStr"/>
+      <c r="B264" s="17" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C263" s="16" t="inlineStr">
+      <c r="C264" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D263" s="17" t="inlineStr"/>
-      <c r="E263" s="18" t="inlineStr">
+      <c r="D264" s="17" t="inlineStr"/>
+      <c r="E264" s="18" t="inlineStr">
         <is>
           <t>Tonight (Jul 2 evening): ATM in Ehrwald — withdraw €60–80 cash for the family · Coburger Hütte is cash only — no card reader on the mountain · budget: Kaiserschmarrn ~€12 · Tiroler Gröstl ~€14 · drinks ~€4–6 each</t>
         </is>
       </c>
-      <c r="F263" s="19" t="inlineStr">
+      <c r="F264" s="19" t="inlineStr">
         <is>
           <t>€60 / €12 / €14</t>
         </is>
       </c>
     </row>
-    <row r="264" ht="38" customHeight="1">
-      <c r="A264" s="6" t="inlineStr"/>
-      <c r="B264" s="7" t="inlineStr">
+    <row r="265" ht="38" customHeight="1">
+      <c r="A265" s="6" t="inlineStr"/>
+      <c r="B265" s="7" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C264" s="8" t="inlineStr">
+      <c r="C265" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D264" s="7" t="inlineStr"/>
-      <c r="E264" s="9" t="inlineStr">
+      <c r="D265" s="7" t="inlineStr"/>
+      <c r="E265" s="9" t="inlineStr">
         <is>
           <t>7:45am — Depart Bichlbach — 5 min drive to Ehrwalder Almbahn valley station · free parking for cable car guests · arrive ~7:55am</t>
         </is>
       </c>
-      <c r="F264" s="10" t="inlineStr">
+      <c r="F265" s="10" t="inlineStr">
         <is>
           <t>5 min</t>
         </is>
       </c>
     </row>
-    <row r="265" ht="44" customHeight="1">
-      <c r="A265" s="16" t="inlineStr"/>
-      <c r="B265" s="17" t="inlineStr">
+    <row r="266" ht="44" customHeight="1">
+      <c r="A266" s="16" t="inlineStr"/>
+      <c r="B266" s="17" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C265" s="16" t="inlineStr">
+      <c r="C266" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D265" s="17" t="inlineStr"/>
-      <c r="E265" s="18" t="inlineStr">
+      <c r="D266" s="17" t="inlineStr"/>
+      <c r="E266" s="18" t="inlineStr">
         <is>
           <t>⭐ 8:00am — Ehrwalder Almbahn — first cable car of the day · ~€26/adult · free parking · 5 min at top for Zugspitze platform view · ⚠️ July high season: opens 8:00am</t>
         </is>
       </c>
-      <c r="F265" s="19" t="inlineStr">
+      <c r="F266" s="19" t="inlineStr">
         <is>
           <t>€26 / 5 min</t>
         </is>
       </c>
     </row>
-    <row r="266" ht="50" customHeight="1">
-      <c r="A266" s="20" t="inlineStr"/>
-      <c r="B266" s="21" t="inlineStr">
+    <row r="267" ht="50" customHeight="1">
+      <c r="A267" s="20" t="inlineStr"/>
+      <c r="B267" s="21" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C266" s="22" t="inlineStr">
+      <c r="C267" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D266" s="21" t="inlineStr"/>
-      <c r="E266" s="23" t="inlineStr">
+      <c r="D267" s="21" t="inlineStr"/>
+      <c r="E267" s="23" t="inlineStr">
         <is>
           <t>8:10am — Hike to Seebensee — 5.6km from top station · wide gravel path · 152m elevation gain · easy · allow 1.5hrs · arrive ~9:45am · ➕ E-bikes available at valley station — cuts hike to 25 min if family wants to save le</t>
         </is>
       </c>
-      <c r="F266" s="24" t="inlineStr">
+      <c r="F267" s="24" t="inlineStr">
         <is>
           <t>6km / 5hr / 25 min</t>
         </is>
       </c>
     </row>
-    <row r="267" ht="50" customHeight="1">
-      <c r="A267" s="6" t="inlineStr"/>
-      <c r="B267" s="7" t="inlineStr">
+    <row r="268" ht="50" customHeight="1">
+      <c r="A268" s="6" t="inlineStr"/>
+      <c r="B268" s="7" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C267" s="8" t="inlineStr">
+      <c r="C268" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D267" s="7" t="inlineStr"/>
-      <c r="E267" s="9" t="inlineStr">
+      <c r="D268" s="7" t="inlineStr"/>
+      <c r="E268" s="9" t="inlineStr">
         <is>
           <t>⭐ ⭐ 9:45am — Seebensee mirror reflection — crystal-clear turquoise water · Zugspitze reflected · winds pick up after 10:30am — 9:45am arrival is perfectly timed · allow 30 min · benches along the southern shore</t>
         </is>
       </c>
-      <c r="F267" s="10" t="inlineStr">
+      <c r="F268" s="10" t="inlineStr">
         <is>
           <t>30 min</t>
         </is>
       </c>
     </row>
-    <row r="268" ht="44" customHeight="1">
-      <c r="A268" s="20" t="inlineStr"/>
-      <c r="B268" s="21" t="inlineStr">
+    <row r="269" ht="44" customHeight="1">
+      <c r="A269" s="20" t="inlineStr"/>
+      <c r="B269" s="21" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C268" s="22" t="inlineStr">
+      <c r="C269" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D268" s="21" t="inlineStr"/>
-      <c r="E268" s="23" t="inlineStr">
+      <c r="D269" s="21" t="inlineStr"/>
+      <c r="E269" s="23" t="inlineStr">
         <is>
           <t>10:15am — Drachensee ascent — 1.4km · 217m elevation gain · 30–45 min · ⚠️ slippery if rained Jul 2 · best-grip boots · steeper than Seebensee section but short</t>
         </is>
       </c>
-      <c r="F268" s="24" t="inlineStr">
+      <c r="F269" s="24" t="inlineStr">
         <is>
           <t>4km / 45 min</t>
         </is>
       </c>
     </row>
-    <row r="269" ht="46" customHeight="1">
-      <c r="A269" s="16" t="inlineStr"/>
-      <c r="B269" s="17" t="inlineStr">
+    <row r="270" ht="46" customHeight="1">
+      <c r="A270" s="16" t="inlineStr"/>
+      <c r="B270" s="17" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C269" s="16" t="inlineStr">
+      <c r="C270" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D269" s="17" t="inlineStr"/>
-      <c r="E269" s="18" t="inlineStr">
+      <c r="D270" s="17" t="inlineStr"/>
+      <c r="E270" s="18" t="inlineStr">
         <is>
           <t>⭐ ⭐ 11:00am — Coburger Hütte (1,917m) — legendary Kaiserschmarrn — MUST · cash only — bring €60–80 family · outdoor table facing deep blue Drachensee below · allow 1hr 45min</t>
         </is>
       </c>
-      <c r="F269" s="19" t="inlineStr">
+      <c r="F270" s="19" t="inlineStr">
         <is>
           <t>€60 / 1hr / 45min</t>
         </is>
       </c>
     </row>
-    <row r="270" ht="40" customHeight="1">
-      <c r="A270" s="20" t="inlineStr"/>
-      <c r="B270" s="21" t="inlineStr">
+    <row r="271" ht="40" customHeight="1">
+      <c r="A271" s="20" t="inlineStr"/>
+      <c r="B271" s="21" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C270" s="22" t="inlineStr">
+      <c r="C271" s="22" t="inlineStr">
         <is>
           <t>Hike</t>
         </is>
       </c>
-      <c r="D270" s="21" t="inlineStr"/>
-      <c r="E270" s="23" t="inlineStr">
+      <c r="D271" s="21" t="inlineStr"/>
+      <c r="E271" s="23" t="inlineStr">
         <is>
           <t>12:45pm — Descent to cable car station — ~1.5hrs back down · same trail · arrive top station ~2:15pm · cable car down · back at car ~2:45pm</t>
         </is>
       </c>
-      <c r="F270" s="24" t="inlineStr">
+      <c r="F271" s="24" t="inlineStr">
         <is>
           <t>5hr</t>
         </is>
       </c>
     </row>
-    <row r="271" ht="39" customHeight="1">
-      <c r="A271" s="6" t="inlineStr"/>
-      <c r="B271" s="7" t="inlineStr">
+    <row r="272" ht="39" customHeight="1">
+      <c r="A272" s="6" t="inlineStr"/>
+      <c r="B272" s="7" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C271" s="8" t="inlineStr">
+      <c r="C272" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D271" s="7" t="inlineStr"/>
-      <c r="E271" s="9" t="inlineStr">
+      <c r="D272" s="7" t="inlineStr"/>
+      <c r="E272" s="9" t="inlineStr">
         <is>
           <t>3:00pm — Back at Landhaus Bichlbach — shower · rest legs · pack bags for tomorrow · checkout 8am — Neuschwanstein 9:30am · alarm 7:00am</t>
         </is>
       </c>
-      <c r="F271" s="10" t="inlineStr"/>
-    </row>
-    <row r="272" ht="46" customHeight="1">
-      <c r="A272" s="16" t="inlineStr"/>
-      <c r="B272" s="17" t="inlineStr">
+      <c r="F272" s="10" t="inlineStr"/>
+    </row>
+    <row r="273" ht="46" customHeight="1">
+      <c r="A273" s="16" t="inlineStr"/>
+      <c r="B273" s="17" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C272" s="16" t="inlineStr">
+      <c r="C273" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D272" s="17" t="inlineStr"/>
-      <c r="E272" s="18" t="inlineStr">
+      <c r="D273" s="17" t="inlineStr"/>
+      <c r="E273" s="18" t="inlineStr">
         <is>
           <t>⭐ 7:30pm — Heiterwanger See sunset walk — 20 min walk from Landhaus along the Panoramaweg · flat · easy · clears the lactic acid · alpenglow after sunset on the higher path</t>
         </is>
       </c>
-      <c r="F272" s="19" t="inlineStr">
+      <c r="F273" s="19" t="inlineStr">
         <is>
           <t>20 min</t>
         </is>
       </c>
     </row>
-    <row r="273" ht="39" customHeight="1">
-      <c r="A273" s="11" t="inlineStr"/>
-      <c r="B273" s="12" t="inlineStr">
+    <row r="274" ht="39" customHeight="1">
+      <c r="A274" s="11" t="inlineStr"/>
+      <c r="B274" s="12" t="inlineStr">
         <is>
           <t>Jul 3</t>
         </is>
       </c>
-      <c r="C273" s="13" t="inlineStr">
+      <c r="C274" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D273" s="12" t="inlineStr"/>
-      <c r="E273" s="14" t="inlineStr">
+      <c r="D274" s="12" t="inlineStr"/>
+      <c r="E274" s="14" t="inlineStr">
         <is>
           <t>Dinner — Gasthof Bichlbach or hotel restaurant — early dinner + early bed · alarm 7:00am tomorrow · Neuschwanstein 9:30am — last big day</t>
         </is>
       </c>
-      <c r="F273" s="15" t="inlineStr"/>
-    </row>
-    <row r="274" ht="33" customHeight="1">
-      <c r="A274" s="30" t="inlineStr"/>
-      <c r="B274" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C274" s="32" t="inlineStr">
-        <is>
-          <t>Coburger Hütte cash only — withdraw €60–80 at Raiffeisenbank ATM in Ehrwald village tonight · budget: Kaiserschmarrn ~€12 · Tiroler Gröstl ~€14 · drinks ~€4–6 each</t>
-        </is>
-      </c>
-    </row>
-    <row r="275" ht="34" customHeight="1">
+      <c r="F274" s="15" t="inlineStr"/>
+    </row>
+    <row r="275" ht="33" customHeight="1">
       <c r="A275" s="30" t="inlineStr"/>
       <c r="B275" s="31" t="inlineStr">
         <is>
@@ -5938,7 +5949,7 @@
       </c>
       <c r="C275" s="32" t="inlineStr">
         <is>
-          <t>Seebensee mirror reflection — must arrive before 10:30am · mountain winds create ripples by midday · morning start from Bichlbach (8:30am) guarantees the calm water window</t>
+          <t>Coburger Hütte cash only — withdraw €60–80 at Raiffeisenbank ATM in Ehrwald village tonight · budget: Kaiserschmarrn ~€12 · Tiroler Gröstl ~€14 · drinks ~€4–6 each</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5962,7 @@
       </c>
       <c r="C276" s="32" t="inlineStr">
         <is>
-          <t>️ Zugspitze platform at top station — take 5 min before walking to Seebensee · look north toward Germany · see the "other side" of the Zugspitze (2,962m) — same peak visible from Garmisch-Partenkirchen</t>
+          <t>Seebensee mirror reflection — must arrive before 10:30am · mountain winds create ripples by midday · morning start from Bichlbach (8:30am) guarantees the calm water window</t>
         </is>
       </c>
     </row>
@@ -5964,180 +5975,169 @@
       </c>
       <c r="C277" s="32" t="inlineStr">
         <is>
+          <t>️ Zugspitze platform at top station — take 5 min before walking to Seebensee · look north toward Germany · see the "other side" of the Zugspitze (2,962m) — same peak visible from Garmisch-Partenkirchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="278" ht="34" customHeight="1">
+      <c r="A278" s="30" t="inlineStr"/>
+      <c r="B278" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C278" s="32" t="inlineStr">
+        <is>
           <t>Panoramaweg for Heiterwanger See — take the higher Panoramaweg trail not the lakeside path · stays above the valley floor to catch alpenglow after sunset · 20 min from hotel · flat + easy</t>
         </is>
       </c>
     </row>
-    <row r="278" ht="3" customHeight="1">
-      <c r="A278" s="33" t="n"/>
-      <c r="B278" s="33" t="n"/>
-      <c r="C278" s="33" t="n"/>
-      <c r="D278" s="33" t="n"/>
-      <c r="E278" s="33" t="n"/>
-      <c r="F278" s="33" t="n"/>
-    </row>
-    <row r="279" ht="20" customHeight="1">
-      <c r="A279" s="3" t="inlineStr">
+    <row r="279" ht="3" customHeight="1">
+      <c r="A279" s="33" t="n"/>
+      <c r="B279" s="33" t="n"/>
+      <c r="C279" s="33" t="n"/>
+      <c r="D279" s="33" t="n"/>
+      <c r="E279" s="33" t="n"/>
+      <c r="F279" s="33" t="n"/>
+    </row>
+    <row r="280" ht="20" customHeight="1">
+      <c r="A280" s="3" t="inlineStr">
         <is>
           <t>DAY 15  |  Jul 4  |  Zurich Day — Old Town · Lake · Caliente Festival → ZRH  |  ~185 km / 115 mi  ~2h direct · saves 100km vs castle route</t>
         </is>
       </c>
     </row>
-    <row r="280" ht="15" customHeight="1">
-      <c r="A280" s="4" t="inlineStr">
+    <row r="281" ht="15" customHeight="1">
+      <c r="A281" s="4" t="inlineStr">
         <is>
           <t>Timeline: 8:00am Bichlbach checkout ▸ ~10:00am Airport Hotel ZRH ▸ 10:30am return Europcar ▸ 11:00am train to Zurich HB ▸ 11:15am Lindenhof + Grossmünster + Fraumünster ▸ 1:00pm Bahnhofstrasse + Sprüngli ▸ 1:45pm Lake Zurich waterfront ▸ 2:30pm Caliente! Latin Festival ▸ 4:30pm dinner by the lake ▸ 6:00pm train back ▸ early bed</t>
         </is>
       </c>
     </row>
-    <row r="281" ht="22" customHeight="1">
-      <c r="A281" s="5" t="inlineStr">
+    <row r="282" ht="22" customHeight="1">
+      <c r="A282" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ Return Europcar ZRH first thing — 10:30am · 5 min drive · done before Zurich  |  ✅ Caliente! Latin Festival Jul 4 — final day · Europe's largest Latin festival · lakefront · family-friendly  |  ✅ Confirm Hilton shuttle 5:30am at front desk tonight — CHF 7/person · NOT walk (2km)  |  ⚠️ Swiss vignette — verify on windscreen before crossing border</t>
         </is>
       </c>
     </row>
-    <row r="282" ht="44" customHeight="1">
-      <c r="A282" s="6" t="inlineStr"/>
-      <c r="B282" s="7" t="inlineStr">
+    <row r="283" ht="44" customHeight="1">
+      <c r="A283" s="6" t="inlineStr"/>
+      <c r="B283" s="7" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C282" s="8" t="inlineStr">
+      <c r="C283" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D282" s="7" t="inlineStr"/>
-      <c r="E282" s="9" t="inlineStr">
+      <c r="D283" s="7" t="inlineStr"/>
+      <c r="E283" s="9" t="inlineStr">
         <is>
           <t>8:00am — Checkout Landhaus Bichlbach + depart — ~185km direct to Zurich Airport · ~2hrs via A17/A12/A14 · no border stress · no peak Saturday mountain parking</t>
         </is>
       </c>
-      <c r="F282" s="10" t="inlineStr">
+      <c r="F283" s="10" t="inlineStr">
         <is>
           <t>~185km / ~2hr</t>
         </is>
       </c>
     </row>
-    <row r="283" ht="35" customHeight="1">
-      <c r="A283" s="16" t="inlineStr"/>
-      <c r="B283" s="17" t="inlineStr">
+    <row r="284" ht="35" customHeight="1">
+      <c r="A284" s="16" t="inlineStr"/>
+      <c r="B284" s="17" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C283" s="16" t="inlineStr">
+      <c r="C284" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D283" s="17" t="inlineStr"/>
-      <c r="E283" s="18" t="inlineStr">
+      <c r="D284" s="17" t="inlineStr"/>
+      <c r="E284" s="18" t="inlineStr">
         <is>
           <t>Swiss vignette check — cameras trigger a CHF 200 fine if missing · verify on windscreen before entering Switzerland</t>
         </is>
       </c>
-      <c r="F283" s="19" t="inlineStr">
+      <c r="F284" s="19" t="inlineStr">
         <is>
           <t>CHF 200</t>
         </is>
       </c>
     </row>
-    <row r="284" ht="41" customHeight="1">
-      <c r="A284" s="25" t="inlineStr"/>
-      <c r="B284" s="26" t="inlineStr">
+    <row r="285" ht="41" customHeight="1">
+      <c r="A285" s="25" t="inlineStr"/>
+      <c r="B285" s="26" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C284" s="27" t="inlineStr">
+      <c r="C285" s="27" t="inlineStr">
         <is>
           <t>Stay</t>
         </is>
       </c>
-      <c r="D284" s="26" t="inlineStr"/>
-      <c r="E284" s="28" t="inlineStr">
+      <c r="D285" s="26" t="inlineStr"/>
+      <c r="E285" s="28" t="inlineStr">
         <is>
           <t>~10:00am — Airport Hotel Zurich — drop bags at hotel · Lindbergh-Platz 1, 8152 Glattbrugg · check-in may not be ready — leave bags at reception</t>
         </is>
       </c>
-      <c r="F284" s="29" t="inlineStr"/>
-    </row>
-    <row r="285" ht="46" customHeight="1">
-      <c r="A285" s="6" t="inlineStr"/>
-      <c r="B285" s="7" t="inlineStr">
+      <c r="F285" s="29" t="inlineStr"/>
+    </row>
+    <row r="286" ht="46" customHeight="1">
+      <c r="A286" s="6" t="inlineStr"/>
+      <c r="B286" s="7" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C285" s="8" t="inlineStr">
+      <c r="C286" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D285" s="7" t="inlineStr"/>
-      <c r="E285" s="9" t="inlineStr">
+      <c r="D286" s="7" t="inlineStr"/>
+      <c r="E286" s="9" t="inlineStr">
         <is>
           <t>10:30am — Return Europcar ZRH — 5 min drive from hotel · confirm return closed out correctly · take Hilton shuttle back · keep boarding passes + passports in hand-carry</t>
         </is>
       </c>
-      <c r="F285" s="10" t="inlineStr">
+      <c r="F286" s="10" t="inlineStr">
         <is>
           <t>5 min</t>
         </is>
       </c>
     </row>
-    <row r="286" ht="38" customHeight="1">
-      <c r="A286" s="16" t="inlineStr"/>
-      <c r="B286" s="17" t="inlineStr">
+    <row r="287" ht="38" customHeight="1">
+      <c r="A287" s="16" t="inlineStr"/>
+      <c r="B287" s="17" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C286" s="16" t="inlineStr">
+      <c r="C287" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D286" s="17" t="inlineStr"/>
-      <c r="E286" s="18" t="inlineStr">
+      <c r="D287" s="17" t="inlineStr"/>
+      <c r="E287" s="18" t="inlineStr">
         <is>
           <t>11:00am — Train to Zurich HB — Zurich Airport → Zurich HB · 10 min · CHF 7 · runs every 10 min from the airport underground station</t>
         </is>
       </c>
-      <c r="F286" s="19" t="inlineStr">
+      <c r="F287" s="19" t="inlineStr">
         <is>
           <t>10 min / CHF 7 / 10 min</t>
         </is>
       </c>
     </row>
-    <row r="287" ht="37" customHeight="1">
-      <c r="A287" s="20" t="inlineStr"/>
-      <c r="B287" s="21" t="inlineStr">
-        <is>
-          <t>Jul 4</t>
-        </is>
-      </c>
-      <c r="C287" s="22" t="inlineStr">
-        <is>
-          <t>Hike</t>
-        </is>
-      </c>
-      <c r="D287" s="21" t="inlineStr"/>
-      <c r="E287" s="23" t="inlineStr">
-        <is>
-          <t>⭐ 11:15am — Lindenhof viewpoint — hilltop square · best city panorama without climbing · Romans used it as a fort · free · 15 min</t>
-        </is>
-      </c>
-      <c r="F287" s="24" t="inlineStr">
-        <is>
-          <t>15 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="288" ht="40" customHeight="1">
+    <row r="288" ht="37" customHeight="1">
       <c r="A288" s="20" t="inlineStr"/>
       <c r="B288" s="21" t="inlineStr">
         <is>
@@ -6152,40 +6152,40 @@
       <c r="D288" s="21" t="inlineStr"/>
       <c r="E288" s="23" t="inlineStr">
         <is>
+          <t>⭐ 11:15am — Lindenhof viewpoint — hilltop square · best city panorama without climbing · Romans used it as a fort · free · 15 min</t>
+        </is>
+      </c>
+      <c r="F288" s="24" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="289" ht="40" customHeight="1">
+      <c r="A289" s="20" t="inlineStr"/>
+      <c r="B289" s="21" t="inlineStr">
+        <is>
+          <t>Jul 4</t>
+        </is>
+      </c>
+      <c r="C289" s="22" t="inlineStr">
+        <is>
+          <t>Hike</t>
+        </is>
+      </c>
+      <c r="D289" s="21" t="inlineStr"/>
+      <c r="E289" s="23" t="inlineStr">
+        <is>
           <t>⭐ ⭐ 11:30am — Grossmünster — twin-towered landmark · climb to the top for panorama of city + Lake Zurich · kids love the tower climb · ~CHF 5</t>
         </is>
       </c>
-      <c r="F288" s="24" t="inlineStr">
+      <c r="F289" s="24" t="inlineStr">
         <is>
           <t>CHF 5</t>
         </is>
       </c>
     </row>
-    <row r="289" ht="37" customHeight="1">
-      <c r="A289" s="16" t="inlineStr"/>
-      <c r="B289" s="17" t="inlineStr">
-        <is>
-          <t>Jul 4</t>
-        </is>
-      </c>
-      <c r="C289" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D289" s="17" t="inlineStr"/>
-      <c r="E289" s="18" t="inlineStr">
-        <is>
-          <t>⭐ 12:15pm — Fraumünster — Marc Chagall stained glass windows — genuinely stunning · unlike anything else on the trip · ~CHF 5</t>
-        </is>
-      </c>
-      <c r="F289" s="19" t="inlineStr">
-        <is>
-          <t>CHF 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="290" ht="43" customHeight="1">
+    <row r="290" ht="37" customHeight="1">
       <c r="A290" s="16" t="inlineStr"/>
       <c r="B290" s="17" t="inlineStr">
         <is>
@@ -6200,16 +6200,16 @@
       <c r="D290" s="17" t="inlineStr"/>
       <c r="E290" s="18" t="inlineStr">
         <is>
-          <t>1:00pm — Bahnhofstrasse — one of the world's great shopping streets · Confiserie Sprüngli for Swiss chocolate + Luxemburgerli macarons — MUST · 30 min stroll</t>
+          <t>⭐ 12:15pm — Fraumünster — Marc Chagall stained glass windows — genuinely stunning · unlike anything else on the trip · ~CHF 5</t>
         </is>
       </c>
       <c r="F290" s="19" t="inlineStr">
         <is>
-          <t>30 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="291" ht="39" customHeight="1">
+          <t>CHF 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="43" customHeight="1">
       <c r="A291" s="16" t="inlineStr"/>
       <c r="B291" s="17" t="inlineStr">
         <is>
@@ -6224,16 +6224,16 @@
       <c r="D291" s="17" t="inlineStr"/>
       <c r="E291" s="18" t="inlineStr">
         <is>
-          <t>⭐ ⭐ 1:45pm — Lake Zurich waterfront — Bürkliplatz · swans · paddle boats · Alps visible in the background on a clear day · free · 45 min</t>
+          <t>1:00pm — Bahnhofstrasse — one of the world's great shopping streets · Confiserie Sprüngli for Swiss chocolate + Luxemburgerli macarons — MUST · 30 min stroll</t>
         </is>
       </c>
       <c r="F291" s="19" t="inlineStr">
         <is>
-          <t>45 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="292" ht="50" customHeight="1">
+          <t>30 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="292" ht="39" customHeight="1">
       <c r="A292" s="16" t="inlineStr"/>
       <c r="B292" s="17" t="inlineStr">
         <is>
@@ -6248,93 +6248,104 @@
       <c r="D292" s="17" t="inlineStr"/>
       <c r="E292" s="18" t="inlineStr">
         <is>
+          <t>⭐ ⭐ 1:45pm — Lake Zurich waterfront — Bürkliplatz · swans · paddle boats · Alps visible in the background on a clear day · free · 45 min</t>
+        </is>
+      </c>
+      <c r="F292" s="19" t="inlineStr">
+        <is>
+          <t>45 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="50" customHeight="1">
+      <c r="A293" s="16" t="inlineStr"/>
+      <c r="B293" s="17" t="inlineStr">
+        <is>
+          <t>Jul 4</t>
+        </is>
+      </c>
+      <c r="C293" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D293" s="17" t="inlineStr"/>
+      <c r="E293" s="18" t="inlineStr">
+        <is>
           <t>⭐ ⭐ 2:30pm — Caliente! Latin Festival — Jul 3–5 2026 · Europe's largest Latin festival · Kasernenareal · South American music + dancing + food stalls · Jul 4 is the final day — biggest atmosphere · family-friendly · free</t>
         </is>
       </c>
-      <c r="F292" s="19" t="inlineStr"/>
-    </row>
-    <row r="293" ht="44" customHeight="1">
-      <c r="A293" s="11" t="inlineStr"/>
-      <c r="B293" s="12" t="inlineStr">
+      <c r="F293" s="19" t="inlineStr"/>
+    </row>
+    <row r="294" ht="44" customHeight="1">
+      <c r="A294" s="11" t="inlineStr"/>
+      <c r="B294" s="12" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C293" s="13" t="inlineStr">
+      <c r="C294" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D293" s="12" t="inlineStr"/>
-      <c r="E293" s="14" t="inlineStr">
+      <c r="D294" s="12" t="inlineStr"/>
+      <c r="E294" s="14" t="inlineStr">
         <is>
           <t>4:30pm — Early dinner by Lake Zurich — Zeughauskeller (15th century armory beer hall · hearty Swiss meals) · or lakeside restaurant at Bürkliplatz · allow 1.5hrs</t>
         </is>
       </c>
-      <c r="F293" s="15" t="inlineStr">
+      <c r="F294" s="15" t="inlineStr">
         <is>
           <t>5hr</t>
         </is>
       </c>
     </row>
-    <row r="294" ht="27" customHeight="1">
-      <c r="A294" s="16" t="inlineStr"/>
-      <c r="B294" s="17" t="inlineStr">
+    <row r="295" ht="27" customHeight="1">
+      <c r="A295" s="16" t="inlineStr"/>
+      <c r="B295" s="17" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C294" s="16" t="inlineStr">
+      <c r="C295" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D294" s="17" t="inlineStr"/>
-      <c r="E294" s="18" t="inlineStr">
+      <c r="D295" s="17" t="inlineStr"/>
+      <c r="E295" s="18" t="inlineStr">
         <is>
           <t>6:00pm — Train back to airport — Zurich HB → Zurich Airport · 10 min · CHF 7</t>
         </is>
       </c>
-      <c r="F294" s="19" t="inlineStr">
+      <c r="F295" s="19" t="inlineStr">
         <is>
           <t>10 min / CHF 7</t>
         </is>
       </c>
     </row>
-    <row r="295" ht="47" customHeight="1">
-      <c r="A295" s="25" t="inlineStr"/>
-      <c r="B295" s="26" t="inlineStr">
+    <row r="296" ht="47" customHeight="1">
+      <c r="A296" s="25" t="inlineStr"/>
+      <c r="B296" s="26" t="inlineStr">
         <is>
           <t>Jul 4</t>
         </is>
       </c>
-      <c r="C295" s="27" t="inlineStr">
+      <c r="C296" s="27" t="inlineStr">
         <is>
           <t>Stay</t>
         </is>
       </c>
-      <c r="D295" s="26" t="inlineStr"/>
-      <c r="E295" s="28" t="inlineStr">
+      <c r="D296" s="26" t="inlineStr"/>
+      <c r="E296" s="28" t="inlineStr">
         <is>
           <t>6:30pm — Airport Hotel Zurich — pack final bags · passports in hand-carry · boarding passes to phone wallet · confirm 5:30am shuttle at front desk · set two alarms · early bed</t>
         </is>
       </c>
-      <c r="F295" s="29" t="inlineStr"/>
-    </row>
-    <row r="296" ht="31" customHeight="1">
-      <c r="A296" s="30" t="inlineStr"/>
-      <c r="B296" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C296" s="32" t="inlineStr">
-        <is>
-          <t>⚠️ Castle gate 9:20am — be at the GATE not the ticket centre by 9:20am · €17.50/adult incl. booking fee · guide does not wait · strictly timed entry</t>
-        </is>
-      </c>
-    </row>
-    <row r="297" ht="34" customHeight="1">
+      <c r="F296" s="29" t="inlineStr"/>
+    </row>
+    <row r="297" ht="31" customHeight="1">
       <c r="A297" s="30" t="inlineStr"/>
       <c r="B297" s="31" t="inlineStr">
         <is>
@@ -6343,11 +6354,11 @@
       </c>
       <c r="C297" s="32" t="inlineStr">
         <is>
-          <t>Aescher Swing event Jul 4 from 5pm — restaurant will be extremely crowded for the evening event · arrive 1:30–2:00pm · eat + leave before 4pm · if terrace full: Siedwurst at the kiosk + wooden bench · same views</t>
-        </is>
-      </c>
-    </row>
-    <row r="298" ht="30" customHeight="1">
+          <t>⚠️ Castle gate 9:20am — be at the GATE not the ticket centre by 9:20am · €17.50/adult incl. booking fee · guide does not wait · strictly timed entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="298" ht="34" customHeight="1">
       <c r="A298" s="30" t="inlineStr"/>
       <c r="B298" s="31" t="inlineStr">
         <is>
@@ -6356,11 +6367,11 @@
       </c>
       <c r="C298" s="32" t="inlineStr">
         <is>
-          <t>Wildkirchli caves — 30°C outside · 10°C inside the caves · pack a light layer in your daypack · 5 min walk through the cave on the path to Aescher</t>
-        </is>
-      </c>
-    </row>
-    <row r="299" ht="34" customHeight="1">
+          <t>Aescher Swing event Jul 4 from 5pm — restaurant will be extremely crowded for the evening event · arrive 1:30–2:00pm · eat + leave before 4pm · if terrace full: Siedwurst at the kiosk + wooden bench · same views</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="30" customHeight="1">
       <c r="A299" s="30" t="inlineStr"/>
       <c r="B299" s="31" t="inlineStr">
         <is>
@@ -6369,7 +6380,7 @@
       </c>
       <c r="C299" s="32" t="inlineStr">
         <is>
-          <t>Return car tonight — drop bags at Airport Hotel Zurich · drive 5 min to Europcar ZRH car return · take Hilton shuttle back · Europcar open until midnight · eliminates 5:30am stress tomorrow</t>
+          <t>Wildkirchli caves — 30°C outside · 10°C inside the caves · pack a light layer in your daypack · 5 min walk through the cave on the path to Aescher</t>
         </is>
       </c>
     </row>
@@ -6382,11 +6393,11 @@
       </c>
       <c r="C300" s="32" t="inlineStr">
         <is>
-          <t>Aescher food — Chäs-Chnöpfli (Swiss mac and cheese with Appenzeller) · or Rösti · or Siedwurst at the kiosk if terrace full · same cliff view from the wooden benches outside</t>
-        </is>
-      </c>
-    </row>
-    <row r="301" ht="32" customHeight="1">
+          <t>Return car tonight — drop bags at Airport Hotel Zurich · drive 5 min to Europcar ZRH car return · take Hilton shuttle back · Europcar open until midnight · eliminates 5:30am stress tomorrow</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="34" customHeight="1">
       <c r="A301" s="30" t="inlineStr"/>
       <c r="B301" s="31" t="inlineStr">
         <is>
@@ -6395,148 +6406,137 @@
       </c>
       <c r="C301" s="32" t="inlineStr">
         <is>
+          <t>Aescher food — Chäs-Chnöpfli (Swiss mac and cheese with Appenzeller) · or Rösti · or Siedwurst at the kiosk if terrace full · same cliff view from the wooden benches outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="32" customHeight="1">
+      <c r="A302" s="30" t="inlineStr"/>
+      <c r="B302" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C302" s="32" t="inlineStr">
+        <is>
           <t>⚠️ 5:00am alarm Jul 5 — set two alarms · FI571 departs 7:55am · check-in opens 5:30am · hotel is 5 min walk to terminal · boarding passes on phone tonight</t>
         </is>
       </c>
     </row>
-    <row r="302" ht="3" customHeight="1">
-      <c r="A302" s="33" t="n"/>
-      <c r="B302" s="33" t="n"/>
-      <c r="C302" s="33" t="n"/>
-      <c r="D302" s="33" t="n"/>
-      <c r="E302" s="33" t="n"/>
-      <c r="F302" s="33" t="n"/>
-    </row>
-    <row r="303" ht="20" customHeight="1">
-      <c r="A303" s="3" t="inlineStr">
+    <row r="303" ht="3" customHeight="1">
+      <c r="A303" s="33" t="n"/>
+      <c r="B303" s="33" t="n"/>
+      <c r="C303" s="33" t="n"/>
+      <c r="D303" s="33" t="n"/>
+      <c r="E303" s="33" t="n"/>
+      <c r="F303" s="33" t="n"/>
+    </row>
+    <row r="304" ht="20" customHeight="1">
+      <c r="A304" s="3" t="inlineStr">
         <is>
           <t>DAY 16  |  Jul 5  |  Homebound — ZRH → KEF → MCO · The Final Leg  |  —  —</t>
         </is>
       </c>
     </row>
-    <row r="304" ht="15" customHeight="1">
-      <c r="A304" s="4" t="inlineStr">
+    <row r="305" ht="15" customHeight="1">
+      <c r="A305" s="4" t="inlineStr">
         <is>
           <t>Timeline: Sat night: app check-in ▸ confirm shuttle ▸ 5am wake ▸ 5:30am Hilton shuttle (NOT walk) ▸ 5:45am Terminal 2 · Check-in Row 3 ▸ 6am security + E Gate Skymetro ▸ 7:55am FI571 ZRH→KEF ▸ KEF Pylsur layover ▸ 8:50pm MCO home</t>
         </is>
       </c>
     </row>
-    <row r="305" ht="22" customHeight="1">
-      <c r="A305" s="5" t="inlineStr">
+    <row r="306" ht="22" customHeight="1">
+      <c r="A306" s="5" t="inlineStr">
         <is>
           <t>Key: ✅ Take hotel shuttle NOT walk — Hilton is 2km from terminal · not walkable with luggage · CHF 7/person  |  ✅ Icelandair app check-in Saturday night — digital boarding pass · fast bag drop at Check-in 2 Row 3  |  ✅ US Customs at MCO not KEF — do not leave transit area in Iceland</t>
         </is>
       </c>
     </row>
-    <row r="306" ht="39" customHeight="1">
-      <c r="A306" s="34" t="inlineStr"/>
-      <c r="B306" s="35" t="inlineStr">
+    <row r="307" ht="39" customHeight="1">
+      <c r="A307" s="34" t="inlineStr"/>
+      <c r="B307" s="35" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C306" s="36" t="inlineStr">
+      <c r="C307" s="36" t="inlineStr">
         <is>
           <t>Alert</t>
         </is>
       </c>
-      <c r="D306" s="35" t="inlineStr"/>
-      <c r="E306" s="37" t="inlineStr">
+      <c r="D307" s="35" t="inlineStr"/>
+      <c r="E307" s="37" t="inlineStr">
         <is>
           <t>✅ Night before (Jul 4 Saturday evening) — final prep — (2) Check Europcar/Booking.com email — confirm car return was closed out correctly</t>
         </is>
       </c>
-      <c r="F306" s="38" t="inlineStr"/>
-    </row>
-    <row r="307" ht="40" customHeight="1">
-      <c r="A307" s="11" t="inlineStr"/>
-      <c r="B307" s="12" t="inlineStr">
+      <c r="F307" s="38" t="inlineStr"/>
+    </row>
+    <row r="308" ht="40" customHeight="1">
+      <c r="A308" s="11" t="inlineStr"/>
+      <c r="B308" s="12" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C307" s="13" t="inlineStr">
+      <c r="C308" s="13" t="inlineStr">
         <is>
           <t>Eat</t>
         </is>
       </c>
-      <c r="D307" s="12" t="inlineStr"/>
-      <c r="E307" s="14" t="inlineStr">
+      <c r="D308" s="12" t="inlineStr"/>
+      <c r="E308" s="14" t="inlineStr">
         <is>
           <t>⏰ 5:00am — Wake up — perfect timing · do not wake earlier unless extra bags need special handling · hotel breakfast starts at 5:30am if needed</t>
         </is>
       </c>
-      <c r="F307" s="15" t="inlineStr"/>
-    </row>
-    <row r="308" ht="31" customHeight="1">
-      <c r="A308" s="16" t="inlineStr"/>
-      <c r="B308" s="17" t="inlineStr">
+      <c r="F308" s="15" t="inlineStr"/>
+    </row>
+    <row r="309" ht="31" customHeight="1">
+      <c r="A309" s="16" t="inlineStr"/>
+      <c r="B309" s="17" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C308" s="16" t="inlineStr">
+      <c r="C309" s="16" t="inlineStr">
         <is>
           <t>Stop</t>
         </is>
       </c>
-      <c r="D308" s="17" t="inlineStr"/>
-      <c r="E308" s="18" t="inlineStr">
+      <c r="D309" s="17" t="inlineStr"/>
+      <c r="E309" s="18" t="inlineStr">
         <is>
           <t>⚠️ 5:30am — Hilton shuttle — ❌ do NOT walk · 2km to terminal · CHF 7/person · confirm seat tonight</t>
         </is>
       </c>
-      <c r="F308" s="19" t="inlineStr">
+      <c r="F309" s="19" t="inlineStr">
         <is>
           <t>2km / CHF 7</t>
         </is>
       </c>
     </row>
-    <row r="309" ht="31" customHeight="1">
-      <c r="A309" s="25" t="inlineStr"/>
-      <c r="B309" s="26" t="inlineStr">
+    <row r="310" ht="31" customHeight="1">
+      <c r="A310" s="25" t="inlineStr"/>
+      <c r="B310" s="26" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C309" s="27" t="inlineStr">
+      <c r="C310" s="27" t="inlineStr">
         <is>
           <t>Stay</t>
         </is>
       </c>
-      <c r="D309" s="26" t="inlineStr"/>
-      <c r="E309" s="28" t="inlineStr">
+      <c r="D310" s="26" t="inlineStr"/>
+      <c r="E310" s="28" t="inlineStr">
         <is>
           <t>✈️ 5:45am — Terminal 2, Check-in Row 3 — bag drop opens 5:25am · digital boarding pass on phone</t>
         </is>
       </c>
-      <c r="F309" s="29" t="inlineStr"/>
-    </row>
-    <row r="310" ht="30" customHeight="1">
-      <c r="A310" s="16" t="inlineStr"/>
-      <c r="B310" s="17" t="inlineStr">
-        <is>
-          <t>Jul 5</t>
-        </is>
-      </c>
-      <c r="C310" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D310" s="17" t="inlineStr"/>
-      <c r="E310" s="18" t="inlineStr">
-        <is>
-          <t>6:00am — Security + E Gates — Skymetro train from main terminal · allow 45 min · Sunday busy</t>
-        </is>
-      </c>
-      <c r="F310" s="19" t="inlineStr">
-        <is>
-          <t>45 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="311" ht="38" customHeight="1">
+      <c r="F310" s="29" t="inlineStr"/>
+    </row>
+    <row r="311" ht="30" customHeight="1">
       <c r="A311" s="16" t="inlineStr"/>
       <c r="B311" s="17" t="inlineStr">
         <is>
@@ -6551,56 +6551,56 @@
       <c r="D311" s="17" t="inlineStr"/>
       <c r="E311" s="18" t="inlineStr">
         <is>
+          <t>6:00am — Security + E Gates — Skymetro train from main terminal · allow 45 min · Sunday busy</t>
+        </is>
+      </c>
+      <c r="F311" s="19" t="inlineStr">
+        <is>
+          <t>45 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="38" customHeight="1">
+      <c r="A312" s="16" t="inlineStr"/>
+      <c r="B312" s="17" t="inlineStr">
+        <is>
+          <t>Jul 5</t>
+        </is>
+      </c>
+      <c r="C312" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D312" s="17" t="inlineStr"/>
+      <c r="E312" s="18" t="inlineStr">
+        <is>
           <t>Spend remaining Swiss Francs — airport shops + cafés open by 6:00am · CHF coins and small bills are hard to exchange back in the US</t>
         </is>
       </c>
-      <c r="F311" s="19" t="inlineStr"/>
-    </row>
-    <row r="312" ht="19" customHeight="1">
-      <c r="A312" s="6" t="inlineStr"/>
-      <c r="B312" s="7" t="inlineStr">
+      <c r="F312" s="19" t="inlineStr"/>
+    </row>
+    <row r="313" ht="19" customHeight="1">
+      <c r="A313" s="6" t="inlineStr"/>
+      <c r="B313" s="7" t="inlineStr">
         <is>
           <t>Jul 5</t>
         </is>
       </c>
-      <c r="C312" s="8" t="inlineStr">
+      <c r="C313" s="8" t="inlineStr">
         <is>
           <t>Drive</t>
         </is>
       </c>
-      <c r="D312" s="7" t="inlineStr"/>
-      <c r="E312" s="9" t="inlineStr">
+      <c r="D313" s="7" t="inlineStr"/>
+      <c r="E313" s="9" t="inlineStr">
         <is>
           <t>✈️ 7:55am — FI571 departs ZRH → KEF</t>
         </is>
       </c>
-      <c r="F312" s="10" t="inlineStr"/>
-    </row>
-    <row r="313" ht="37" customHeight="1">
-      <c r="A313" s="16" t="inlineStr"/>
-      <c r="B313" s="17" t="inlineStr">
-        <is>
-          <t>Jul 5</t>
-        </is>
-      </c>
-      <c r="C313" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D313" s="17" t="inlineStr"/>
-      <c r="E313" s="18" t="inlineStr">
-        <is>
-          <t>KEF layover tip — 1.5–2hr layover is just enough time · grab a Pylsur — duty-free is excellent here if you missed anything</t>
-        </is>
-      </c>
-      <c r="F313" s="19" t="inlineStr">
-        <is>
-          <t>2hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="314" ht="35" customHeight="1">
+      <c r="F313" s="10" t="inlineStr"/>
+    </row>
+    <row r="314" ht="37" customHeight="1">
       <c r="A314" s="16" t="inlineStr"/>
       <c r="B314" s="17" t="inlineStr">
         <is>
@@ -6615,25 +6615,36 @@
       <c r="D314" s="17" t="inlineStr"/>
       <c r="E314" s="18" t="inlineStr">
         <is>
+          <t>KEF layover tip — 1.5–2hr layover is just enough time · grab a Pylsur — duty-free is excellent here if you missed anything</t>
+        </is>
+      </c>
+      <c r="F314" s="19" t="inlineStr">
+        <is>
+          <t>2hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="35" customHeight="1">
+      <c r="A315" s="16" t="inlineStr"/>
+      <c r="B315" s="17" t="inlineStr">
+        <is>
+          <t>Jul 5</t>
+        </is>
+      </c>
+      <c r="C315" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D315" s="17" t="inlineStr"/>
+      <c r="E315" s="18" t="inlineStr">
+        <is>
           <t>8:50pm — Arrive Orlando MCO — clear US Customs + Immigration at MCO · allow 45–60 min for customs on Sunday evening</t>
         </is>
       </c>
-      <c r="F314" s="19" t="inlineStr">
+      <c r="F315" s="19" t="inlineStr">
         <is>
           <t>60 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="315" ht="34" customHeight="1">
-      <c r="A315" s="30" t="inlineStr"/>
-      <c r="B315" s="31" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="C315" s="32" t="inlineStr">
-        <is>
-          <t>⚠️ Do NOT walk to terminal — Hilton Zurich Airport is ~2km from Terminal 2 in Glattbrugg · take the hotel shuttle · CHF 7/person · confirm 5:30am seat at front desk on Saturday evening</t>
         </is>
       </c>
     </row>
@@ -6646,7 +6657,7 @@
       </c>
       <c r="C316" s="32" t="inlineStr">
         <is>
-          <t>Saturday night app check-in — Icelandair app · download boarding passes to Apple/Google Wallet · check Europcar email for car return confirmation · passports in hand-carry bag · two alarms set</t>
+          <t>⚠️ Do NOT walk to terminal — Hilton Zurich Airport is ~2km from Terminal 2 in Glattbrugg · take the hotel shuttle · CHF 7/person · confirm 5:30am seat at front desk on Saturday evening</t>
         </is>
       </c>
     </row>
@@ -6659,11 +6670,11 @@
       </c>
       <c r="C317" s="32" t="inlineStr">
         <is>
-          <t>ZRH Terminal 2 details — Icelandair Check-in 2, Row 3 · E Gates for US-bound flights · Skymetro train from main terminal · extra security check at E Gate is standard · allow 45 min total at airport before gate</t>
-        </is>
-      </c>
-    </row>
-    <row r="318" ht="31" customHeight="1">
+          <t>Saturday night app check-in — Icelandair app · download boarding passes to Apple/Google Wallet · check Europcar email for car return confirmation · passports in hand-carry bag · two alarms set</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="34" customHeight="1">
       <c r="A318" s="30" t="inlineStr"/>
       <c r="B318" s="31" t="inlineStr">
         <is>
@@ -6672,17 +6683,30 @@
       </c>
       <c r="C318" s="32" t="inlineStr">
         <is>
+          <t>ZRH Terminal 2 details — Icelandair Check-in 2, Row 3 · E Gates for US-bound flights · Skymetro train from main terminal · extra security check at E Gate is standard · allow 45 min total at airport before gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="31" customHeight="1">
+      <c r="A319" s="30" t="inlineStr"/>
+      <c r="B319" s="31" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C319" s="32" t="inlineStr">
+        <is>
           <t>KEF layover — 1.5–2hrs · Pylsur hot dog (best in the world) · Skyr yoghurt · duty-free is excellent · US customs at MCO not here · do not leave transit</t>
         </is>
       </c>
     </row>
-    <row r="319" ht="3" customHeight="1">
-      <c r="A319" s="33" t="n"/>
-      <c r="B319" s="33" t="n"/>
-      <c r="C319" s="33" t="n"/>
-      <c r="D319" s="33" t="n"/>
-      <c r="E319" s="33" t="n"/>
-      <c r="F319" s="33" t="n"/>
+    <row r="320" ht="3" customHeight="1">
+      <c r="A320" s="33" t="n"/>
+      <c r="B320" s="33" t="n"/>
+      <c r="C320" s="33" t="n"/>
+      <c r="D320" s="33" t="n"/>
+      <c r="E320" s="33" t="n"/>
+      <c r="F320" s="33" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="113">
@@ -6694,45 +6718,44 @@
     <mergeCell ref="C217:F217"/>
     <mergeCell ref="C258:F258"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A303:F303"/>
-    <mergeCell ref="A200:F200"/>
+    <mergeCell ref="A263:F263"/>
+    <mergeCell ref="A144:F144"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A280:F280"/>
-    <mergeCell ref="A161:F161"/>
     <mergeCell ref="C73:F73"/>
-    <mergeCell ref="C315:F315"/>
     <mergeCell ref="A202:F202"/>
+    <mergeCell ref="C302:F302"/>
     <mergeCell ref="C121:F121"/>
     <mergeCell ref="C50:F50"/>
     <mergeCell ref="A186:F186"/>
     <mergeCell ref="C277:F277"/>
-    <mergeCell ref="A260:F260"/>
     <mergeCell ref="C236:F236"/>
     <mergeCell ref="C276:F276"/>
     <mergeCell ref="A241:F241"/>
     <mergeCell ref="C120:F120"/>
     <mergeCell ref="A124:F124"/>
     <mergeCell ref="C300:F300"/>
+    <mergeCell ref="C278:F278"/>
     <mergeCell ref="A305:F305"/>
+    <mergeCell ref="A243:F243"/>
     <mergeCell ref="A221:F221"/>
     <mergeCell ref="C17:F17"/>
     <mergeCell ref="C158:F158"/>
     <mergeCell ref="A163:F163"/>
     <mergeCell ref="A101:F101"/>
     <mergeCell ref="C19:F19"/>
+    <mergeCell ref="A223:F223"/>
+    <mergeCell ref="A306:F306"/>
     <mergeCell ref="C317:F317"/>
+    <mergeCell ref="C199:F199"/>
     <mergeCell ref="C96:F96"/>
-    <mergeCell ref="A141:F141"/>
+    <mergeCell ref="C239:F239"/>
+    <mergeCell ref="C319:F319"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="C235:F235"/>
     <mergeCell ref="A262:F262"/>
-    <mergeCell ref="A240:F240"/>
-    <mergeCell ref="C216:F216"/>
     <mergeCell ref="C98:F98"/>
     <mergeCell ref="A125:F125"/>
     <mergeCell ref="C218:F218"/>
-    <mergeCell ref="C274:F274"/>
-    <mergeCell ref="C137:F137"/>
     <mergeCell ref="A142:F142"/>
     <mergeCell ref="A304:F304"/>
     <mergeCell ref="A79:F79"/>
@@ -6743,23 +6766,24 @@
     <mergeCell ref="C76:F76"/>
     <mergeCell ref="C181:F181"/>
     <mergeCell ref="C119:F119"/>
+    <mergeCell ref="A282:F282"/>
+    <mergeCell ref="A164:F164"/>
     <mergeCell ref="A56:F56"/>
-    <mergeCell ref="C155:F155"/>
     <mergeCell ref="C237:F237"/>
     <mergeCell ref="A242:F242"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="C53:F53"/>
+    <mergeCell ref="A203:F203"/>
     <mergeCell ref="C34:F34"/>
     <mergeCell ref="C179:F179"/>
     <mergeCell ref="C157:F157"/>
+    <mergeCell ref="C160:F160"/>
     <mergeCell ref="C97:F97"/>
     <mergeCell ref="A102:F102"/>
     <mergeCell ref="C318:F318"/>
     <mergeCell ref="C256:F256"/>
     <mergeCell ref="A143:F143"/>
     <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A279:F279"/>
-    <mergeCell ref="C255:F255"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A103:F103"/>
     <mergeCell ref="A281:F281"/>
@@ -6767,28 +6791,27 @@
     <mergeCell ref="C51:F51"/>
     <mergeCell ref="C95:F95"/>
     <mergeCell ref="A78:F78"/>
-    <mergeCell ref="C178:F178"/>
     <mergeCell ref="C297:F297"/>
+    <mergeCell ref="C219:F219"/>
     <mergeCell ref="C299:F299"/>
     <mergeCell ref="A80:F80"/>
     <mergeCell ref="A37:F37"/>
-    <mergeCell ref="C296:F296"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A57:F57"/>
+    <mergeCell ref="C140:F140"/>
     <mergeCell ref="C298:F298"/>
     <mergeCell ref="A185:F185"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="C275:F275"/>
     <mergeCell ref="C156:F156"/>
-    <mergeCell ref="A184:F184"/>
     <mergeCell ref="C74:F74"/>
+    <mergeCell ref="C259:F259"/>
     <mergeCell ref="C197:F197"/>
     <mergeCell ref="C35:F35"/>
-    <mergeCell ref="A220:F220"/>
-    <mergeCell ref="C196:F196"/>
     <mergeCell ref="A201:F201"/>
     <mergeCell ref="C99:F99"/>
+    <mergeCell ref="C183:F183"/>
     <mergeCell ref="A261:F261"/>
     <mergeCell ref="C301:F301"/>
     <mergeCell ref="C180:F180"/>
@@ -6799,6 +6822,7 @@
     <mergeCell ref="C198:F198"/>
     <mergeCell ref="C238:F238"/>
     <mergeCell ref="C182:F182"/>
+    <mergeCell ref="A187:F187"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
P2 Compatsch booked ✅ · Ticket 325F53124754 · Order P039-60627-41931420C6 · €30 · Jul 1 05:00-23:00 · plate AI55582 · pass St. Valentin before 09:00 · bring voucher as entry ticket
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="30">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -157,12 +157,6 @@
     <font>
       <name val="Arial"/>
       <color rgb="006B7280"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="0092400E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -338,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -542,22 +536,10 @@
     <xf numFmtId="0" fontId="23" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -575,13 +557,13 @@
     <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -590,19 +572,19 @@
     <xf numFmtId="0" fontId="23" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4966,7 +4948,7 @@
     <row r="223" ht="22" customHeight="1">
       <c r="A223" s="5" t="inlineStr">
         <is>
-          <t>Key: ️ Plan A: P2 Compatsch — keep checking seiseralm.it for cancellations · must arrive before 9am · €30  |   Plan B: Seis cable car → Compatsch — park in Seis · ~€30/adult RT · no booking · no 9am rule · same trailhead  |   St. Valentin gate closes 9:00am SHARP — leave Collalbo 7:45am · arrive 8:30am · no exceptions  |  ❌ Skip Rifugio Zallinger — 4hr RT or 2 extra lifts · impractical · eat at Tschötsch Alm instead  |  ⚠️ Brenner Lueg Bridge construction 2026 — 30–45 min delay · Digital Flex toll essential</t>
+          <t>Key: ✅ P2 Compatsch booked · Ticket 325F53124754 · pass St. Valentin before 09:00 · bring voucher  |   St. Valentin gate closes 9:00am SHARP — leave Collalbo 7:45am · arrive 8:30am · no exceptions  |  ❌ Skip Rifugio Zallinger — 4hr RT or 2 extra lifts · impractical · eat at Tschötsch Alm instead  |  ⚠️ Brenner Lueg Bridge construction 2026 — 30–45 min delay · Digital Flex toll essential</t>
         </is>
       </c>
     </row>
@@ -5019,26 +5001,26 @@
       </c>
     </row>
     <row r="226" ht="50" customHeight="1">
-      <c r="A226" s="20" t="inlineStr"/>
-      <c r="B226" s="21" t="inlineStr">
+      <c r="A226" s="16" t="inlineStr"/>
+      <c r="B226" s="17" t="inlineStr">
         <is>
           <t>Jul 1</t>
         </is>
       </c>
-      <c r="C226" s="22" t="inlineStr">
-        <is>
-          <t>Hike</t>
-        </is>
-      </c>
-      <c r="D226" s="21" t="inlineStr"/>
-      <c r="E226" s="23" t="inlineStr">
-        <is>
-          <t>P2 Compatsch parking — ⚠️ Currently fully booked · keep checking seiseralm.it for cancellations · slots open up to 6 days before · €30 cash · must arrive before 9am · cameras enforce the gate ·  Plan B: Seis–Compatsch ca</t>
-        </is>
-      </c>
-      <c r="F226" s="24" t="inlineStr">
-        <is>
-          <t>€30 / €30 / €65</t>
+      <c r="C226" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D226" s="17" t="inlineStr"/>
+      <c r="E226" s="18" t="inlineStr">
+        <is>
+          <t>️ P2 Compatsch parking — ✅ Booked · Ticket 325F53124754 · €30 · ⚠️ Pass St. Valentin checkpoint before 09:00 SHARP · entry allowed 05:00–09:30 · plate AI55582 auto-read at barrier · bring voucher — it is your entry ticke</t>
+        </is>
+      </c>
+      <c r="F226" s="19" t="inlineStr">
+        <is>
+          <t>€30</t>
         </is>
       </c>
     </row>
@@ -7693,28 +7675,32 @@
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="69" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B8" s="70" t="inlineStr">
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>P2 Compatsch parking — Jul 1</t>
         </is>
       </c>
-      <c r="C8" s="71" t="inlineStr">
-        <is>
-          <t>seiseralm.it · €30/day · must arrive before 9am · QR code scan at barrier above Hotel Zorzi · booking system opens end of June 2026</t>
-        </is>
-      </c>
-      <c r="D8" s="71" t="inlineStr">
-        <is>
-          <t>Booking NOT open yet — system opens ~Jun 25 · check seiseralm.it daily from Jun 25 · book immediately when live · within 6-day window from Collalbo · Plan B: Seis cable car (no booking needed)</t>
-        </is>
-      </c>
-      <c r="E8" s="72" t="inlineStr"/>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Ticket 325F53124754 · Order P039-60627-41931420C6 · €30 · Jul 1 05:00–23:00 · entry 05:00–09:30 · plate AI55582 · seieralmbahn.it</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>Booked ✅ · Pass St. Valentin checkpoint before 09:00 · bring voucher as entry ticket · no cancellation</t>
+        </is>
+      </c>
+      <c r="E8" s="70" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="73" t="inlineStr">
+      <c r="A9" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7730,14 +7716,14 @@
         </is>
       </c>
       <c r="D9" s="24" t="inlineStr"/>
-      <c r="E9" s="74" t="inlineStr">
+      <c r="E9" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="73" t="inlineStr">
+      <c r="A10" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7753,14 +7739,14 @@
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr"/>
-      <c r="E10" s="74" t="inlineStr">
+      <c r="E10" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="73" t="inlineStr">
+      <c r="A11" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7776,14 +7762,14 @@
         </is>
       </c>
       <c r="D11" s="24" t="inlineStr"/>
-      <c r="E11" s="74" t="inlineStr">
+      <c r="E11" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="73" t="inlineStr">
+      <c r="A12" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7799,14 +7785,14 @@
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr"/>
-      <c r="E12" s="74" t="inlineStr">
+      <c r="E12" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="73" t="inlineStr">
+      <c r="A13" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7822,14 +7808,14 @@
         </is>
       </c>
       <c r="D13" s="24" t="inlineStr"/>
-      <c r="E13" s="74" t="inlineStr">
+      <c r="E13" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="73" t="inlineStr">
+      <c r="A14" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7845,14 +7831,14 @@
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr"/>
-      <c r="E14" s="74" t="inlineStr">
+      <c r="E14" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="73" t="inlineStr">
+      <c r="A15" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7872,14 +7858,14 @@
           <t>Booked ✅ — print tickets before departure</t>
         </is>
       </c>
-      <c r="E15" s="74" t="inlineStr">
+      <c r="E15" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="73" t="inlineStr">
+      <c r="A16" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7895,14 +7881,14 @@
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr"/>
-      <c r="E16" s="74" t="inlineStr">
+      <c r="E16" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="73" t="inlineStr">
+      <c r="A17" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7922,14 +7908,14 @@
           <t>Booked ✅ · Arrive Seelände dock by 8:55am (20 min before) · Keep return tickets separately</t>
         </is>
       </c>
-      <c r="E17" s="74" t="inlineStr">
+      <c r="E17" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="73" t="inlineStr">
+      <c r="A18" s="69" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7949,7 +7935,7 @@
           <t>Booked ✅ · update licence plate night before (Jun 28 in Sillian)</t>
         </is>
       </c>
-      <c r="E18" s="74" t="inlineStr">
+      <c r="E18" s="70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -8014,17 +8000,17 @@
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="75" t="inlineStr">
+      <c r="A3" s="71" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B3" s="76" t="inlineStr">
+      <c r="B3" s="72" t="inlineStr">
         <is>
           <t>Jun 20–21</t>
         </is>
       </c>
-      <c r="C3" s="76" t="inlineStr">
+      <c r="C3" s="72" t="inlineStr">
         <is>
           <t>Farmhouse Lodge, Vík</t>
         </is>
@@ -8041,17 +8027,17 @@
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="77" t="inlineStr">
+      <c r="A4" s="73" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B4" s="78" t="inlineStr">
+      <c r="B4" s="74" t="inlineStr">
         <is>
           <t>Jun 21–22</t>
         </is>
       </c>
-      <c r="C4" s="78" t="inlineStr">
+      <c r="C4" s="74" t="inlineStr">
         <is>
           <t>BergOne</t>
         </is>
@@ -8068,17 +8054,17 @@
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="75" t="inlineStr">
+      <c r="A5" s="71" t="inlineStr">
         <is>
           <t>3–4</t>
         </is>
       </c>
-      <c r="B5" s="76" t="inlineStr">
+      <c r="B5" s="72" t="inlineStr">
         <is>
           <t>Jun 22–24</t>
         </is>
       </c>
-      <c r="C5" s="76" t="inlineStr">
+      <c r="C5" s="72" t="inlineStr">
         <is>
           <t>Camping Jungfrau</t>
         </is>
@@ -8095,17 +8081,17 @@
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="77" t="inlineStr">
+      <c r="A6" s="73" t="inlineStr">
         <is>
           <t>5–6</t>
         </is>
       </c>
-      <c r="B6" s="78" t="inlineStr">
+      <c r="B6" s="74" t="inlineStr">
         <is>
           <t>Jun 24–26</t>
         </is>
       </c>
-      <c r="C6" s="78" t="inlineStr">
+      <c r="C6" s="74" t="inlineStr">
         <is>
           <t>One-Bedroom Apartment, Berchtesgaden</t>
         </is>
@@ -8122,17 +8108,17 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="75" t="inlineStr">
+      <c r="A7" s="71" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B7" s="76" t="inlineStr">
+      <c r="B7" s="72" t="inlineStr">
         <is>
           <t>Jun 26–28</t>
         </is>
       </c>
-      <c r="C7" s="76" t="inlineStr">
+      <c r="C7" s="72" t="inlineStr">
         <is>
           <t>Kaiserblick Goisern</t>
         </is>
@@ -8149,17 +8135,17 @@
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="77" t="inlineStr">
+      <c r="A8" s="73" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B8" s="78" t="inlineStr">
+      <c r="B8" s="74" t="inlineStr">
         <is>
           <t>Jun 28–29</t>
         </is>
       </c>
-      <c r="C8" s="78" t="inlineStr">
+      <c r="C8" s="74" t="inlineStr">
         <is>
           <t>Hotel Schwarzer Adler Sillian</t>
         </is>
@@ -8176,17 +8162,17 @@
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="75" t="inlineStr">
+      <c r="A9" s="71" t="inlineStr">
         <is>
           <t>10–11</t>
         </is>
       </c>
-      <c r="B9" s="76" t="inlineStr">
+      <c r="B9" s="72" t="inlineStr">
         <is>
           <t>Jun 29–Jul 1</t>
         </is>
       </c>
-      <c r="C9" s="76" t="inlineStr">
+      <c r="C9" s="72" t="inlineStr">
         <is>
           <t>Kaiserau 1907, Collalbo</t>
         </is>
@@ -8203,17 +8189,17 @@
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="77" t="inlineStr">
+      <c r="A10" s="73" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B10" s="78" t="inlineStr">
+      <c r="B10" s="74" t="inlineStr">
         <is>
           <t>Jul 1–2</t>
         </is>
       </c>
-      <c r="C10" s="78" t="inlineStr">
+      <c r="C10" s="74" t="inlineStr">
         <is>
           <t>Keyone Rooms Finkenberg</t>
         </is>
@@ -8230,17 +8216,17 @@
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="75" t="inlineStr">
+      <c r="A11" s="71" t="inlineStr">
         <is>
           <t>13-14-15</t>
         </is>
       </c>
-      <c r="B11" s="76" t="inlineStr">
+      <c r="B11" s="72" t="inlineStr">
         <is>
           <t>Jul 2–4</t>
         </is>
       </c>
-      <c r="C11" s="76" t="inlineStr">
+      <c r="C11" s="72" t="inlineStr">
         <is>
           <t>Landhaus Bichlbach</t>
         </is>
@@ -8257,17 +8243,17 @@
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="77" t="inlineStr">
+      <c r="A12" s="73" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B12" s="78" t="inlineStr">
+      <c r="B12" s="74" t="inlineStr">
         <is>
           <t>Jul 4–5</t>
         </is>
       </c>
-      <c r="C12" s="78" t="inlineStr">
+      <c r="C12" s="74" t="inlineStr">
         <is>
           <t>Airport Hotel Zurich</t>
         </is>
@@ -8336,17 +8322,17 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="76" t="inlineStr">
+      <c r="A3" s="72" t="inlineStr">
         <is>
           <t>Flights x4 (confirmed)</t>
         </is>
       </c>
-      <c r="B3" s="79" t="inlineStr">
+      <c r="B3" s="75" t="inlineStr">
         <is>
           <t>$4,088</t>
         </is>
       </c>
-      <c r="C3" s="80" t="inlineStr">
+      <c r="C3" s="76" t="inlineStr">
         <is>
           <t>$4,088</t>
         </is>
@@ -8358,17 +8344,17 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="76" t="inlineStr">
+      <c r="A4" s="72" t="inlineStr">
         <is>
           <t>Accommodation 15 nights (confirmed)</t>
         </is>
       </c>
-      <c r="B4" s="79" t="inlineStr">
+      <c r="B4" s="75" t="inlineStr">
         <is>
           <t>$3,032</t>
         </is>
       </c>
-      <c r="C4" s="80" t="inlineStr">
+      <c r="C4" s="76" t="inlineStr">
         <is>
           <t>$3,032</t>
         </is>
@@ -8380,17 +8366,17 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="76" t="inlineStr">
+      <c r="A5" s="72" t="inlineStr">
         <is>
           <t>Car Rental ZRH + KEF (confirmed)</t>
         </is>
       </c>
-      <c r="B5" s="79" t="inlineStr">
+      <c r="B5" s="75" t="inlineStr">
         <is>
           <t>$1,182</t>
         </is>
       </c>
-      <c r="C5" s="80" t="inlineStr">
+      <c r="C5" s="76" t="inlineStr">
         <is>
           <t>$1,182</t>
         </is>
@@ -8407,12 +8393,12 @@
           <t>Food &amp; Drinks</t>
         </is>
       </c>
-      <c r="B6" s="81" t="inlineStr">
+      <c r="B6" s="77" t="inlineStr">
         <is>
           <t>$1,850</t>
         </is>
       </c>
-      <c r="C6" s="82" t="inlineStr"/>
+      <c r="C6" s="78" t="inlineStr"/>
       <c r="D6" s="19" t="inlineStr">
         <is>
           <t>Update daily</t>
@@ -8420,18 +8406,18 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="83" t="inlineStr">
+      <c r="A7" s="79" t="inlineStr">
         <is>
           <t>Activities &amp; Entry Fees</t>
         </is>
       </c>
-      <c r="B7" s="84" t="inlineStr">
+      <c r="B7" s="80" t="inlineStr">
         <is>
           <t>$1,100</t>
         </is>
       </c>
-      <c r="C7" s="85" t="inlineStr"/>
-      <c r="D7" s="86" t="inlineStr">
+      <c r="C7" s="81" t="inlineStr"/>
+      <c r="D7" s="82" t="inlineStr">
         <is>
           <t>Cable cars, castle entries</t>
         </is>
@@ -8443,12 +8429,12 @@
           <t>Fuel &amp; Tolls</t>
         </is>
       </c>
-      <c r="B8" s="81" t="inlineStr">
+      <c r="B8" s="77" t="inlineStr">
         <is>
           <t>$1,000</t>
         </is>
       </c>
-      <c r="C8" s="82" t="inlineStr"/>
+      <c r="C8" s="78" t="inlineStr"/>
       <c r="D8" s="19" t="inlineStr">
         <is>
           <t>Grossglockner 46.50 EUR, Schlegeis 17 EUR, Auronzo 40 EUR</t>
@@ -8456,32 +8442,32 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="83" t="inlineStr">
+      <c r="A9" s="79" t="inlineStr">
         <is>
           <t>Shopping &amp; Misc</t>
         </is>
       </c>
-      <c r="B9" s="84" t="inlineStr">
+      <c r="B9" s="80" t="inlineStr">
         <is>
           <t>$400</t>
         </is>
       </c>
-      <c r="C9" s="85" t="inlineStr"/>
-      <c r="D9" s="86" t="inlineStr"/>
+      <c r="C9" s="81" t="inlineStr"/>
+      <c r="D9" s="82" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="87" t="inlineStr">
+      <c r="A10" s="83" t="inlineStr">
         <is>
           <t>TOTAL CONFIRMED</t>
         </is>
       </c>
-      <c r="B10" s="88" t="inlineStr">
+      <c r="B10" s="84" t="inlineStr">
         <is>
           <t>$8,302</t>
         </is>
       </c>
-      <c r="C10" s="88" t="inlineStr"/>
-      <c r="D10" s="89" t="inlineStr">
+      <c r="C10" s="84" t="inlineStr"/>
+      <c r="D10" s="85" t="inlineStr">
         <is>
           <t>vs est. ~$11,600-$12,900</t>
         </is>

</xml_diff>

<commit_message>
Day 10 Braies: clarified no reservation needed Jun 29 (system only activates Jul 1) · drive straight to P3 · pay cash on arrival
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -4308,7 +4308,7 @@
     <row r="187" ht="22" customHeight="1">
       <c r="A187" s="5" t="inlineStr">
         <is>
-          <t>Key: ✅ 8am departure — relaxed start · Braies 8:45am · still beautiful · P3 no reservation  |  ❌ Prato Piazza dropped — already have Alpe di Siusi Day 12 · same alpine meadow experience  |  ✅ Auronzo gate 11:15am — well within 9am–8:59pm slot · plate auto-read · no queue  |  ⚠️ Cadini final 50m narrow ridge — secondary viewpoint 20m back is 95% as good  |  ⚠️ Update Auronzo licence plate Jun 28 evening at pass.auronzo.info before Sillian dinner</t>
+          <t>Key: ✅ Braies Jun 29 — NO reservation needed · reservation system only starts Jul 1 · drive straight to P3 · pay €12 cash on arrival · 8:45am arrival perfect  |  ❌ Prato Piazza dropped — already have Alpe di Siusi Day 12 · same alpine meadow experience  |  ✅ Auronzo gate 11:15am — well within 9am–8:59pm slot · plate auto-read · no queue  |  ⚠️ Cadini final 50m narrow ridge — secondary viewpoint 20m back is 95% as good  |  ⚠️ Update Auronzo licence plate Jun 28 evening at pass.auronzo.info before Sillian dinner</t>
         </is>
       </c>
     </row>
@@ -4336,25 +4336,25 @@
         </is>
       </c>
     </row>
-    <row r="189" ht="49" customHeight="1">
-      <c r="A189" s="16" t="inlineStr"/>
-      <c r="B189" s="17" t="inlineStr">
+    <row r="189" ht="50" customHeight="1">
+      <c r="A189" s="6" t="inlineStr"/>
+      <c r="B189" s="7" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C189" s="16" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="D189" s="17" t="inlineStr"/>
-      <c r="E189" s="18" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ 8:45am — Lago di Braies — park P3 ~€12 · no reservation needed · walk the best half of the lakeside circuit · famous stilt boathouse · morning views · allow 1.5hrs · leave by 10:15am</t>
-        </is>
-      </c>
-      <c r="F189" s="19" t="inlineStr">
+      <c r="C189" s="8" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="D189" s="7" t="inlineStr"/>
+      <c r="E189" s="9" t="inlineStr">
+        <is>
+          <t>⭐ ⭐ 8:45am — Lago di Braies — park P3 ~€12 cash · 500m walk to lake · ✅ No reservation needed — Jun 29 is before Jul 1 · Reservation system only activates Jul 1–Sep 15 · drive straight in · pay cash at P3 on arrival · wa</t>
+        </is>
+      </c>
+      <c r="F189" s="10" t="inlineStr">
         <is>
           <t>€12 / 5hr</t>
         </is>

</xml_diff>

<commit_message>
Day 10: 7am departure · 8am Braies full 3.5km circuit + rowboat rental · all times shifted · Misurina 10am · Auronzo 10:45am · Cadini 11:15am · lunch 1pm · Tre Cime 2pm · Collalbo 4:30pm
</commit_message>
<xml_diff>
--- a/Europe-2026-VRFamilyTravels-Final.xlsx
+++ b/Europe-2026-VRFamilyTravels-Final.xlsx
@@ -4301,138 +4301,138 @@
     <row r="186" ht="15" customHeight="1">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Timeline: 8am Sillian ▸ 8:45am Braies P3 ▸ 10:15am depart ▸ Misurina coffee ▸ 11:15am Auronzo gate ▸ 11:45am Cadini Trail 117 ▸ 1:30pm lunch ▸ 2:30pm Tre Cime walk ▸ 3:45pm Gardena Pass ▸ 5pm Collalbo</t>
+          <t>Timeline: 7:00am Sillian ▸ 8:00am Braies P3 ▸ 8:05am full lake circuit 3.5km ▸ 9:05am rowboat optional ▸ 9:30am depart ▸ 10:15am Misurina coffee ▸ 11:15am Auronzo gate ▸ 11:45am Cadini Trail 117 ▸ 1:30pm lunch ▸ 2:30pm Tre Cime walk ▸ 3:45pm Gardena Pass ▸ 5:00pm Collalbo</t>
         </is>
       </c>
     </row>
     <row r="187" ht="22" customHeight="1">
       <c r="A187" s="5" t="inlineStr">
         <is>
-          <t>Key: ✅ Braies Jun 29 — NO reservation needed · reservation system only starts Jul 1 · drive straight to P3 · pay €12 cash on arrival · 8:45am arrival perfect  |  ❌ Prato Piazza dropped — already have Alpe di Siusi Day 12 · same alpine meadow experience  |  ✅ Auronzo gate 11:15am — well within 9am–8:59pm slot · plate auto-read · no queue  |  ⚠️ Cadini final 50m narrow ridge — secondary viewpoint 20m back is 95% as good  |  ⚠️ Update Auronzo licence plate Jun 28 evening at pass.auronzo.info before Sillian dinner</t>
-        </is>
-      </c>
-    </row>
-    <row r="188" ht="48" customHeight="1">
-      <c r="A188" s="6" t="inlineStr"/>
-      <c r="B188" s="7" t="inlineStr">
+          <t>Key: ✅ Braies 8:00am — NO reservation needed · reservation system only starts Jul 1 · drive straight to P3 · pay €12 cash · full 3.5km circuit + rowboat at 8am  |   Rowboat rental at Braies — €20/30min · fits 4 · opens 8am · first in queue · iconic birthday photo for Veena  |  ❌ Prato Piazza dropped — already have Alpe di Siusi Day 12 · same alpine meadow experience  |  ✅ Auronzo gate 11:15am — well within 9am–8:59pm slot · plate auto-read · no queue  |  ⚠️ Cadini final 50m narrow ridge — secondary viewpoint 20m back is 95% as good  |  ⚠️ Update Auronzo licence plate Jun 28 evening at pass.auronzo.info before Sillian dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="50" customHeight="1">
+      <c r="A188" s="16" t="inlineStr"/>
+      <c r="B188" s="17" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C188" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D188" s="7" t="inlineStr"/>
-      <c r="E188" s="9" t="inlineStr">
-        <is>
-          <t>8:00am — Depart Sillian — 45 min straight across the Italian border · download offline Dolomites maps tonight if not done · update Auronzo plate at pass.auronzo.info tonight (Jun 28)</t>
-        </is>
-      </c>
-      <c r="F188" s="10" t="inlineStr">
-        <is>
-          <t>45 min</t>
+      <c r="C188" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D188" s="17" t="inlineStr"/>
+      <c r="E188" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⭐ ⭐ 8:00am — Lago di Braies — park P3 ~€12 cash · 500m walk to lake · ✅ No reservation needed — Jun 29 is before Jul 1 · reservation system only activates Jul 1–Sep 15 · ⭐ Full 3.5km lake circuit — ~1hr · golden morning </t>
+        </is>
+      </c>
+      <c r="F188" s="19" t="inlineStr">
+        <is>
+          <t>€12 / 5km / ~1hr</t>
         </is>
       </c>
     </row>
     <row r="189" ht="50" customHeight="1">
-      <c r="A189" s="6" t="inlineStr"/>
-      <c r="B189" s="7" t="inlineStr">
+      <c r="A189" s="16" t="inlineStr"/>
+      <c r="B189" s="17" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C189" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D189" s="7" t="inlineStr"/>
-      <c r="E189" s="9" t="inlineStr">
-        <is>
-          <t>⭐ ⭐ 8:45am — Lago di Braies — park P3 ~€12 cash · 500m walk to lake · ✅ No reservation needed — Jun 29 is before Jul 1 · Reservation system only activates Jul 1–Sep 15 · drive straight in · pay cash at P3 on arrival · wa</t>
-        </is>
-      </c>
-      <c r="F189" s="10" t="inlineStr">
-        <is>
-          <t>€12 / 5hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="190" ht="44" customHeight="1">
-      <c r="A190" s="6" t="inlineStr"/>
-      <c r="B190" s="7" t="inlineStr">
+      <c r="C189" s="16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="D189" s="17" t="inlineStr"/>
+      <c r="E189" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⭐ ⭐ 8:00am — Lago di Braies — park P3 ~€12 cash · 500m walk to lake · ✅ No reservation needed — Jun 29 is before Jul 1 · reservation system only activates Jul 1–Sep 15 · ⭐ Full 3.5km lake circuit — ~1hr · golden morning </t>
+        </is>
+      </c>
+      <c r="F189" s="19" t="inlineStr">
+        <is>
+          <t>€12 / 5km / ~1hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="42" customHeight="1">
+      <c r="A190" s="11" t="inlineStr"/>
+      <c r="B190" s="12" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C190" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D190" s="7" t="inlineStr"/>
-      <c r="E190" s="9" t="inlineStr">
-        <is>
-          <t>☕ 10:15am — Drive via Lago di Misurina — 1hr drive down the valley · stop at Rifugio Misurina café · 15 min coffee + mirror-reflection photo of Tre Cime in the lake</t>
-        </is>
-      </c>
-      <c r="F190" s="10" t="inlineStr">
-        <is>
-          <t>1hr / 15 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="191" ht="45" customHeight="1">
-      <c r="A191" s="6" t="inlineStr"/>
-      <c r="B191" s="7" t="inlineStr">
+      <c r="C190" s="13" t="inlineStr">
+        <is>
+          <t>Eat</t>
+        </is>
+      </c>
+      <c r="D190" s="12" t="inlineStr"/>
+      <c r="E190" s="14" t="inlineStr">
+        <is>
+          <t>☕ 10:00am — Lago di Misurina coffee stop — mirror lake reflection · Rifugio Misurina terrace · 15 min · Tre Cime visible from the terrace on clear days</t>
+        </is>
+      </c>
+      <c r="F190" s="15" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="48" customHeight="1">
+      <c r="A191" s="11" t="inlineStr"/>
+      <c r="B191" s="12" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C191" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D191" s="7" t="inlineStr"/>
-      <c r="E191" s="9" t="inlineStr">
-        <is>
-          <t>⚠️ 11:15am — Auronzo gate — ✅ Pre-booked · PASS3CIME_26017885 · Ticket P26134547 · 9am–8:59pm slot · plate reads automatically · drive straight up · €40 paid · no queue</t>
-        </is>
-      </c>
-      <c r="F191" s="10" t="inlineStr">
-        <is>
-          <t>€40</t>
-        </is>
-      </c>
-    </row>
-    <row r="192" ht="50" customHeight="1">
-      <c r="A192" s="20" t="inlineStr"/>
-      <c r="B192" s="21" t="inlineStr">
+      <c r="C191" s="13" t="inlineStr">
+        <is>
+          <t>Eat</t>
+        </is>
+      </c>
+      <c r="D191" s="12" t="inlineStr"/>
+      <c r="E191" s="14" t="inlineStr">
+        <is>
+          <t>⚠️ 10:45am — Auronzo gate — ✅ Pre-booked · PASS3CIME_26017885 · Ticket P26134547 · 9am–8:59pm slot · plate AI55582 auto-read · no queue · 7km toll road to Rifugio Auronzo at 2,333m</t>
+        </is>
+      </c>
+      <c r="F191" s="15" t="inlineStr">
+        <is>
+          <t>7km</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="42" customHeight="1">
+      <c r="A192" s="11" t="inlineStr"/>
+      <c r="B192" s="12" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C192" s="22" t="inlineStr">
-        <is>
-          <t>Hike</t>
-        </is>
-      </c>
-      <c r="D192" s="21" t="inlineStr"/>
-      <c r="E192" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">⭐ ⭐ 11:45am — Cadini di Misurina Trail 117 — hike out to the iconic jagged peak viewpoint · 45 min RT at normal pace · ⚠️ final 50m is a narrow ridge · secondary viewpoint 20m back is 95% as good · allow 1hr 45min total </t>
-        </is>
-      </c>
-      <c r="F192" s="24" t="inlineStr">
-        <is>
-          <t>45 min / 1hr / 45min</t>
-        </is>
-      </c>
-    </row>
-    <row r="193" ht="29" customHeight="1">
+      <c r="C192" s="13" t="inlineStr">
+        <is>
+          <t>Eat</t>
+        </is>
+      </c>
+      <c r="D192" s="12" t="inlineStr"/>
+      <c r="E192" s="14" t="inlineStr">
+        <is>
+          <t>☕ 10:00am — Lago di Misurina coffee stop — mirror lake reflection · Rifugio Misurina terrace · 15 min · Tre Cime visible from the terrace on clear days</t>
+        </is>
+      </c>
+      <c r="F192" s="15" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="35" customHeight="1">
       <c r="A193" s="11" t="inlineStr"/>
       <c r="B193" s="12" t="inlineStr">
         <is>
@@ -4447,16 +4447,16 @@
       <c r="D193" s="12" t="inlineStr"/>
       <c r="E193" s="14" t="inlineStr">
         <is>
-          <t>1:30pm — Lunch at Rifugio Auronzo — cash is faster · hearty mountain lunch · allow 1hr</t>
+          <t>1:00pm — Lunch at Rifugio Auronzo — cash is faster · hearty mountain lunch · allow 1hr · budget €40–50 family cash</t>
         </is>
       </c>
       <c r="F193" s="15" t="inlineStr">
         <is>
-          <t>1hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="194" ht="40" customHeight="1">
+          <t>1hr / €40</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="50" customHeight="1">
       <c r="A194" s="11" t="inlineStr"/>
       <c r="B194" s="12" t="inlineStr">
         <is>
@@ -4471,16 +4471,16 @@
       <c r="D194" s="12" t="inlineStr"/>
       <c r="E194" s="14" t="inlineStr">
         <is>
-          <t>2:30pm — Tre Cime Highlights Walk — flat path to Rifugio Lavaredo (20 min each way) · see the towering north faces up close · allow 1hr 15min</t>
+          <t>2:00pm — Tre Cime highlights walk — 4km RT · 1hr · flat gravel path · walk to Rifugio Lavaredo (20 min each way) · best views of the Three Peaks · easy for kids · loose stones · hiking shoes recommended</t>
         </is>
       </c>
       <c r="F194" s="15" t="inlineStr">
         <is>
-          <t>20 min / 1hr / 15min</t>
-        </is>
-      </c>
-    </row>
-    <row r="195" ht="50" customHeight="1">
+          <t>4km / 1hr / 20 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="48" customHeight="1">
       <c r="A195" s="6" t="inlineStr"/>
       <c r="B195" s="7" t="inlineStr">
         <is>
@@ -4495,34 +4495,34 @@
       <c r="D195" s="7" t="inlineStr"/>
       <c r="E195" s="9" t="inlineStr">
         <is>
-          <t>3:45pm — Passo Gardena scenic drive — drive back down toll road · SS243 Gardena Pass (2,121m) · hairpin turns · low gear descent · ➕ Lagazuoi cable car optional if energy · ~1hr 15min drive</t>
-        </is>
-      </c>
-      <c r="F195" s="10" t="inlineStr">
-        <is>
-          <t>~1hr / 15min</t>
-        </is>
-      </c>
-    </row>
-    <row r="196" ht="43" customHeight="1">
-      <c r="A196" s="25" t="inlineStr"/>
-      <c r="B196" s="26" t="inlineStr">
+          <t>3:15pm — Passo Gardena scenic drive — drive back down toll road · SS243 Gardena Pass 2,121m · stunning Sella Group + Sassolungo views · pull over at any viewpoint on the way down</t>
+        </is>
+      </c>
+      <c r="F195" s="10" t="inlineStr"/>
+    </row>
+    <row r="196" ht="50" customHeight="1">
+      <c r="A196" s="11" t="inlineStr"/>
+      <c r="B196" s="12" t="inlineStr">
         <is>
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="C196" s="27" t="inlineStr">
-        <is>
-          <t>Stay</t>
-        </is>
-      </c>
-      <c r="D196" s="26" t="inlineStr"/>
-      <c r="E196" s="28" t="inlineStr">
-        <is>
-          <t>5:00pm — Kaiserau 1907, Collalbo — ✅ Check in · Via Peter Mayr 65, 39054 Collalbo · check-in 15:00–22:00 · unpack · rest · open a bottle of Italian wine</t>
-        </is>
-      </c>
-      <c r="F196" s="29" t="inlineStr"/>
+      <c r="C196" s="13" t="inlineStr">
+        <is>
+          <t>Eat</t>
+        </is>
+      </c>
+      <c r="D196" s="12" t="inlineStr"/>
+      <c r="E196" s="14" t="inlineStr">
+        <is>
+          <t>4:30pm — Kaiserau 1907, Collalbo — ✅ Check in · Via Peter Mayr 65, 39054 Collalbo · check-in from 3pm ·  Veena’s birthday dinner — book restaurant table tonight · Renon Earth Pyramids 5 min walk — evening light is magica</t>
+        </is>
+      </c>
+      <c r="F196" s="15" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="34" customHeight="1">
       <c r="A197" s="30" t="inlineStr"/>

</xml_diff>